<commit_message>
Rework scoring to derive all inputs from Min Engagement geometry
Remove dependency on layout type labels from main workbook. All scoring
now computed from cutter pocket data in Min Engagement files:

- Redundancy: detected from radial overlap between blade pairs (0.70 avg
  for Redundant layouts vs 0.38 for SingleSet, confirming geometry works)
- Force direction: axial vs radial ratio from orientation vectors (dz/dx/dy)
- 6-3 offset: Z-position gap between blade groups at nose region
- Blade exposure equality: how uniformly blades cover the profile
- Back rake, side rake, cutter density, spacing: all from ME Assy.Model
- Engagement thresholds: from ME Settings sheet

Main workbook only used for bit number identification and bit size fallback.

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Bit Applications Tool r2.xlsx
+++ b/Bit Applications Tool r2.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -4401,10 +4401,10 @@
         </is>
       </c>
       <c r="AO5" s="47" t="n">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
       <c r="AP5" s="48" t="n">
-        <v>3.1</v>
+        <v>6.5</v>
       </c>
       <c r="AQ5" s="163" t="n">
         <v>0</v>
@@ -4935,10 +4935,10 @@
         </is>
       </c>
       <c r="AO7" s="74" t="n">
-        <v>4.5</v>
+        <v>3.1</v>
       </c>
       <c r="AP7" s="75" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="AQ7" s="168" t="n">
         <v>0.1</v>
@@ -5993,10 +5993,10 @@
         </is>
       </c>
       <c r="AO11" s="47" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="AP11" s="48" t="n">
-        <v>7</v>
+        <v>5.6</v>
       </c>
       <c r="AQ11" s="167" t="n">
         <v>0.02</v>
@@ -6265,10 +6265,10 @@
         </is>
       </c>
       <c r="AO12" s="47" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="AP12" s="48" t="n">
-        <v>5.5</v>
+        <v>4.3</v>
       </c>
       <c r="AQ12" s="163" t="n">
         <v>0</v>
@@ -6805,10 +6805,10 @@
         </is>
       </c>
       <c r="AO14" s="47" t="n">
-        <v>5.1</v>
+        <v>5.6</v>
       </c>
       <c r="AP14" s="48" t="n">
-        <v>5.4</v>
+        <v>4</v>
       </c>
       <c r="AQ14" s="163" t="n">
         <v>0</v>
@@ -8669,10 +8669,10 @@
         </is>
       </c>
       <c r="AO21" s="47" t="n">
-        <v>1.5</v>
+        <v>2.7</v>
       </c>
       <c r="AP21" s="48" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
       <c r="AQ21" s="163" t="n">
         <v>0</v>
@@ -9737,10 +9737,10 @@
         </is>
       </c>
       <c r="AO25" s="47" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP25" s="48" t="n">
-        <v>6</v>
+        <v>4.8</v>
       </c>
       <c r="AQ25" s="163" t="n">
         <v>0</v>
@@ -10553,10 +10553,10 @@
         </is>
       </c>
       <c r="AO28" s="47" t="n">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="AP28" s="48" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
       <c r="AQ28" s="163" t="n">
         <v>0</v>
@@ -10825,10 +10825,10 @@
         </is>
       </c>
       <c r="AO29" s="47" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
       <c r="AP29" s="48" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="AQ29" s="163" t="n">
         <v>0</v>
@@ -11103,7 +11103,7 @@
         </is>
       </c>
       <c r="AO30" s="47" t="n">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="AP30" s="48" t="n">
         <v>4.8</v>
@@ -11409,10 +11409,10 @@
         </is>
       </c>
       <c r="AO31" s="46" t="n">
-        <v>1.5</v>
+        <v>2.3</v>
       </c>
       <c r="AP31" s="48" t="n">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="AQ31" s="163" t="n">
         <v>0</v>
@@ -11713,10 +11713,10 @@
         </is>
       </c>
       <c r="AO32" s="46" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="AP32" s="48" t="n">
-        <v>0.7</v>
+        <v>1.6</v>
       </c>
       <c r="AQ32" s="163" t="n">
         <v>0</v>
@@ -11993,10 +11993,10 @@
         </is>
       </c>
       <c r="AO33" s="47" t="n">
-        <v>3.3</v>
+        <v>4.6</v>
       </c>
       <c r="AP33" s="48" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
       <c r="AQ33" s="163" t="n">
         <v>0</v>
@@ -12273,10 +12273,10 @@
         </is>
       </c>
       <c r="AO34" s="47" t="n">
-        <v>3.2</v>
+        <v>4.4</v>
       </c>
       <c r="AP34" s="48" t="n">
-        <v>3.2</v>
+        <v>4.1</v>
       </c>
       <c r="AQ34" s="163" t="n">
         <v>0</v>
@@ -12553,10 +12553,10 @@
         </is>
       </c>
       <c r="AO35" s="47" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="AP35" s="48" t="n">
-        <v>4.1</v>
+        <v>3.3</v>
       </c>
       <c r="AQ35" s="163" t="n">
         <v>0</v>
@@ -12839,10 +12839,10 @@
         </is>
       </c>
       <c r="AO36" s="46" t="n">
-        <v>3.5</v>
+        <v>5.8</v>
       </c>
       <c r="AP36" s="48" t="n">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="AQ36" s="163" t="n">
         <v>0</v>
@@ -13111,10 +13111,10 @@
         </is>
       </c>
       <c r="AO37" s="47" t="n">
-        <v>5.5</v>
+        <v>4.6</v>
       </c>
       <c r="AP37" s="48" t="n">
-        <v>4.3</v>
+        <v>5</v>
       </c>
       <c r="AQ37" s="163" t="n">
         <v>0</v>
@@ -13414,7 +13414,7 @@
         <v>4.3</v>
       </c>
       <c r="AP38" s="48" t="n">
-        <v>5.6</v>
+        <v>5.1</v>
       </c>
       <c r="AQ38" s="163" t="n">
         <v>0</v>
@@ -13949,10 +13949,10 @@
         </is>
       </c>
       <c r="AO40" s="47" t="n">
-        <v>5.7</v>
+        <v>7</v>
       </c>
       <c r="AP40" s="48" t="n">
-        <v>5.1</v>
+        <v>3.3</v>
       </c>
       <c r="AQ40" s="163" t="n">
         <v>0</v>
@@ -14249,10 +14249,10 @@
         </is>
       </c>
       <c r="AO41" s="46" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="AP41" s="48" t="n">
-        <v>4.4</v>
+        <v>6</v>
       </c>
       <c r="AQ41" s="163" t="n">
         <v>0</v>
@@ -14529,10 +14529,10 @@
         </is>
       </c>
       <c r="AO42" s="47" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="AP42" s="48" t="n">
-        <v>5.1</v>
+        <v>6.2</v>
       </c>
       <c r="AQ42" s="163" t="n">
         <v>0</v>
@@ -14827,10 +14827,10 @@
         </is>
       </c>
       <c r="AO43" s="46" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="AP43" s="48" t="n">
-        <v>2.5</v>
+        <v>3.8</v>
       </c>
       <c r="AQ43" s="163" t="n">
         <v>0</v>
@@ -15109,10 +15109,10 @@
         </is>
       </c>
       <c r="AO44" s="47" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="AP44" s="48" t="n">
         <v>1.6</v>
-      </c>
-      <c r="AP44" s="48" t="n">
-        <v>2.4</v>
       </c>
       <c r="AQ44" s="163" t="n">
         <v>0</v>
@@ -15385,10 +15385,10 @@
         </is>
       </c>
       <c r="AO45" s="47" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="AP45" s="48" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="AQ45" s="163" t="n">
         <v>0</v>
@@ -15663,10 +15663,10 @@
         </is>
       </c>
       <c r="AO46" s="47" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="AP46" s="48" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="AQ46" s="163" t="n">
         <v>0</v>
@@ -15941,10 +15941,10 @@
         </is>
       </c>
       <c r="AO47" s="47" t="n">
-        <v>2.5</v>
+        <v>3.9</v>
       </c>
       <c r="AP47" s="48" t="n">
-        <v>4.3</v>
+        <v>6</v>
       </c>
       <c r="AQ47" s="163" t="n">
         <v>0</v>
@@ -16227,10 +16227,10 @@
         </is>
       </c>
       <c r="AO48" s="47" t="n">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="AP48" s="48" t="n">
-        <v>3.4</v>
+        <v>4.9</v>
       </c>
       <c r="AQ48" s="163" t="n">
         <v>0</v>
@@ -16521,10 +16521,10 @@
         </is>
       </c>
       <c r="AO49" s="46" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="AP49" s="48" t="n">
-        <v>6.4</v>
+        <v>5.1</v>
       </c>
       <c r="AQ49" s="163" t="n">
         <v>0</v>
@@ -16801,10 +16801,10 @@
         </is>
       </c>
       <c r="AO50" s="47" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="AP50" s="48" t="n">
-        <v>5</v>
+        <v>6.9</v>
       </c>
       <c r="AQ50" s="163" t="n">
         <v>0</v>
@@ -17103,10 +17103,10 @@
         </is>
       </c>
       <c r="AO51" s="46" t="n">
-        <v>2.2</v>
+        <v>3.7</v>
       </c>
       <c r="AP51" s="48" t="n">
-        <v>8</v>
+        <v>7.5</v>
       </c>
       <c r="AQ51" s="163" t="n">
         <v>0</v>
@@ -17387,10 +17387,10 @@
         </is>
       </c>
       <c r="AO52" s="47" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="AP52" s="48" t="n">
-        <v>5.8</v>
+        <v>4.8</v>
       </c>
       <c r="AQ52" s="163" t="n">
         <v>0</v>
@@ -17658,10 +17658,10 @@
         </is>
       </c>
       <c r="AO53" s="47" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="AP53" s="48" t="n">
-        <v>2.3</v>
+        <v>4</v>
       </c>
       <c r="AQ53" s="163" t="n">
         <v>0</v>
@@ -17928,10 +17928,10 @@
         </is>
       </c>
       <c r="AO54" s="47" t="n">
-        <v>1</v>
+        <v>1.7</v>
       </c>
       <c r="AP54" s="48" t="n">
-        <v>5</v>
+        <v>3.3</v>
       </c>
       <c r="AQ54" s="163" t="n">
         <v>0</v>
@@ -18194,10 +18194,10 @@
         </is>
       </c>
       <c r="AO55" s="47" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AP55" s="48" t="n">
-        <v>4.6</v>
+        <v>9</v>
       </c>
       <c r="AQ55" s="163" t="n">
         <v>0</v>
@@ -18470,10 +18470,10 @@
         </is>
       </c>
       <c r="AO56" s="47" t="n">
-        <v>2.9</v>
+        <v>4.4</v>
       </c>
       <c r="AP56" s="48" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="AQ56" s="163" t="n">
         <v>0</v>
@@ -18750,10 +18750,10 @@
         </is>
       </c>
       <c r="AO57" s="47" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AP57" s="48" t="n">
-        <v>3.5</v>
+        <v>7.4</v>
       </c>
       <c r="AQ57" s="163" t="n">
         <v>0</v>
@@ -19026,10 +19026,10 @@
         </is>
       </c>
       <c r="AO58" s="47" t="n">
-        <v>0.9</v>
+        <v>1.5</v>
       </c>
       <c r="AP58" s="48" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="AQ58" s="163" t="n">
         <v>0</v>
@@ -19305,7 +19305,7 @@
         </is>
       </c>
       <c r="AO59" s="47" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="AP59" s="48" t="n">
         <v>3.4</v>
@@ -19587,10 +19587,10 @@
         </is>
       </c>
       <c r="AO60" s="47" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="AP60" s="48" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="AQ60" s="163" t="n">
         <v>0</v>
@@ -19867,10 +19867,10 @@
         </is>
       </c>
       <c r="AO61" s="47" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
       <c r="AP61" s="48" t="n">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="AQ61" s="163" t="n">
         <v>0</v>
@@ -20149,10 +20149,10 @@
         </is>
       </c>
       <c r="AO62" s="47" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
       <c r="AP62" s="48" t="n">
-        <v>2.8</v>
+        <v>0.4</v>
       </c>
       <c r="AQ62" s="163" t="n">
         <v>0</v>
@@ -20425,10 +20425,10 @@
         </is>
       </c>
       <c r="AO63" s="47" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="AP63" s="48" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
       <c r="AQ63" s="163" t="n">
         <v>0</v>
@@ -20706,10 +20706,10 @@
         </is>
       </c>
       <c r="AO64" s="47" t="n">
-        <v>1.8</v>
+        <v>3.3</v>
       </c>
       <c r="AP64" s="48" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="AQ64" s="163" t="n">
         <v>0</v>
@@ -20986,10 +20986,10 @@
         </is>
       </c>
       <c r="AO65" s="47" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="AP65" s="48" t="n">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="AQ65" s="163" t="n">
         <v>0.083</v>
@@ -21275,10 +21275,10 @@
         </is>
       </c>
       <c r="AO66" s="47" t="n">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="AP66" s="48" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
       <c r="AQ66" s="163" t="n">
         <v>0</v>
@@ -21563,10 +21563,10 @@
         </is>
       </c>
       <c r="AO67" s="47" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="AP67" s="48" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="AQ67" s="163" t="n">
         <v>0</v>
@@ -21851,10 +21851,10 @@
         </is>
       </c>
       <c r="AO68" s="47" t="n">
-        <v>4.7</v>
+        <v>5</v>
       </c>
       <c r="AP68" s="48" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="AQ68" s="163" t="n">
         <v>0</v>
@@ -22147,10 +22147,10 @@
         </is>
       </c>
       <c r="AO69" s="47" t="n">
-        <v>2.4</v>
+        <v>3.2</v>
       </c>
       <c r="AP69" s="48" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="AQ69" s="163" t="n">
         <v>0</v>
@@ -22422,7 +22422,7 @@
         <v>0.2</v>
       </c>
       <c r="AP70" s="48" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="AQ70" s="163" t="n">
         <v>0</v>
@@ -22709,10 +22709,10 @@
         </is>
       </c>
       <c r="AO71" s="47" t="n">
-        <v>1.7</v>
+        <v>2.9</v>
       </c>
       <c r="AP71" s="48" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ71" s="163" t="n">
         <v>0</v>
@@ -22989,10 +22989,10 @@
         </is>
       </c>
       <c r="AO72" s="47" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="AP72" s="48" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AQ72" s="163" t="n">
         <v>0</v>
@@ -23268,10 +23268,10 @@
         </is>
       </c>
       <c r="AO73" s="47" t="n">
-        <v>3.1</v>
+        <v>5.1</v>
       </c>
       <c r="AP73" s="48" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="AQ73" s="163" t="n">
         <v>0</v>
@@ -23547,7 +23547,7 @@
         </is>
       </c>
       <c r="AO74" s="47" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="AP74" s="48" t="n">
         <v>3.1</v>
@@ -23828,10 +23828,10 @@
         </is>
       </c>
       <c r="AO75" s="47" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="AP75" s="48" t="n">
-        <v>3.2</v>
+        <v>5.9</v>
       </c>
       <c r="AQ75" s="163" t="n">
         <v>0</v>
@@ -24105,10 +24105,10 @@
         </is>
       </c>
       <c r="AO76" s="47" t="n">
-        <v>1.3</v>
+        <v>2.3</v>
       </c>
       <c r="AP76" s="48" t="n">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="AQ76" s="163" t="n">
         <v>0</v>
@@ -24327,10 +24327,10 @@
         </is>
       </c>
       <c r="AO77" s="47" t="n">
-        <v>5.4</v>
+        <v>6</v>
       </c>
       <c r="AP77" s="48" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="AQ77" s="163" t="n">
         <v>0</v>
@@ -24618,10 +24618,10 @@
         </is>
       </c>
       <c r="AO78" s="47" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="AP78" s="48" t="n">
-        <v>2.7</v>
+        <v>4.7</v>
       </c>
       <c r="AQ78" s="163" t="n">
         <v>0</v>
@@ -24907,10 +24907,10 @@
         </is>
       </c>
       <c r="AO79" s="47" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="AP79" s="48" t="n">
-        <v>7.3</v>
+        <v>7.8</v>
       </c>
       <c r="AQ79" s="163" t="n">
         <v>0</v>
@@ -25195,10 +25195,10 @@
         </is>
       </c>
       <c r="AO80" s="47" t="n">
-        <v>5.1</v>
+        <v>7.4</v>
       </c>
       <c r="AP80" s="48" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="AQ80" s="163" t="n">
         <v>0</v>
@@ -25465,10 +25465,10 @@
         </is>
       </c>
       <c r="AO81" s="47" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="AP81" s="48" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="AQ81" s="163" t="n">
         <v>0</v>
@@ -25741,10 +25741,10 @@
         </is>
       </c>
       <c r="AO82" s="47" t="n">
-        <v>2.5</v>
+        <v>3.8</v>
       </c>
       <c r="AP82" s="48" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="AQ82" s="163" t="n">
         <v>0</v>
@@ -26033,10 +26033,10 @@
         </is>
       </c>
       <c r="AO83" s="47" t="n">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="AP83" s="48" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
       <c r="AQ83" s="163" t="n">
         <v>0</v>
@@ -26319,10 +26319,10 @@
         </is>
       </c>
       <c r="AO84" s="47" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="AP84" s="48" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="AQ84" s="163" t="n">
         <v>0</v>
@@ -26603,10 +26603,10 @@
         </is>
       </c>
       <c r="AO85" s="47" t="n">
-        <v>1.7</v>
+        <v>3.1</v>
       </c>
       <c r="AP85" s="48" t="n">
-        <v>4.2</v>
+        <v>3.5</v>
       </c>
       <c r="AQ85" s="163" t="n">
         <v>0</v>
@@ -26890,7 +26890,7 @@
         <v>1.3</v>
       </c>
       <c r="AP86" s="48" t="n">
-        <v>6.1</v>
+        <v>6.8</v>
       </c>
       <c r="AQ86" s="163" t="n">
         <v>0</v>
@@ -27164,10 +27164,10 @@
         </is>
       </c>
       <c r="AO87" s="47" t="n">
-        <v>6.8</v>
+        <v>8.5</v>
       </c>
       <c r="AP87" s="48" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
       <c r="AQ87" s="163" t="n">
         <v>0</v>
@@ -27442,10 +27442,10 @@
         </is>
       </c>
       <c r="AO88" s="47" t="n">
-        <v>3.5</v>
+        <v>4.7</v>
       </c>
       <c r="AP88" s="48" t="n">
-        <v>3.5</v>
+        <v>3.8</v>
       </c>
       <c r="AQ88" s="163" t="n">
         <v>0</v>
@@ -27714,10 +27714,10 @@
         </is>
       </c>
       <c r="AO89" s="47" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="AP89" s="48" t="n">
-        <v>1.7</v>
+        <v>2.1</v>
       </c>
       <c r="AQ89" s="163" t="n">
         <v>0</v>
@@ -28005,10 +28005,10 @@
         </is>
       </c>
       <c r="AO90" s="47" t="n">
-        <v>3.5</v>
+        <v>5.8</v>
       </c>
       <c r="AP90" s="48" t="n">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="AQ90" s="163" t="n">
         <v>0</v>
@@ -28297,10 +28297,10 @@
         </is>
       </c>
       <c r="AO91" s="45" t="n">
-        <v>2.9</v>
+        <v>4.7</v>
       </c>
       <c r="AP91" s="48" t="n">
-        <v>4.6</v>
+        <v>3.7</v>
       </c>
       <c r="AQ91" s="163" t="n">
         <v>0</v>
@@ -28575,10 +28575,10 @@
         </is>
       </c>
       <c r="AO92" s="47" t="n">
-        <v>3</v>
+        <v>4.3</v>
       </c>
       <c r="AP92" s="48" t="n">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
       <c r="AQ92" s="163" t="n">
         <v>0</v>
@@ -28868,10 +28868,10 @@
         </is>
       </c>
       <c r="AO93" s="47" t="n">
-        <v>4.4</v>
+        <v>7.1</v>
       </c>
       <c r="AP93" s="48" t="n">
-        <v>0.6</v>
+        <v>3.3</v>
       </c>
       <c r="AQ93" s="163" t="n">
         <v>0</v>
@@ -29142,10 +29142,10 @@
         </is>
       </c>
       <c r="AO94" s="47" t="n">
-        <v>2.5</v>
+        <v>4.3</v>
       </c>
       <c r="AP94" s="48" t="n">
-        <v>5.8</v>
+        <v>5.2</v>
       </c>
       <c r="AQ94" s="163" t="n">
         <v>0</v>
@@ -29423,10 +29423,10 @@
         </is>
       </c>
       <c r="AO95" s="47" t="n">
-        <v>3</v>
+        <v>4.3</v>
       </c>
       <c r="AP95" s="48" t="n">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
       <c r="AQ95" s="163" t="n">
         <v>0</v>
@@ -29704,10 +29704,10 @@
         </is>
       </c>
       <c r="AO96" s="47" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="AP96" s="48" t="n">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="AQ96" s="163" t="n">
         <v>0</v>
@@ -29980,7 +29980,7 @@
         </is>
       </c>
       <c r="AO97" s="47" t="n">
-        <v>3.8</v>
+        <v>5.4</v>
       </c>
       <c r="AP97" s="88" t="n">
         <v>2.9</v>
@@ -30256,10 +30256,10 @@
         </is>
       </c>
       <c r="AO98" s="47" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="AP98" s="48" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="AQ98" s="163" t="n">
         <v>0</v>
@@ -30527,10 +30527,10 @@
         </is>
       </c>
       <c r="AO99" s="47" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="AP99" s="48" t="n">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="AQ99" s="163" t="n">
         <v>0.1</v>
@@ -30810,10 +30810,10 @@
         </is>
       </c>
       <c r="AO100" s="47" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="AP100" s="48" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="AQ100" s="163" t="n">
         <v>0</v>
@@ -31090,10 +31090,10 @@
         </is>
       </c>
       <c r="AO101" s="47" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AP101" s="48" t="n">
-        <v>5.3</v>
+        <v>4.4</v>
       </c>
       <c r="AQ101" s="163" t="n">
         <v>0.01</v>
@@ -31367,10 +31367,10 @@
         </is>
       </c>
       <c r="AO102" s="47" t="n">
-        <v>2.6</v>
+        <v>3.9</v>
       </c>
       <c r="AP102" s="48" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="AQ102" s="163" t="n">
         <v>0</v>
@@ -31633,10 +31633,10 @@
         </is>
       </c>
       <c r="AO103" s="47" t="n">
-        <v>3.5</v>
+        <v>6.2</v>
       </c>
       <c r="AP103" s="48" t="n">
-        <v>4</v>
+        <v>2.2</v>
       </c>
       <c r="AQ103" s="163" t="n">
         <v>0</v>
@@ -31911,10 +31911,10 @@
         </is>
       </c>
       <c r="AO104" s="47" t="n">
-        <v>3.2</v>
+        <v>4.4</v>
       </c>
       <c r="AP104" s="48" t="n">
-        <v>2.6</v>
+        <v>1.8</v>
       </c>
       <c r="AQ104" s="163" t="n">
         <v>0</v>
@@ -32188,10 +32188,10 @@
         </is>
       </c>
       <c r="AO105" s="47" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="AP105" s="48" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="AQ105" s="163" t="n">
         <v>0</v>
@@ -32460,10 +32460,10 @@
         </is>
       </c>
       <c r="AO106" s="47" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="AP106" s="48" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="AQ106" s="163" t="n">
         <v>0</v>
@@ -32726,7 +32726,7 @@
         </is>
       </c>
       <c r="AO107" s="47" t="n">
-        <v>3.8</v>
+        <v>5.4</v>
       </c>
       <c r="AP107" s="88" t="n">
         <v>2.9</v>
@@ -32995,10 +32995,10 @@
         </is>
       </c>
       <c r="AO108" s="47" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="AP108" s="48" t="n">
         <v>1.9</v>
-      </c>
-      <c r="AP108" s="48" t="n">
-        <v>2.4</v>
       </c>
       <c r="AQ108" s="163" t="n">
         <v>0</v>
@@ -33263,10 +33263,10 @@
         </is>
       </c>
       <c r="AO109" s="47" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="AP109" s="48" t="n">
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
       <c r="AQ109" s="163" t="n">
         <v>0</v>
@@ -33529,10 +33529,10 @@
         </is>
       </c>
       <c r="AO110" s="47" t="n">
-        <v>1.5</v>
+        <v>2.4</v>
       </c>
       <c r="AP110" s="48" t="n">
-        <v>4.1</v>
+        <v>2.9</v>
       </c>
       <c r="AQ110" s="163" t="n">
         <v>0</v>
@@ -33805,10 +33805,10 @@
         </is>
       </c>
       <c r="AO111" s="47" t="n">
-        <v>0.6</v>
+        <v>2.1</v>
       </c>
       <c r="AP111" s="48" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="AQ111" s="163" t="n">
         <v>0</v>
@@ -34077,10 +34077,10 @@
         </is>
       </c>
       <c r="AO112" s="47" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="AP112" s="48" t="n">
-        <v>2.1</v>
+        <v>0.1</v>
       </c>
       <c r="AQ112" s="163" t="n">
         <v>0.03</v>
@@ -34354,10 +34354,10 @@
         </is>
       </c>
       <c r="AO113" s="47" t="n">
-        <v>4.2</v>
+        <v>6</v>
       </c>
       <c r="AP113" s="48" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="AQ113" s="163" t="n">
         <v>0</v>
@@ -34634,10 +34634,10 @@
         </is>
       </c>
       <c r="AO114" s="47" t="n">
-        <v>2.9</v>
+        <v>4.1</v>
       </c>
       <c r="AP114" s="48" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AQ114" s="163" t="n">
         <v>0.03</v>
@@ -34917,10 +34917,10 @@
         </is>
       </c>
       <c r="AO115" s="47" t="n">
-        <v>2.9</v>
+        <v>4.1</v>
       </c>
       <c r="AP115" s="48" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AQ115" s="163" t="n">
         <v>0.06</v>
@@ -35200,10 +35200,10 @@
         </is>
       </c>
       <c r="AO116" s="47" t="n">
-        <v>2.9</v>
+        <v>3.8</v>
       </c>
       <c r="AP116" s="48" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AQ116" s="163" t="n">
         <v>0.09</v>
@@ -35475,10 +35475,10 @@
         </is>
       </c>
       <c r="AO117" s="47" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="AP117" s="48" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="AQ117" s="163" t="n">
         <v>0</v>
@@ -35752,10 +35752,10 @@
         </is>
       </c>
       <c r="AO118" s="47" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="AP118" s="48" t="n">
-        <v>4.1</v>
+        <v>5.2</v>
       </c>
       <c r="AQ118" s="163" t="n">
         <v>0</v>
@@ -36029,10 +36029,10 @@
         </is>
       </c>
       <c r="AO119" s="74" t="n">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="AP119" s="75" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="AQ119" s="173" t="n">
         <v>0</v>
@@ -36302,10 +36302,10 @@
         </is>
       </c>
       <c r="AO120" s="74" t="n">
-        <v>5.5</v>
+        <v>6.6</v>
       </c>
       <c r="AP120" s="75" t="n">
-        <v>6.8</v>
+        <v>4.4</v>
       </c>
       <c r="AQ120" s="168" t="n">
         <v>0</v>
@@ -36580,10 +36580,10 @@
         </is>
       </c>
       <c r="AO121" s="74" t="n">
-        <v>5.4</v>
+        <v>8.1</v>
       </c>
       <c r="AP121" s="75" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="AQ121" s="168" t="n">
         <v>0</v>
@@ -36854,10 +36854,10 @@
         </is>
       </c>
       <c r="AO122" s="74" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="AP122" s="75" t="n">
         <v>3.7</v>
-      </c>
-      <c r="AP122" s="75" t="n">
-        <v>5.6</v>
       </c>
       <c r="AQ122" s="168" t="n">
         <v>0</v>
@@ -37126,10 +37126,10 @@
         </is>
       </c>
       <c r="AO123" s="47" t="n">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
       <c r="AP123" s="88" t="n">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
       <c r="AQ123" s="164" t="n">
         <v>0.035</v>
@@ -37412,10 +37412,10 @@
         </is>
       </c>
       <c r="AO124" s="47" t="n">
-        <v>5.1</v>
+        <v>7.4</v>
       </c>
       <c r="AP124" s="88" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="AQ124" s="164" t="n">
         <v>0</v>
@@ -37686,10 +37686,10 @@
         </is>
       </c>
       <c r="AO125" s="74" t="n">
-        <v>4.7</v>
+        <v>6.8</v>
       </c>
       <c r="AP125" s="75" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="AQ125" s="168" t="n">
         <v>0</v>
@@ -37967,7 +37967,7 @@
         <v>1.8</v>
       </c>
       <c r="AP126" s="75" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="AQ126" s="168" t="n">
         <v>0</v>
@@ -38253,7 +38253,7 @@
         <v>1.8</v>
       </c>
       <c r="AP127" s="48" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="AQ127" s="167" t="n">
         <v>0</v>
@@ -38522,10 +38522,10 @@
         </is>
       </c>
       <c r="AO128" s="74" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
       <c r="AP128" s="75" t="n">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="AQ128" s="168" t="n">
         <v>0.083</v>
@@ -38812,10 +38812,10 @@
         </is>
       </c>
       <c r="AO129" s="74" t="n">
-        <v>4.7</v>
+        <v>5.2</v>
       </c>
       <c r="AP129" s="75" t="n">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="AQ129" s="167" t="n">
         <v>0</v>
@@ -39093,7 +39093,7 @@
         <v>9</v>
       </c>
       <c r="AP130" s="88" t="n">
-        <v>1.5</v>
+        <v>2.3</v>
       </c>
       <c r="AQ130" s="164" t="n">
         <v>0</v>
@@ -39368,10 +39368,10 @@
         </is>
       </c>
       <c r="AO131" s="47" t="n">
-        <v>3.2</v>
+        <v>4.3</v>
       </c>
       <c r="AP131" s="88" t="n">
-        <v>8.300000000000001</v>
+        <v>6.6</v>
       </c>
       <c r="AQ131" s="164" t="n">
         <v>0</v>
@@ -39642,10 +39642,10 @@
         </is>
       </c>
       <c r="AO132" s="47" t="n">
-        <v>2.6</v>
+        <v>4.3</v>
       </c>
       <c r="AP132" s="88" t="n">
-        <v>7</v>
+        <v>5.6</v>
       </c>
       <c r="AQ132" s="164" t="n">
         <v>0</v>
@@ -39918,10 +39918,10 @@
         </is>
       </c>
       <c r="AO133" s="47" t="n">
-        <v>5.4</v>
+        <v>6.8</v>
       </c>
       <c r="AP133" s="88" t="n">
-        <v>2.5</v>
+        <v>0.4</v>
       </c>
       <c r="AQ133" s="164" t="n">
         <v>0</v>
@@ -40468,10 +40468,10 @@
         </is>
       </c>
       <c r="AO135" s="47" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="AP135" s="88" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
       <c r="AQ135" s="164" t="n">
         <v>0</v>
@@ -40758,10 +40758,10 @@
         </is>
       </c>
       <c r="AO136" s="47" t="n">
-        <v>2.9</v>
+        <v>5</v>
       </c>
       <c r="AP136" s="88" t="n">
-        <v>7.7</v>
+        <v>7.1</v>
       </c>
       <c r="AQ136" s="164" t="n">
         <v>0</v>
@@ -41034,10 +41034,10 @@
         </is>
       </c>
       <c r="AO137" s="45" t="n">
-        <v>7.3</v>
+        <v>8.6</v>
       </c>
       <c r="AP137" s="48" t="n">
-        <v>5.2</v>
+        <v>6.2</v>
       </c>
       <c r="AQ137" s="167" t="n">
         <v>0</v>
@@ -41594,10 +41594,10 @@
         </is>
       </c>
       <c r="AO139" s="47" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="AP139" s="48" t="n">
-        <v>9</v>
+        <v>6.3</v>
       </c>
       <c r="AQ139" s="167" t="n">
         <v>0</v>
@@ -41872,10 +41872,10 @@
         </is>
       </c>
       <c r="AO140" s="88" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="AP140" s="118" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="AQ140" s="172" t="n">
         <v>0.038</v>
@@ -42152,10 +42152,10 @@
         </is>
       </c>
       <c r="AO141" s="74" t="n">
-        <v>7.3</v>
+        <v>9</v>
       </c>
       <c r="AP141" s="88" t="n">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="AQ141" s="167" t="n">
         <v>0</v>
@@ -42426,10 +42426,10 @@
         </is>
       </c>
       <c r="AO142" s="47" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="AP142" s="118" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="AQ142" s="167" t="n">
         <v>0.01</v>
@@ -42700,10 +42700,10 @@
         </is>
       </c>
       <c r="AO143" s="47" t="n">
-        <v>4.6</v>
+        <v>7.4</v>
       </c>
       <c r="AP143" s="118" t="n">
-        <v>5.4</v>
+        <v>2.9</v>
       </c>
       <c r="AQ143" s="172" t="n">
         <v>0</v>
@@ -43254,10 +43254,10 @@
         </is>
       </c>
       <c r="AO145" s="74" t="n">
-        <v>5.8</v>
+        <v>7.2</v>
       </c>
       <c r="AP145" s="118" t="n">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="AQ145" s="172" t="n">
         <v>0</v>
@@ -43538,10 +43538,10 @@
         </is>
       </c>
       <c r="AO146" s="47" t="n">
-        <v>3.9</v>
+        <v>5.8</v>
       </c>
       <c r="AP146" s="88" t="n">
-        <v>2.1</v>
+        <v>0.7</v>
       </c>
       <c r="AQ146" s="164" t="n">
         <v>0</v>
@@ -43818,10 +43818,10 @@
         </is>
       </c>
       <c r="AO147" s="74" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="AP147" s="48" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="AQ147" s="167" t="n">
         <v>0</v>
@@ -44100,10 +44100,10 @@
         </is>
       </c>
       <c r="AO148" s="74" t="n">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="AP148" s="48" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="AQ148" s="167" t="n">
         <v>0</v>
@@ -44378,10 +44378,10 @@
         </is>
       </c>
       <c r="AO149" s="47" t="n">
-        <v>7.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AP149" s="118" t="n">
-        <v>5.5</v>
+        <v>6.6</v>
       </c>
       <c r="AQ149" s="164" t="n">
         <v>0</v>
@@ -44656,10 +44656,10 @@
         </is>
       </c>
       <c r="AO150" s="47" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="AP150" s="118" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="AQ150" s="172" t="n">
         <v>0</v>
@@ -44936,10 +44936,10 @@
         </is>
       </c>
       <c r="AO151" s="74" t="n">
-        <v>5.4</v>
+        <v>7</v>
       </c>
       <c r="AP151" s="118" t="n">
-        <v>6.8</v>
+        <v>4.6</v>
       </c>
       <c r="AQ151" s="172" t="n">
         <v>0</v>
@@ -45500,10 +45500,10 @@
         </is>
       </c>
       <c r="AO153" s="74" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="AP153" s="118" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="AQ153" s="174" t="n">
         <v>0</v>
@@ -46044,10 +46044,10 @@
         </is>
       </c>
       <c r="AO155" s="74" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="AP155" s="118" t="n">
-        <v>1.6</v>
+        <v>0.1</v>
       </c>
       <c r="AQ155" s="172" t="n">
         <v>0</v>
@@ -46326,10 +46326,10 @@
         </is>
       </c>
       <c r="AO156" s="47" t="n">
-        <v>5.9</v>
+        <v>7.4</v>
       </c>
       <c r="AP156" s="88" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
       <c r="AQ156" s="164" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Populate BAT r2.xlsx with zone-specific engagement values (BA-BE) and updated ratings (AO-AP)
Enhanced compute_ratings.py with compute_zone_engagement() to extract per-zone
backup engagement thresholds from ME files. Classifies backup cutters by zone
(nose/taper) and type (PDC/knuckle), pairs with primaries, and converts Z offsets
to ft/hr at 100 RPM using Settings sheet IPR classes. Also computes 6-3 layout
engagement for primary PDCs on secondary blades.

Results: 130 bits scored (AO/AP), 117 bits with zone engagement (BA-BE).

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Bit Applications Tool r2.xlsx
+++ b/Bit Applications Tool r2.xlsx
@@ -4444,15 +4444,15 @@
       <c r="AZ5" s="43" t="n">
         <v>15</v>
       </c>
-      <c r="BA5" s="43" t="n"/>
+      <c r="BA5" s="43" t="n">
+        <v>31</v>
+      </c>
       <c r="BB5" s="53" t="n"/>
-      <c r="BC5" s="53" t="n"/>
-      <c r="BD5" s="53" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE5" s="53" t="n">
-        <v>0</v>
-      </c>
+      <c r="BC5" s="53" t="n">
+        <v>31</v>
+      </c>
+      <c r="BD5" s="53" t="n"/>
+      <c r="BE5" s="53" t="n"/>
       <c r="BF5" s="43" t="inlineStr">
         <is>
           <t>20-15</t>
@@ -4978,10 +4978,10 @@
       <c r="AZ7" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA7" s="77" t="n">
-        <v>100</v>
-      </c>
-      <c r="BB7" s="79" t="n"/>
+      <c r="BA7" s="77" t="n"/>
+      <c r="BB7" s="79" t="n">
+        <v>31</v>
+      </c>
       <c r="BC7" s="79" t="n"/>
       <c r="BD7" s="79" t="n"/>
       <c r="BE7" s="79" t="n"/>
@@ -6036,9 +6036,7 @@
       <c r="AZ11" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA11" s="16" t="n">
-        <v>20</v>
-      </c>
+      <c r="BA11" s="16" t="n"/>
       <c r="BB11" s="64" t="n"/>
       <c r="BC11" s="64" t="n"/>
       <c r="BD11" s="64" t="n"/>
@@ -6308,12 +6306,12 @@
       <c r="AZ12" s="16" t="n">
         <v>12.5</v>
       </c>
-      <c r="BA12" s="16" t="n"/>
-      <c r="BB12" s="64" t="n">
-        <v>110</v>
-      </c>
+      <c r="BA12" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB12" s="64" t="n"/>
       <c r="BC12" s="64" t="n">
-        <v>110</v>
+        <v>31</v>
       </c>
       <c r="BD12" s="64" t="n"/>
       <c r="BE12" s="64" t="n"/>
@@ -6848,12 +6846,14 @@
       <c r="AZ14" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA14" s="16" t="n"/>
+      <c r="BA14" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB14" s="64" t="n">
-        <v>110</v>
+        <v>234</v>
       </c>
       <c r="BC14" s="64" t="n">
-        <v>120</v>
+        <v>31</v>
       </c>
       <c r="BD14" s="64" t="n"/>
       <c r="BE14" s="64" t="n"/>
@@ -8712,10 +8712,10 @@
       </c>
       <c r="BA21" s="16" t="n"/>
       <c r="BB21" s="64" t="n">
-        <v>50</v>
+        <v>156</v>
       </c>
       <c r="BC21" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD21" s="64" t="n"/>
       <c r="BE21" s="64" t="n"/>
@@ -9779,11 +9779,9 @@
         <v>10</v>
       </c>
       <c r="BA25" s="16" t="n"/>
-      <c r="BB25" s="64" t="n">
-        <v>10</v>
-      </c>
+      <c r="BB25" s="64" t="n"/>
       <c r="BC25" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD25" s="64" t="n"/>
       <c r="BE25" s="64" t="n"/>
@@ -10596,9 +10594,15 @@
       <c r="AZ28" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA28" s="16" t="n"/>
-      <c r="BB28" s="64" t="n"/>
-      <c r="BC28" s="64" t="n"/>
+      <c r="BA28" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB28" s="64" t="n">
+        <v>78</v>
+      </c>
+      <c r="BC28" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BD28" s="64" t="n"/>
       <c r="BE28" s="64" t="n"/>
       <c r="BF28" s="16" t="n">
@@ -10868,12 +10872,12 @@
       <c r="AZ29" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA29" s="16" t="n"/>
-      <c r="BB29" s="64" t="n">
-        <v>70</v>
-      </c>
+      <c r="BA29" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB29" s="64" t="n"/>
       <c r="BC29" s="64" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="BD29" s="64" t="n"/>
       <c r="BE29" s="64" t="n"/>
@@ -11146,12 +11150,12 @@
       <c r="AZ30" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA30" s="16" t="n"/>
-      <c r="BB30" s="64" t="n">
-        <v>110</v>
-      </c>
+      <c r="BA30" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB30" s="64" t="n"/>
       <c r="BC30" s="64" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="BD30" s="64" t="n"/>
       <c r="BE30" s="64" t="n"/>
@@ -11452,14 +11456,12 @@
       </c>
       <c r="BA31" s="16" t="n"/>
       <c r="BB31" s="64" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="BC31" s="64" t="n">
-        <v>60</v>
-      </c>
-      <c r="BD31" s="64" t="n">
-        <v>0</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD31" s="64" t="n"/>
       <c r="BE31" s="64" t="n"/>
       <c r="BF31" s="16" t="n">
         <v>15</v>
@@ -11755,11 +11757,11 @@
         <v>7.5</v>
       </c>
       <c r="BA32" s="16" t="n"/>
-      <c r="BB32" s="64" t="n"/>
+      <c r="BB32" s="64" t="n">
+        <v>47</v>
+      </c>
       <c r="BC32" s="64" t="n"/>
-      <c r="BD32" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BD32" s="64" t="n"/>
       <c r="BE32" s="64" t="n"/>
       <c r="BF32" s="16" t="n">
         <v>17.5</v>
@@ -12034,12 +12036,14 @@
       <c r="AZ33" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA33" s="16" t="n"/>
-      <c r="BB33" s="64" t="n"/>
+      <c r="BA33" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB33" s="64" t="n">
+        <v>78</v>
+      </c>
       <c r="BC33" s="64" t="n"/>
-      <c r="BD33" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BD33" s="64" t="n"/>
       <c r="BE33" s="64" t="n"/>
       <c r="BF33" s="16" t="n">
         <v>20</v>
@@ -12314,12 +12318,14 @@
       <c r="AZ34" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA34" s="16" t="n"/>
-      <c r="BB34" s="64" t="n"/>
+      <c r="BA34" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB34" s="64" t="n">
+        <v>78</v>
+      </c>
       <c r="BC34" s="64" t="n"/>
-      <c r="BD34" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BD34" s="64" t="n"/>
       <c r="BE34" s="64" t="n"/>
       <c r="BF34" s="16" t="n">
         <v>20</v>
@@ -12880,9 +12886,15 @@
       <c r="AZ36" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA36" s="16" t="n"/>
-      <c r="BB36" s="64" t="n"/>
-      <c r="BC36" s="64" t="n"/>
+      <c r="BA36" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB36" s="64" t="n">
+        <v>31</v>
+      </c>
+      <c r="BC36" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BD36" s="64" t="n"/>
       <c r="BE36" s="64" t="n"/>
       <c r="BF36" s="16" t="n">
@@ -13154,19 +13166,17 @@
       <c r="AZ37" s="16" t="n">
         <v>12.5</v>
       </c>
-      <c r="BA37" s="16" t="n"/>
+      <c r="BA37" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB37" s="64" t="n">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="BC37" s="64" t="n">
-        <v>120</v>
-      </c>
-      <c r="BD37" s="64" t="n">
-        <v>70</v>
-      </c>
-      <c r="BE37" s="64" t="n">
-        <v>80</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD37" s="64" t="n"/>
+      <c r="BE37" s="64" t="n"/>
       <c r="BF37" s="16" t="n">
         <v>15</v>
       </c>
@@ -13454,12 +13464,12 @@
       <c r="AZ38" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="BA38" s="16" t="n"/>
-      <c r="BB38" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA38" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB38" s="64" t="n"/>
       <c r="BC38" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD38" s="64" t="n"/>
       <c r="BE38" s="64" t="n"/>
@@ -13992,19 +14002,15 @@
       <c r="AZ40" s="16" t="n">
         <v>12.5</v>
       </c>
-      <c r="BA40" s="16" t="n"/>
-      <c r="BB40" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA40" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB40" s="64" t="n"/>
       <c r="BC40" s="64" t="n">
-        <v>120</v>
-      </c>
-      <c r="BD40" s="64" t="n">
-        <v>70</v>
-      </c>
-      <c r="BE40" s="64" t="n">
-        <v>80</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD40" s="64" t="n"/>
+      <c r="BE40" s="64" t="n"/>
       <c r="BF40" s="16" t="n">
         <v>15</v>
       </c>
@@ -14292,14 +14298,12 @@
       </c>
       <c r="BA41" s="16" t="n"/>
       <c r="BB41" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BC41" s="64" t="n">
-        <v>80</v>
-      </c>
-      <c r="BD41" s="64" t="n">
-        <v>410</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BD41" s="64" t="n"/>
       <c r="BE41" s="64" t="n"/>
       <c r="BF41" s="16" t="n">
         <v>15</v>
@@ -14572,16 +14576,16 @@
       <c r="AZ42" s="16" t="n">
         <v>12.5</v>
       </c>
-      <c r="BA42" s="16" t="n"/>
+      <c r="BA42" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB42" s="64" t="n">
-        <v>230</v>
+        <v>31</v>
       </c>
       <c r="BC42" s="64" t="n">
-        <v>200</v>
-      </c>
-      <c r="BD42" s="64" t="n">
-        <v>330</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="BD42" s="64" t="n"/>
       <c r="BE42" s="64" t="n"/>
       <c r="BF42" s="16" t="n">
         <v>15</v>
@@ -14870,14 +14874,12 @@
       </c>
       <c r="BA43" s="16" t="n"/>
       <c r="BB43" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BC43" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD43" s="64" t="n">
-        <v>300</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BD43" s="64" t="n"/>
       <c r="BE43" s="64" t="n"/>
       <c r="BF43" s="16" t="n">
         <v>15</v>
@@ -15150,13 +15152,13 @@
       <c r="AZ44" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA44" s="16" t="n"/>
+      <c r="BA44" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB44" s="64" t="n"/>
       <c r="BC44" s="64" t="n"/>
       <c r="BD44" s="64" t="n"/>
-      <c r="BE44" s="64" t="n">
-        <v>340</v>
-      </c>
+      <c r="BE44" s="64" t="n"/>
       <c r="BF44" s="16" t="n">
         <v>15</v>
       </c>
@@ -15427,11 +15429,9 @@
         <v>10</v>
       </c>
       <c r="BA45" s="16" t="n"/>
-      <c r="BB45" s="64" t="n">
-        <v>190</v>
-      </c>
+      <c r="BB45" s="64" t="n"/>
       <c r="BC45" s="64" t="n">
-        <v>180</v>
+        <v>31</v>
       </c>
       <c r="BD45" s="64" t="n"/>
       <c r="BE45" s="64" t="n"/>
@@ -15705,11 +15705,9 @@
         <v>10</v>
       </c>
       <c r="BA46" s="16" t="n"/>
-      <c r="BB46" s="64" t="n">
-        <v>190</v>
-      </c>
+      <c r="BB46" s="64" t="n"/>
       <c r="BC46" s="64" t="n">
-        <v>180</v>
+        <v>31</v>
       </c>
       <c r="BD46" s="64" t="n"/>
       <c r="BE46" s="64" t="n"/>
@@ -15982,19 +15980,17 @@
       <c r="AZ47" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA47" s="16" t="n"/>
+      <c r="BA47" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB47" s="64" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="BC47" s="64" t="n">
-        <v>30</v>
-      </c>
-      <c r="BD47" s="64" t="n">
-        <v>140</v>
-      </c>
-      <c r="BE47" s="64" t="n">
-        <v>50</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD47" s="64" t="n"/>
+      <c r="BE47" s="64" t="n"/>
       <c r="BF47" s="16" t="n">
         <v>15</v>
       </c>
@@ -16270,13 +16266,11 @@
       </c>
       <c r="BA48" s="16" t="n"/>
       <c r="BB48" s="64" t="n"/>
-      <c r="BC48" s="64" t="n"/>
-      <c r="BD48" s="64" t="n">
-        <v>110</v>
-      </c>
-      <c r="BE48" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BC48" s="64" t="n">
+        <v>47</v>
+      </c>
+      <c r="BD48" s="64" t="n"/>
+      <c r="BE48" s="64" t="n"/>
       <c r="BF48" s="16" t="n">
         <v>15</v>
       </c>
@@ -16563,11 +16557,9 @@
         <v>15</v>
       </c>
       <c r="BA49" s="16" t="n"/>
-      <c r="BB49" s="64" t="n">
-        <v>70</v>
-      </c>
+      <c r="BB49" s="64" t="n"/>
       <c r="BC49" s="64" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="BD49" s="64" t="n"/>
       <c r="BE49" s="64" t="n"/>
@@ -16842,15 +16834,15 @@
       <c r="AZ50" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA50" s="16" t="n"/>
+      <c r="BA50" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB50" s="64" t="n"/>
-      <c r="BC50" s="64" t="n"/>
-      <c r="BD50" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE50" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BC50" s="64" t="n">
+        <v>31</v>
+      </c>
+      <c r="BD50" s="64" t="n"/>
+      <c r="BE50" s="64" t="n"/>
       <c r="BF50" s="16" t="n">
         <v>12.5</v>
       </c>
@@ -17146,14 +17138,12 @@
       </c>
       <c r="BA51" s="16" t="n"/>
       <c r="BB51" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BC51" s="64" t="n">
-        <v>130</v>
-      </c>
-      <c r="BD51" s="64" t="n">
-        <v>320</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD51" s="64" t="n"/>
       <c r="BE51" s="64" t="n"/>
       <c r="BF51" s="16" t="n">
         <v>15</v>
@@ -17699,9 +17689,13 @@
       <c r="AZ53" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA53" s="16" t="n"/>
+      <c r="BA53" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB53" s="64" t="n"/>
-      <c r="BC53" s="64" t="n"/>
+      <c r="BC53" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BD53" s="64" t="n"/>
       <c r="BE53" s="64" t="n"/>
       <c r="BF53" s="16" t="n">
@@ -18235,9 +18229,15 @@
       <c r="AZ55" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA55" s="16" t="n"/>
-      <c r="BB55" s="64" t="n"/>
-      <c r="BC55" s="64" t="n"/>
+      <c r="BA55" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB55" s="64" t="n">
+        <v>31</v>
+      </c>
+      <c r="BC55" s="64" t="n">
+        <v>47</v>
+      </c>
       <c r="BD55" s="64" t="n"/>
       <c r="BE55" s="64" t="n"/>
       <c r="BF55" s="16" t="inlineStr">
@@ -18511,16 +18511,16 @@
       <c r="AZ56" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA56" s="16" t="n"/>
+      <c r="BA56" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB56" s="64" t="n">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="BC56" s="64" t="n">
-        <v>120</v>
-      </c>
-      <c r="BD56" s="64" t="n">
-        <v>80</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BD56" s="64" t="n"/>
       <c r="BE56" s="64" t="n"/>
       <c r="BF56" s="16" t="n">
         <v>17.5</v>
@@ -18791,12 +18791,16 @@
       <c r="AZ57" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA57" s="16" t="n"/>
-      <c r="BB57" s="64" t="n"/>
-      <c r="BC57" s="64" t="n"/>
-      <c r="BD57" s="64" t="n">
-        <v>30</v>
-      </c>
+      <c r="BA57" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB57" s="64" t="n">
+        <v>31</v>
+      </c>
+      <c r="BC57" s="64" t="n">
+        <v>78</v>
+      </c>
+      <c r="BD57" s="64" t="n"/>
       <c r="BE57" s="64" t="n"/>
       <c r="BF57" s="16" t="n">
         <v>18</v>
@@ -19067,12 +19071,12 @@
       <c r="AZ58" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA58" s="16" t="n"/>
-      <c r="BB58" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA58" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB58" s="64" t="n"/>
       <c r="BC58" s="64" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BD58" s="64" t="n"/>
       <c r="BE58" s="64" t="n"/>
@@ -19346,16 +19350,16 @@
       <c r="AZ59" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA59" s="16" t="n"/>
+      <c r="BA59" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB59" s="64" t="n">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="BC59" s="64" t="n">
-        <v>90</v>
-      </c>
-      <c r="BD59" s="64" t="n">
-        <v>110</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BD59" s="64" t="n"/>
       <c r="BE59" s="64" t="n"/>
       <c r="BF59" s="16" t="inlineStr">
         <is>
@@ -19628,16 +19632,16 @@
       <c r="AZ60" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA60" s="16" t="n"/>
+      <c r="BA60" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB60" s="64" t="n">
-        <v>200</v>
+        <v>31</v>
       </c>
       <c r="BC60" s="64" t="n">
-        <v>250</v>
-      </c>
-      <c r="BD60" s="64" t="n">
-        <v>330</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD60" s="64" t="n"/>
       <c r="BE60" s="64" t="n"/>
       <c r="BF60" s="16" t="n">
         <v>15</v>
@@ -19909,11 +19913,9 @@
         <v>10</v>
       </c>
       <c r="BA61" s="16" t="n"/>
-      <c r="BB61" s="64" t="n">
-        <v>190</v>
-      </c>
+      <c r="BB61" s="64" t="n"/>
       <c r="BC61" s="64" t="n">
-        <v>180</v>
+        <v>31</v>
       </c>
       <c r="BD61" s="64" t="n"/>
       <c r="BE61" s="64" t="n"/>
@@ -20190,10 +20192,12 @@
       <c r="AZ62" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="BA62" s="16" t="n"/>
+      <c r="BA62" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB62" s="64" t="n"/>
       <c r="BC62" s="64" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="BD62" s="64" t="n"/>
       <c r="BE62" s="64" t="n"/>
@@ -20467,11 +20471,11 @@
         <v>12.5</v>
       </c>
       <c r="BA63" s="16" t="n"/>
-      <c r="BB63" s="64" t="n"/>
+      <c r="BB63" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BC63" s="64" t="n"/>
-      <c r="BD63" s="64" t="n">
-        <v>350</v>
-      </c>
+      <c r="BD63" s="64" t="n"/>
       <c r="BE63" s="64" t="n"/>
       <c r="BF63" s="16" t="n">
         <v>12.5</v>
@@ -20747,16 +20751,16 @@
       <c r="AZ64" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA64" s="16" t="n"/>
+      <c r="BA64" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB64" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BC64" s="64" t="n">
-        <v>140</v>
-      </c>
-      <c r="BD64" s="64" t="n">
-        <v>0</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD64" s="64" t="n"/>
       <c r="BE64" s="64" t="n"/>
       <c r="BF64" s="16" t="n">
         <v>15</v>
@@ -21030,13 +21034,13 @@
         <v>15</v>
       </c>
       <c r="BA65" s="16" t="n">
-        <v>83</v>
-      </c>
-      <c r="BB65" s="64" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="BB65" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BC65" s="64" t="n"/>
-      <c r="BD65" s="64" t="n">
-        <v>500</v>
-      </c>
+      <c r="BD65" s="64" t="n"/>
       <c r="BE65" s="64" t="n"/>
       <c r="BF65" s="16" t="inlineStr">
         <is>
@@ -21318,19 +21322,17 @@
       <c r="AZ66" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA66" s="16" t="n"/>
+      <c r="BA66" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB66" s="64" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="BC66" s="64" t="n">
-        <v>110</v>
-      </c>
-      <c r="BD66" s="64" t="n">
-        <v>80</v>
-      </c>
-      <c r="BE66" s="64" t="n">
-        <v>130</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD66" s="64" t="n"/>
+      <c r="BE66" s="64" t="n"/>
       <c r="BF66" s="16" t="n">
         <v>15</v>
       </c>
@@ -21606,14 +21608,12 @@
       </c>
       <c r="BA67" s="16" t="n"/>
       <c r="BB67" s="64" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="BC67" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD67" s="64" t="n">
-        <v>140</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="BD67" s="64" t="n"/>
       <c r="BE67" s="64" t="n"/>
       <c r="BF67" s="16" t="n">
         <v>20</v>
@@ -21894,19 +21894,17 @@
       <c r="AZ68" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA68" s="16" t="n"/>
-      <c r="BB68" s="64" t="n">
-        <v>220</v>
-      </c>
+      <c r="BA68" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB68" s="64" t="n"/>
       <c r="BC68" s="64" t="n">
-        <v>210</v>
+        <v>78</v>
       </c>
       <c r="BD68" s="64" t="n">
-        <v>570</v>
-      </c>
-      <c r="BE68" s="64" t="n">
-        <v>730</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BE68" s="64" t="n"/>
       <c r="BF68" s="16" t="n">
         <v>15</v>
       </c>
@@ -22188,16 +22186,16 @@
       <c r="AZ69" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA69" s="16" t="n"/>
+      <c r="BA69" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB69" s="64" t="n">
-        <v>130</v>
+        <v>31</v>
       </c>
       <c r="BC69" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD69" s="64" t="n">
-        <v>310</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD69" s="64" t="n"/>
       <c r="BE69" s="64" t="n"/>
       <c r="BF69" s="16" t="n">
         <v>15</v>
@@ -22460,16 +22458,18 @@
       <c r="AZ70" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="BA70" s="16" t="n"/>
+      <c r="BA70" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB70" s="64" t="n">
-        <v>140</v>
+        <v>78</v>
       </c>
       <c r="BC70" s="64" t="n">
-        <v>130</v>
+        <v>47</v>
       </c>
       <c r="BD70" s="64" t="n"/>
       <c r="BE70" s="64" t="n">
-        <v>520</v>
+        <v>31</v>
       </c>
       <c r="BF70" s="16" t="n">
         <v>15</v>
@@ -22752,14 +22752,12 @@
       </c>
       <c r="BA71" s="16" t="n"/>
       <c r="BB71" s="64" t="n">
-        <v>140</v>
+        <v>31</v>
       </c>
       <c r="BC71" s="64" t="n">
-        <v>120</v>
-      </c>
-      <c r="BD71" s="64" t="n">
-        <v>270</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD71" s="64" t="n"/>
       <c r="BE71" s="64" t="n"/>
       <c r="BF71" s="16" t="n">
         <v>20</v>
@@ -23030,16 +23028,16 @@
       <c r="AZ72" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA72" s="16" t="n"/>
+      <c r="BA72" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB72" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BC72" s="64" t="n">
-        <v>140</v>
-      </c>
-      <c r="BD72" s="64" t="n">
-        <v>360</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD72" s="64" t="n"/>
       <c r="BE72" s="64" t="n"/>
       <c r="BF72" s="16" t="inlineStr">
         <is>
@@ -23309,12 +23307,12 @@
       <c r="AZ73" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA73" s="16" t="n"/>
-      <c r="BB73" s="64" t="n">
-        <v>170</v>
-      </c>
+      <c r="BA73" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB73" s="64" t="n"/>
       <c r="BC73" s="64" t="n">
-        <v>130</v>
+        <v>31</v>
       </c>
       <c r="BD73" s="64" t="n"/>
       <c r="BE73" s="64" t="n"/>
@@ -23588,17 +23586,15 @@
       <c r="AZ74" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA74" s="16" t="n"/>
-      <c r="BB74" s="64" t="n">
-        <v>280</v>
-      </c>
+      <c r="BA74" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB74" s="64" t="n"/>
       <c r="BC74" s="64" t="n">
-        <v>260</v>
+        <v>31</v>
       </c>
       <c r="BD74" s="64" t="n"/>
-      <c r="BE74" s="64" t="n">
-        <v>110</v>
-      </c>
+      <c r="BE74" s="64" t="n"/>
       <c r="BF74" s="16" t="n">
         <v>17.5</v>
       </c>
@@ -23869,17 +23865,15 @@
       <c r="AZ75" s="16" t="n">
         <v>12.5</v>
       </c>
-      <c r="BA75" s="16" t="n"/>
-      <c r="BB75" s="64" t="n">
-        <v>110</v>
-      </c>
+      <c r="BA75" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB75" s="64" t="n"/>
       <c r="BC75" s="64" t="n">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="BD75" s="64" t="n"/>
-      <c r="BE75" s="64" t="n">
-        <v>340</v>
-      </c>
+      <c r="BE75" s="64" t="n"/>
       <c r="BF75" s="16" t="n">
         <v>15</v>
       </c>
@@ -24128,12 +24122,12 @@
       <c r="AX76" s="16" t="n"/>
       <c r="AY76" s="16" t="n"/>
       <c r="AZ76" s="16" t="n"/>
-      <c r="BA76" s="16" t="n"/>
-      <c r="BB76" s="64" t="n">
-        <v>180</v>
-      </c>
+      <c r="BA76" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB76" s="64" t="n"/>
       <c r="BC76" s="64" t="n">
-        <v>160</v>
+        <v>31</v>
       </c>
       <c r="BD76" s="64" t="n"/>
       <c r="BE76" s="64" t="n"/>
@@ -24370,19 +24364,17 @@
       <c r="AZ77" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA77" s="16" t="n"/>
-      <c r="BB77" s="64" t="n">
-        <v>670</v>
-      </c>
+      <c r="BA77" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB77" s="64" t="n"/>
       <c r="BC77" s="64" t="n">
-        <v>730</v>
+        <v>31</v>
       </c>
       <c r="BD77" s="64" t="n">
-        <v>510</v>
-      </c>
-      <c r="BE77" s="64" t="n">
-        <v>0</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="BE77" s="64" t="n"/>
       <c r="BF77" s="16" t="n">
         <v>15</v>
       </c>
@@ -24659,16 +24651,18 @@
       <c r="AZ78" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="BA78" s="16" t="n"/>
-      <c r="BB78" s="64" t="n"/>
+      <c r="BA78" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB78" s="64" t="n">
+        <v>78</v>
+      </c>
       <c r="BC78" s="64" t="n">
-        <v>70</v>
-      </c>
-      <c r="BD78" s="64" t="n">
-        <v>290</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="BD78" s="64" t="n"/>
       <c r="BE78" s="64" t="n">
-        <v>320</v>
+        <v>31</v>
       </c>
       <c r="BF78" s="16" t="n">
         <v>18</v>
@@ -24950,13 +24944,13 @@
       </c>
       <c r="BA79" s="16" t="n"/>
       <c r="BB79" s="64" t="n">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="BC79" s="64" t="n">
-        <v>60</v>
+        <v>109</v>
       </c>
       <c r="BD79" s="64" t="n">
-        <v>250</v>
+        <v>31</v>
       </c>
       <c r="BE79" s="64" t="n"/>
       <c r="BF79" s="16" t="n">
@@ -25236,15 +25230,15 @@
       <c r="AZ80" s="16" t="n">
         <v>12.5</v>
       </c>
-      <c r="BA80" s="16" t="n"/>
+      <c r="BA80" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB80" s="64" t="n"/>
       <c r="BC80" s="64" t="n"/>
       <c r="BD80" s="64" t="n">
-        <v>230</v>
-      </c>
-      <c r="BE80" s="64" t="n">
-        <v>450</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BE80" s="64" t="n"/>
       <c r="BF80" s="16" t="n">
         <v>17.5</v>
       </c>
@@ -25782,16 +25776,16 @@
       <c r="AZ82" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA82" s="16" t="n"/>
+      <c r="BA82" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB82" s="64" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="BC82" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD82" s="64" t="n">
-        <v>20</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD82" s="64" t="n"/>
       <c r="BE82" s="64" t="n"/>
       <c r="BF82" s="16" t="n">
         <v>20</v>
@@ -26076,19 +26070,17 @@
       <c r="AZ83" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA83" s="16" t="n"/>
+      <c r="BA83" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB83" s="64" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="BC83" s="64" t="n">
-        <v>110</v>
-      </c>
-      <c r="BD83" s="64" t="n">
-        <v>80</v>
-      </c>
-      <c r="BE83" s="64" t="n">
-        <v>130</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD83" s="64" t="n"/>
+      <c r="BE83" s="64" t="n"/>
       <c r="BF83" s="16" t="inlineStr">
         <is>
           <t>20-15</t>
@@ -26360,14 +26352,14 @@
       <c r="AZ84" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="BA84" s="16" t="n"/>
-      <c r="BB84" s="64" t="n"/>
-      <c r="BC84" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD84" s="64" t="n">
-        <v>40</v>
-      </c>
+      <c r="BA84" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB84" s="64" t="n">
+        <v>47</v>
+      </c>
+      <c r="BC84" s="64" t="n"/>
+      <c r="BD84" s="64" t="n"/>
       <c r="BE84" s="64" t="n"/>
       <c r="BF84" s="16" t="n">
         <v>15</v>
@@ -26645,13 +26637,11 @@
         <v>5</v>
       </c>
       <c r="BA85" s="16" t="n"/>
-      <c r="BB85" s="64" t="n"/>
-      <c r="BC85" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD85" s="64" t="n">
-        <v>20</v>
-      </c>
+      <c r="BB85" s="64" t="n">
+        <v>31</v>
+      </c>
+      <c r="BC85" s="64" t="n"/>
+      <c r="BD85" s="64" t="n"/>
       <c r="BE85" s="64" t="n"/>
       <c r="BF85" s="16" t="n">
         <v>15</v>
@@ -26928,11 +26918,13 @@
       <c r="AZ86" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="BA86" s="16" t="n"/>
+      <c r="BA86" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB86" s="64" t="n"/>
       <c r="BC86" s="64" t="n"/>
       <c r="BD86" s="64" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="BE86" s="64" t="n"/>
       <c r="BF86" s="16" t="n">
@@ -27207,19 +27199,17 @@
       <c r="AZ87" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA87" s="16" t="n"/>
+      <c r="BA87" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB87" s="64" t="n">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="BC87" s="64" t="n">
-        <v>110</v>
-      </c>
-      <c r="BD87" s="64" t="n">
-        <v>80</v>
-      </c>
-      <c r="BE87" s="64" t="n">
-        <v>130</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD87" s="64" t="n"/>
+      <c r="BE87" s="64" t="n"/>
       <c r="BF87" s="16" t="inlineStr">
         <is>
           <t>20-15</t>
@@ -27483,16 +27473,16 @@
       <c r="AZ88" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA88" s="16" t="n"/>
+      <c r="BA88" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB88" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BC88" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD88" s="64" t="n">
-        <v>280</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD88" s="64" t="n"/>
       <c r="BE88" s="64" t="n"/>
       <c r="BF88" s="16" t="n">
         <v>15</v>
@@ -27755,16 +27745,16 @@
       <c r="AZ89" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA89" s="16" t="n"/>
-      <c r="BB89" s="64" t="n">
-        <v>160</v>
-      </c>
+      <c r="BA89" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB89" s="64" t="n"/>
       <c r="BC89" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BD89" s="64" t="n"/>
       <c r="BE89" s="64" t="n">
-        <v>410</v>
+        <v>31</v>
       </c>
       <c r="BF89" s="16" t="n">
         <v>15</v>
@@ -28046,16 +28036,16 @@
       <c r="AZ90" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA90" s="16" t="n"/>
+      <c r="BA90" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB90" s="64" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="BC90" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD90" s="64" t="n">
-        <v>150</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD90" s="64" t="n"/>
       <c r="BE90" s="64" t="n"/>
       <c r="BF90" s="16" t="n">
         <v>17.5</v>
@@ -28338,15 +28328,15 @@
       <c r="AZ91" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA91" s="16" t="n"/>
-      <c r="BB91" s="64" t="n">
-        <v>170</v>
-      </c>
+      <c r="BA91" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB91" s="64" t="n"/>
       <c r="BC91" s="64" t="n">
-        <v>130</v>
+        <v>31</v>
       </c>
       <c r="BD91" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BE91" s="64" t="n"/>
       <c r="BF91" s="16" t="inlineStr">
@@ -28616,17 +28606,19 @@
       <c r="AZ92" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA92" s="16" t="n"/>
-      <c r="BB92" s="64" t="n">
-        <v>10</v>
-      </c>
+      <c r="BA92" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB92" s="64" t="n"/>
       <c r="BC92" s="64" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BD92" s="64" t="n">
-        <v>190</v>
-      </c>
-      <c r="BE92" s="64" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="BE92" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BF92" s="16" t="n">
         <v>15</v>
       </c>
@@ -28909,15 +28901,17 @@
       <c r="AZ93" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA93" s="16" t="n"/>
-      <c r="BB93" s="64" t="n"/>
-      <c r="BC93" s="64" t="n"/>
-      <c r="BD93" s="64" t="n">
-        <v>10</v>
-      </c>
-      <c r="BE93" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA93" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB93" s="64" t="n">
+        <v>156</v>
+      </c>
+      <c r="BC93" s="64" t="n">
+        <v>78</v>
+      </c>
+      <c r="BD93" s="64" t="n"/>
+      <c r="BE93" s="64" t="n"/>
       <c r="BF93" s="16" t="n">
         <v>20</v>
       </c>
@@ -29183,17 +29177,19 @@
       <c r="AZ94" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA94" s="16" t="n"/>
-      <c r="BB94" s="64" t="n">
-        <v>130</v>
-      </c>
+      <c r="BA94" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB94" s="64" t="n"/>
       <c r="BC94" s="64" t="n">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="BD94" s="64" t="n">
-        <v>310</v>
-      </c>
-      <c r="BE94" s="64" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="BE94" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BF94" s="16" t="n">
         <v>15</v>
       </c>
@@ -29464,17 +29460,19 @@
       <c r="AZ95" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA95" s="16" t="n"/>
-      <c r="BB95" s="64" t="n">
-        <v>30</v>
-      </c>
+      <c r="BA95" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB95" s="64" t="n"/>
       <c r="BC95" s="64" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BD95" s="64" t="n">
-        <v>210</v>
-      </c>
-      <c r="BE95" s="64" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="BE95" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BF95" s="16" t="n">
         <v>15</v>
       </c>
@@ -29745,15 +29743,15 @@
       <c r="AZ96" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA96" s="16" t="n"/>
-      <c r="BB96" s="64" t="n">
-        <v>120</v>
-      </c>
+      <c r="BA96" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB96" s="64" t="n"/>
       <c r="BC96" s="64" t="n">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="BD96" s="64" t="n">
-        <v>200</v>
+        <v>47</v>
       </c>
       <c r="BE96" s="64" t="n"/>
       <c r="BF96" s="16" t="n">
@@ -30021,15 +30019,15 @@
       <c r="AZ97" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA97" s="16" t="n"/>
+      <c r="BA97" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB97" s="64" t="n"/>
-      <c r="BC97" s="79" t="n"/>
-      <c r="BD97" s="64" t="n">
-        <v>290</v>
-      </c>
-      <c r="BE97" s="79" t="n">
-        <v>0</v>
-      </c>
+      <c r="BC97" s="79" t="n">
+        <v>31</v>
+      </c>
+      <c r="BD97" s="64" t="n"/>
+      <c r="BE97" s="79" t="n"/>
       <c r="BF97" s="16" t="n">
         <v>17.5</v>
       </c>
@@ -30300,11 +30298,9 @@
       <c r="BA98" s="16" t="n"/>
       <c r="BB98" s="64" t="n"/>
       <c r="BC98" s="64" t="n"/>
-      <c r="BD98" s="64" t="n">
-        <v>100</v>
-      </c>
+      <c r="BD98" s="64" t="n"/>
       <c r="BE98" s="64" t="n">
-        <v>60</v>
+        <v>156</v>
       </c>
       <c r="BF98" s="16" t="n">
         <v>17.5</v>
@@ -30568,9 +30564,7 @@
       <c r="AZ99" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA99" s="16" t="n">
-        <v>100</v>
-      </c>
+      <c r="BA99" s="16" t="n"/>
       <c r="BB99" s="64" t="n"/>
       <c r="BC99" s="64" t="n"/>
       <c r="BD99" s="64" t="n"/>
@@ -30852,14 +30846,12 @@
         <v>12.5</v>
       </c>
       <c r="BA100" s="16" t="n"/>
-      <c r="BB100" s="64" t="n">
-        <v>70</v>
-      </c>
+      <c r="BB100" s="64" t="n"/>
       <c r="BC100" s="64" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="BD100" s="64" t="n">
-        <v>240</v>
+        <v>31</v>
       </c>
       <c r="BE100" s="64" t="n"/>
       <c r="BF100" s="16" t="n">
@@ -31132,13 +31124,11 @@
         <v>10</v>
       </c>
       <c r="BA101" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="BB101" s="64" t="n">
-        <v>180</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BB101" s="64" t="n"/>
       <c r="BC101" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BD101" s="64" t="n"/>
       <c r="BE101" s="64" t="n"/>
@@ -31408,15 +31398,19 @@
       <c r="AZ102" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA102" s="16" t="n"/>
+      <c r="BA102" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB102" s="64" t="n"/>
       <c r="BC102" s="64" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="BD102" s="64" t="n">
-        <v>40</v>
-      </c>
-      <c r="BE102" s="64" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="BE102" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BF102" s="16" t="n">
         <v>15</v>
       </c>
@@ -31674,12 +31668,14 @@
       <c r="AZ103" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA103" s="16" t="n"/>
+      <c r="BA103" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB103" s="64" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BC103" s="64" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BD103" s="64" t="n"/>
       <c r="BE103" s="64" t="n"/>
@@ -31952,17 +31948,17 @@
       <c r="AZ104" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA104" s="16" t="n"/>
+      <c r="BA104" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB104" s="64" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="BC104" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD104" s="64" t="n"/>
-      <c r="BE104" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BE104" s="64" t="n"/>
       <c r="BF104" s="16" t="n">
         <v>22</v>
       </c>
@@ -32229,15 +32225,15 @@
       <c r="AZ105" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA105" s="16" t="n"/>
-      <c r="BB105" s="64" t="n">
-        <v>10</v>
-      </c>
+      <c r="BA105" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB105" s="64" t="n"/>
       <c r="BC105" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD105" s="64" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="BE105" s="64" t="n"/>
       <c r="BF105" s="16" t="n">
@@ -32767,16 +32763,14 @@
       <c r="AZ107" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA107" s="16" t="n"/>
-      <c r="BB107" s="64" t="n">
-        <v>80</v>
-      </c>
+      <c r="BA107" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB107" s="64" t="n"/>
       <c r="BC107" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD107" s="64" t="n">
-        <v>130</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD107" s="64" t="n"/>
       <c r="BE107" s="79" t="n"/>
       <c r="BF107" s="16" t="n">
         <v>15</v>
@@ -33304,15 +33298,19 @@
       <c r="AZ109" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA109" s="16" t="n"/>
+      <c r="BA109" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB109" s="64" t="n"/>
       <c r="BC109" s="64" t="n">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="BD109" s="64" t="n">
-        <v>250</v>
-      </c>
-      <c r="BE109" s="64" t="n"/>
+        <v>31</v>
+      </c>
+      <c r="BE109" s="64" t="n">
+        <v>31</v>
+      </c>
       <c r="BF109" s="16" t="n">
         <v>15</v>
       </c>
@@ -33847,14 +33845,12 @@
         <v>15</v>
       </c>
       <c r="BA111" s="16" t="n"/>
-      <c r="BB111" s="64" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC111" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BB111" s="64" t="n"/>
+      <c r="BC111" s="64" t="n"/>
       <c r="BD111" s="64" t="n"/>
-      <c r="BE111" s="64" t="n"/>
+      <c r="BE111" s="64" t="n">
+        <v>156</v>
+      </c>
       <c r="BF111" s="16" t="n">
         <v>15</v>
       </c>
@@ -34119,7 +34115,7 @@
         <v>15</v>
       </c>
       <c r="BA112" s="16" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="BB112" s="64" t="n"/>
       <c r="BC112" s="64" t="n"/>
@@ -34395,15 +34391,17 @@
       <c r="AZ113" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA113" s="16" t="n"/>
-      <c r="BB113" s="64" t="n"/>
-      <c r="BC113" s="64" t="n"/>
-      <c r="BD113" s="64" t="n">
-        <v>10</v>
-      </c>
-      <c r="BE113" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA113" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB113" s="64" t="n">
+        <v>234</v>
+      </c>
+      <c r="BC113" s="64" t="n">
+        <v>78</v>
+      </c>
+      <c r="BD113" s="64" t="n"/>
+      <c r="BE113" s="64" t="n"/>
       <c r="BF113" s="16" t="inlineStr">
         <is>
           <t>25-20</t>
@@ -34676,17 +34674,15 @@
         <v>15</v>
       </c>
       <c r="BA114" s="16" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="BB114" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BC114" s="64" t="n">
-        <v>140</v>
-      </c>
-      <c r="BD114" s="64" t="n">
-        <v>360</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD114" s="64" t="n"/>
       <c r="BE114" s="64" t="n"/>
       <c r="BF114" s="16" t="n">
         <v>17.5</v>
@@ -34959,17 +34955,15 @@
         <v>15</v>
       </c>
       <c r="BA115" s="16" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="BB115" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BC115" s="64" t="n">
-        <v>140</v>
-      </c>
-      <c r="BD115" s="64" t="n">
-        <v>360</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD115" s="64" t="n"/>
       <c r="BE115" s="64" t="n"/>
       <c r="BF115" s="16" t="n">
         <v>17.5</v>
@@ -35242,17 +35236,15 @@
         <v>15</v>
       </c>
       <c r="BA116" s="16" t="n">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="BB116" s="64" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
       <c r="BC116" s="64" t="n">
-        <v>140</v>
-      </c>
-      <c r="BD116" s="64" t="n">
-        <v>360</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BD116" s="64" t="n"/>
       <c r="BE116" s="64" t="n"/>
       <c r="BF116" s="16" t="n">
         <v>17.5</v>
@@ -35516,12 +35508,14 @@
       <c r="AZ117" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA117" s="16" t="n"/>
+      <c r="BA117" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB117" s="64" t="n"/>
       <c r="BC117" s="64" t="n"/>
       <c r="BD117" s="64" t="n"/>
       <c r="BE117" s="64" t="n">
-        <v>750</v>
+        <v>47</v>
       </c>
       <c r="BF117" s="16" t="n">
         <v>15</v>
@@ -35793,17 +35787,15 @@
       <c r="AZ118" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA118" s="16" t="n"/>
-      <c r="BB118" s="64" t="n">
-        <v>90</v>
-      </c>
+      <c r="BA118" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB118" s="64" t="n"/>
       <c r="BC118" s="64" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD118" s="64" t="n"/>
-      <c r="BE118" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BE118" s="64" t="n"/>
       <c r="BF118" s="16" t="n">
         <v>15</v>
       </c>
@@ -36070,13 +36062,15 @@
       <c r="AZ119" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA119" s="77" t="n"/>
+      <c r="BA119" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB119" s="79" t="n"/>
-      <c r="BC119" s="79" t="n"/>
+      <c r="BC119" s="79" t="n">
+        <v>31</v>
+      </c>
       <c r="BD119" s="79" t="n"/>
-      <c r="BE119" s="79" t="n">
-        <v>0</v>
-      </c>
+      <c r="BE119" s="79" t="n"/>
       <c r="BF119" s="77" t="n">
         <v>20</v>
       </c>
@@ -36343,17 +36337,17 @@
       <c r="AZ120" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA120" s="77" t="n"/>
+      <c r="BA120" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB120" s="79" t="n">
-        <v>270</v>
+        <v>47</v>
       </c>
       <c r="BC120" s="79" t="n">
-        <v>390</v>
+        <v>31</v>
       </c>
       <c r="BD120" s="111" t="n"/>
-      <c r="BE120" s="111" t="n">
-        <v>590</v>
-      </c>
+      <c r="BE120" s="111" t="n"/>
       <c r="BF120" s="77" t="inlineStr">
         <is>
           <t>22-16</t>
@@ -36621,18 +36615,18 @@
       <c r="AZ121" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA121" s="77" t="n"/>
-      <c r="BB121" s="79" t="n">
-        <v>310</v>
-      </c>
+      <c r="BA121" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB121" s="79" t="n"/>
       <c r="BC121" s="79" t="n">
-        <v>330</v>
+        <v>47</v>
       </c>
       <c r="BD121" s="79" t="n">
-        <v>230</v>
+        <v>109</v>
       </c>
       <c r="BE121" s="79" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BF121" s="77" t="inlineStr">
         <is>
@@ -37168,19 +37162,17 @@
         <v>15</v>
       </c>
       <c r="BA123" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="BB123" s="64" t="n">
-        <v>720</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BB123" s="64" t="n"/>
       <c r="BC123" s="64" t="n">
-        <v>760</v>
+        <v>31</v>
       </c>
       <c r="BD123" s="64" t="n">
-        <v>770</v>
+        <v>109</v>
       </c>
       <c r="BE123" s="79" t="n">
-        <v>800</v>
+        <v>47</v>
       </c>
       <c r="BF123" s="16" t="inlineStr">
         <is>
@@ -37453,11 +37445,13 @@
       <c r="AZ124" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA124" s="16" t="n"/>
+      <c r="BA124" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB124" s="16" t="n"/>
       <c r="BC124" s="77" t="n"/>
       <c r="BD124" s="112" t="n">
-        <v>220</v>
+        <v>47</v>
       </c>
       <c r="BE124" s="77" t="n"/>
       <c r="BF124" s="16" t="inlineStr">
@@ -37727,19 +37721,17 @@
       <c r="AZ125" s="77" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA125" s="77" t="n"/>
-      <c r="BB125" s="79" t="n">
-        <v>150</v>
-      </c>
+      <c r="BA125" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB125" s="79" t="n"/>
       <c r="BC125" s="79" t="n">
-        <v>140</v>
+        <v>31</v>
       </c>
       <c r="BD125" s="79" t="n">
-        <v>70</v>
-      </c>
-      <c r="BE125" s="79" t="n">
-        <v>260</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="BE125" s="79" t="n"/>
       <c r="BF125" s="77" t="n">
         <v>23</v>
       </c>
@@ -38005,12 +37997,12 @@
       <c r="AZ126" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA126" s="77" t="n"/>
-      <c r="BB126" s="79" t="n">
-        <v>420</v>
-      </c>
+      <c r="BA126" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB126" s="79" t="n"/>
       <c r="BC126" s="79" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD126" s="79" t="n"/>
       <c r="BE126" s="79" t="n"/>
@@ -38291,12 +38283,12 @@
       <c r="AZ127" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA127" s="77" t="n"/>
-      <c r="BB127" s="64" t="n">
-        <v>420</v>
-      </c>
+      <c r="BA127" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB127" s="64" t="n"/>
       <c r="BC127" s="79" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD127" s="79" t="n"/>
       <c r="BE127" s="79" t="n"/>
@@ -38566,16 +38558,14 @@
         <v>15</v>
       </c>
       <c r="BA128" s="77" t="n">
-        <v>83</v>
+        <v>31</v>
       </c>
       <c r="BB128" s="77" t="n"/>
       <c r="BC128" s="77" t="n"/>
       <c r="BD128" s="79" t="n">
-        <v>470</v>
-      </c>
-      <c r="BE128" s="79" t="n">
-        <v>1080</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BE128" s="79" t="n"/>
       <c r="BF128" s="77" t="n">
         <v>15</v>
       </c>
@@ -38855,14 +38845,16 @@
       <c r="AZ129" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA129" s="77" t="n"/>
+      <c r="BA129" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB129" s="79" t="n"/>
       <c r="BC129" s="79" t="n"/>
       <c r="BD129" s="79" t="n">
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="BE129" s="79" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="BF129" s="77" t="inlineStr">
         <is>
@@ -39133,14 +39125,16 @@
       <c r="AZ130" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA130" s="16" t="n"/>
+      <c r="BA130" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB130" s="16" t="n"/>
       <c r="BC130" s="77" t="n"/>
       <c r="BD130" s="64" t="n">
-        <v>400</v>
+        <v>78</v>
       </c>
       <c r="BE130" s="79" t="n">
-        <v>720</v>
+        <v>31</v>
       </c>
       <c r="BF130" s="16" t="inlineStr">
         <is>
@@ -39409,17 +39403,15 @@
       <c r="AZ131" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="BA131" s="16" t="n"/>
-      <c r="BB131" s="64" t="n">
-        <v>490</v>
-      </c>
+      <c r="BA131" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB131" s="64" t="n"/>
       <c r="BC131" s="79" t="n">
-        <v>440</v>
+        <v>31</v>
       </c>
       <c r="BD131" s="64" t="n"/>
-      <c r="BE131" s="79" t="n">
-        <v>120</v>
-      </c>
+      <c r="BE131" s="79" t="n"/>
       <c r="BF131" s="16" t="inlineStr">
         <is>
           <t>22.5-15</t>
@@ -39959,14 +39951,16 @@
       <c r="AZ133" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="BA133" s="16" t="n"/>
+      <c r="BA133" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB133" s="64" t="n"/>
       <c r="BC133" s="79" t="n">
-        <v>290</v>
+        <v>31</v>
       </c>
       <c r="BD133" s="64" t="n"/>
       <c r="BE133" s="79" t="n">
-        <v>340</v>
+        <v>47</v>
       </c>
       <c r="BF133" s="16" t="inlineStr">
         <is>
@@ -40799,17 +40793,19 @@
       <c r="AZ136" s="16" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA136" s="16" t="n"/>
-      <c r="BB136" s="64" t="n">
-        <v>0</v>
-      </c>
+      <c r="BA136" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB136" s="64" t="n"/>
       <c r="BC136" s="79" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="BD136" s="64" t="n">
-        <v>80</v>
-      </c>
-      <c r="BE136" s="79" t="n"/>
+        <v>109</v>
+      </c>
+      <c r="BE136" s="79" t="n">
+        <v>109</v>
+      </c>
       <c r="BF136" s="16" t="n">
         <v>25</v>
       </c>
@@ -41077,14 +41073,16 @@
       <c r="AZ137" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA137" s="16" t="n"/>
+      <c r="BA137" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB137" s="64" t="n"/>
       <c r="BC137" s="64" t="n"/>
       <c r="BD137" s="112" t="n">
-        <v>430</v>
+        <v>78</v>
       </c>
       <c r="BE137" s="111" t="n">
-        <v>510</v>
+        <v>31</v>
       </c>
       <c r="BF137" s="16" t="inlineStr">
         <is>
@@ -41635,15 +41633,15 @@
       <c r="AZ139" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA139" s="16" t="n"/>
-      <c r="BB139" s="112" t="n">
-        <v>220</v>
-      </c>
+      <c r="BA139" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB139" s="112" t="n"/>
       <c r="BC139" s="112" t="n">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="BD139" s="112" t="n">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="BE139" s="112" t="n"/>
       <c r="BF139" s="16" t="inlineStr">
@@ -41916,15 +41914,15 @@
         <v>15</v>
       </c>
       <c r="BA140" s="77" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="BB140" s="77" t="n"/>
       <c r="BC140" s="79" t="n"/>
       <c r="BD140" s="79" t="n">
-        <v>400</v>
+        <v>31</v>
       </c>
       <c r="BE140" s="79" t="n">
-        <v>640</v>
+        <v>31</v>
       </c>
       <c r="BF140" s="77" t="inlineStr">
         <is>
@@ -42195,14 +42193,16 @@
       <c r="AZ141" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA141" s="16" t="n"/>
+      <c r="BA141" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB141" s="16" t="n"/>
       <c r="BC141" s="77" t="n"/>
       <c r="BD141" s="112" t="n">
-        <v>420</v>
+        <v>234</v>
       </c>
       <c r="BE141" s="111" t="n">
-        <v>640</v>
+        <v>47</v>
       </c>
       <c r="BF141" s="77" t="inlineStr">
         <is>
@@ -42468,19 +42468,15 @@
         <v>15</v>
       </c>
       <c r="BA142" s="77" t="n">
-        <v>10</v>
-      </c>
-      <c r="BB142" s="79" t="n">
-        <v>110</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BB142" s="79" t="n"/>
       <c r="BC142" s="79" t="n">
-        <v>90</v>
-      </c>
-      <c r="BD142" s="79" t="n">
-        <v>100</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BD142" s="79" t="n"/>
       <c r="BE142" s="79" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="BF142" s="77" t="inlineStr">
         <is>
@@ -43295,18 +43291,20 @@
       <c r="AZ145" s="77" t="n">
         <v>20</v>
       </c>
-      <c r="BA145" s="77" t="n"/>
+      <c r="BA145" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB145" s="79" t="n">
-        <v>300</v>
+        <v>78</v>
       </c>
       <c r="BC145" s="79" t="n">
-        <v>360</v>
+        <v>78</v>
       </c>
       <c r="BD145" s="79" t="n">
-        <v>270</v>
+        <v>31</v>
       </c>
       <c r="BE145" s="79" t="n">
-        <v>320</v>
+        <v>31</v>
       </c>
       <c r="BF145" s="16" t="inlineStr">
         <is>
@@ -43584,7 +43582,7 @@
       <c r="BC146" s="77" t="n"/>
       <c r="BD146" s="16" t="n"/>
       <c r="BE146" s="79" t="n">
-        <v>670</v>
+        <v>31</v>
       </c>
       <c r="BF146" s="16" t="n">
         <v>23</v>
@@ -43861,17 +43859,15 @@
       </c>
       <c r="BA147" s="77" t="n"/>
       <c r="BB147" s="64" t="n">
-        <v>320</v>
+        <v>234</v>
       </c>
       <c r="BC147" s="64" t="n">
-        <v>340</v>
+        <v>31</v>
       </c>
       <c r="BD147" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="BE147" s="79" t="n">
-        <v>530</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="BE147" s="79" t="n"/>
       <c r="BF147" s="16" t="n">
         <v>23</v>
       </c>
@@ -44143,14 +44139,16 @@
       <c r="AZ148" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA148" s="77" t="n"/>
+      <c r="BA148" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB148" s="16" t="n"/>
       <c r="BC148" s="16" t="n"/>
       <c r="BD148" s="79" t="n">
-        <v>400</v>
+        <v>31</v>
       </c>
       <c r="BE148" s="79" t="n">
-        <v>640</v>
+        <v>31</v>
       </c>
       <c r="BF148" s="16" t="inlineStr">
         <is>
@@ -44421,14 +44419,16 @@
       <c r="AZ149" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="BA149" s="16" t="n"/>
+      <c r="BA149" s="16" t="n">
+        <v>31</v>
+      </c>
       <c r="BB149" s="64" t="n"/>
       <c r="BC149" s="79" t="n"/>
       <c r="BD149" s="64" t="n">
-        <v>340</v>
+        <v>234</v>
       </c>
       <c r="BE149" s="79" t="n">
-        <v>350</v>
+        <v>109</v>
       </c>
       <c r="BF149" s="16" t="inlineStr">
         <is>
@@ -44697,18 +44697,16 @@
       <c r="AZ150" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA150" s="77" t="n"/>
-      <c r="BB150" s="79" t="n">
-        <v>110</v>
-      </c>
+      <c r="BA150" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB150" s="79" t="n"/>
       <c r="BC150" s="79" t="n">
-        <v>90</v>
-      </c>
-      <c r="BD150" s="79" t="n">
-        <v>100</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BD150" s="79" t="n"/>
       <c r="BE150" s="79" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="BF150" s="77" t="inlineStr">
         <is>
@@ -44977,17 +44975,17 @@
       <c r="AZ151" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="BA151" s="77" t="n"/>
+      <c r="BA151" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB151" s="79" t="n">
-        <v>270</v>
+        <v>47</v>
       </c>
       <c r="BC151" s="79" t="n">
-        <v>390</v>
+        <v>31</v>
       </c>
       <c r="BD151" s="111" t="n"/>
-      <c r="BE151" s="111" t="n">
-        <v>590</v>
-      </c>
+      <c r="BE151" s="111" t="n"/>
       <c r="BF151" s="77" t="inlineStr">
         <is>
           <t>22-16</t>
@@ -45541,10 +45539,12 @@
       <c r="AZ153" s="77" t="n">
         <v>20</v>
       </c>
-      <c r="BA153" s="77" t="n"/>
+      <c r="BA153" s="77" t="n">
+        <v>31</v>
+      </c>
       <c r="BB153" s="79" t="n"/>
       <c r="BC153" s="79" t="n">
-        <v>280</v>
+        <v>47</v>
       </c>
       <c r="BD153" s="79" t="n"/>
       <c r="BE153" s="79" t="n"/>
@@ -46085,19 +46085,17 @@
       <c r="AZ155" s="77" t="n">
         <v>7.5</v>
       </c>
-      <c r="BA155" s="77" t="n"/>
-      <c r="BB155" s="79" t="n">
-        <v>170</v>
-      </c>
+      <c r="BA155" s="77" t="n">
+        <v>31</v>
+      </c>
+      <c r="BB155" s="79" t="n"/>
       <c r="BC155" s="79" t="n">
-        <v>160</v>
+        <v>47</v>
       </c>
       <c r="BD155" s="79" t="n">
-        <v>80</v>
-      </c>
-      <c r="BE155" s="79" t="n">
-        <v>290</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="BE155" s="79" t="n"/>
       <c r="BF155" s="77" t="n">
         <v>23</v>
       </c>
@@ -46368,19 +46366,17 @@
         <v>15</v>
       </c>
       <c r="BA156" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="BB156" s="64" t="n">
-        <v>720</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="BB156" s="64" t="n"/>
       <c r="BC156" s="64" t="n">
-        <v>760</v>
+        <v>31</v>
       </c>
       <c r="BD156" s="64" t="n">
-        <v>770</v>
+        <v>78</v>
       </c>
       <c r="BE156" s="79" t="n">
-        <v>930</v>
+        <v>47</v>
       </c>
       <c r="BF156" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Read actual engagement values from ME file summary (rows 29-30, cols JH-JK)
Instead of estimating zone-specific engagement from Z offsets alone, now reads
pre-computed values directly from the ME file's "Sceondary Cutting Structure"
summary area. Handles v6 (cols JH/JI) and v7/v8 (cols JJ/JK) column mappings.
ME file values override Z-offset estimates when available; estimates remain as
fallback for files without the summary block.

BB/BC/BD/BE population improved (e.g., BB: 52→84, BD: 35→73).
Values verified against known ME file data (9944, 2110, 4288, 5674).

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Bit Applications Tool r2.xlsx
+++ b/Bit Applications Tool r2.xlsx
@@ -6309,9 +6309,11 @@
       <c r="BA12" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB12" s="64" t="n"/>
+      <c r="BB12" s="64" t="n">
+        <v>110</v>
+      </c>
       <c r="BC12" s="64" t="n">
-        <v>31</v>
+        <v>110</v>
       </c>
       <c r="BD12" s="64" t="n"/>
       <c r="BE12" s="64" t="n"/>
@@ -6850,10 +6852,10 @@
         <v>31</v>
       </c>
       <c r="BB14" s="64" t="n">
-        <v>234</v>
+        <v>110</v>
       </c>
       <c r="BC14" s="64" t="n">
-        <v>31</v>
+        <v>120</v>
       </c>
       <c r="BD14" s="64" t="n"/>
       <c r="BE14" s="64" t="n"/>
@@ -8712,7 +8714,7 @@
       </c>
       <c r="BA21" s="16" t="n"/>
       <c r="BB21" s="64" t="n">
-        <v>156</v>
+        <v>50</v>
       </c>
       <c r="BC21" s="64" t="n">
         <v>31</v>
@@ -9779,7 +9781,9 @@
         <v>10</v>
       </c>
       <c r="BA25" s="16" t="n"/>
-      <c r="BB25" s="64" t="n"/>
+      <c r="BB25" s="64" t="n">
+        <v>10</v>
+      </c>
       <c r="BC25" s="64" t="n">
         <v>31</v>
       </c>
@@ -10598,13 +10602,17 @@
         <v>31</v>
       </c>
       <c r="BB28" s="64" t="n">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="BC28" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD28" s="64" t="n"/>
-      <c r="BE28" s="64" t="n"/>
+        <v>110</v>
+      </c>
+      <c r="BD28" s="64" t="n">
+        <v>80</v>
+      </c>
+      <c r="BE28" s="64" t="n">
+        <v>130</v>
+      </c>
       <c r="BF28" s="16" t="n">
         <v>15</v>
       </c>
@@ -10875,9 +10883,11 @@
       <c r="BA29" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB29" s="64" t="n"/>
+      <c r="BB29" s="64" t="n">
+        <v>70</v>
+      </c>
       <c r="BC29" s="64" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="BD29" s="64" t="n"/>
       <c r="BE29" s="64" t="n"/>
@@ -11153,9 +11163,11 @@
       <c r="BA30" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB30" s="64" t="n"/>
+      <c r="BB30" s="64" t="n">
+        <v>110</v>
+      </c>
       <c r="BC30" s="64" t="n">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="BD30" s="64" t="n"/>
       <c r="BE30" s="64" t="n"/>
@@ -11456,10 +11468,10 @@
       </c>
       <c r="BA31" s="16" t="n"/>
       <c r="BB31" s="64" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="BC31" s="64" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="BD31" s="64" t="n"/>
       <c r="BE31" s="64" t="n"/>
@@ -13170,13 +13182,17 @@
         <v>31</v>
       </c>
       <c r="BB37" s="64" t="n">
-        <v>156</v>
+        <v>70</v>
       </c>
       <c r="BC37" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD37" s="64" t="n"/>
-      <c r="BE37" s="64" t="n"/>
+        <v>120</v>
+      </c>
+      <c r="BD37" s="64" t="n">
+        <v>70</v>
+      </c>
+      <c r="BE37" s="64" t="n">
+        <v>80</v>
+      </c>
       <c r="BF37" s="16" t="n">
         <v>15</v>
       </c>
@@ -14301,9 +14317,11 @@
         <v>31</v>
       </c>
       <c r="BC41" s="64" t="n">
-        <v>47</v>
-      </c>
-      <c r="BD41" s="64" t="n"/>
+        <v>80</v>
+      </c>
+      <c r="BD41" s="64" t="n">
+        <v>410</v>
+      </c>
       <c r="BE41" s="64" t="n"/>
       <c r="BF41" s="16" t="n">
         <v>15</v>
@@ -14580,12 +14598,14 @@
         <v>31</v>
       </c>
       <c r="BB42" s="64" t="n">
-        <v>31</v>
+        <v>230</v>
       </c>
       <c r="BC42" s="64" t="n">
-        <v>78</v>
-      </c>
-      <c r="BD42" s="64" t="n"/>
+        <v>200</v>
+      </c>
+      <c r="BD42" s="64" t="n">
+        <v>330</v>
+      </c>
       <c r="BE42" s="64" t="n"/>
       <c r="BF42" s="16" t="n">
         <v>15</v>
@@ -14879,7 +14899,9 @@
       <c r="BC43" s="64" t="n">
         <v>47</v>
       </c>
-      <c r="BD43" s="64" t="n"/>
+      <c r="BD43" s="64" t="n">
+        <v>300</v>
+      </c>
       <c r="BE43" s="64" t="n"/>
       <c r="BF43" s="16" t="n">
         <v>15</v>
@@ -15157,7 +15179,9 @@
       </c>
       <c r="BB44" s="64" t="n"/>
       <c r="BC44" s="64" t="n"/>
-      <c r="BD44" s="64" t="n"/>
+      <c r="BD44" s="64" t="n">
+        <v>340</v>
+      </c>
       <c r="BE44" s="64" t="n"/>
       <c r="BF44" s="16" t="n">
         <v>15</v>
@@ -15429,9 +15453,11 @@
         <v>10</v>
       </c>
       <c r="BA45" s="16" t="n"/>
-      <c r="BB45" s="64" t="n"/>
+      <c r="BB45" s="64" t="n">
+        <v>190</v>
+      </c>
       <c r="BC45" s="64" t="n">
-        <v>31</v>
+        <v>180</v>
       </c>
       <c r="BD45" s="64" t="n"/>
       <c r="BE45" s="64" t="n"/>
@@ -15705,9 +15731,11 @@
         <v>10</v>
       </c>
       <c r="BA46" s="16" t="n"/>
-      <c r="BB46" s="64" t="n"/>
+      <c r="BB46" s="64" t="n">
+        <v>190</v>
+      </c>
       <c r="BC46" s="64" t="n">
-        <v>31</v>
+        <v>180</v>
       </c>
       <c r="BD46" s="64" t="n"/>
       <c r="BE46" s="64" t="n"/>
@@ -15984,13 +16012,17 @@
         <v>31</v>
       </c>
       <c r="BB47" s="64" t="n">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="BC47" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD47" s="64" t="n"/>
-      <c r="BE47" s="64" t="n"/>
+        <v>30</v>
+      </c>
+      <c r="BD47" s="64" t="n">
+        <v>140</v>
+      </c>
+      <c r="BE47" s="64" t="n">
+        <v>50</v>
+      </c>
       <c r="BF47" s="16" t="n">
         <v>15</v>
       </c>
@@ -16269,7 +16301,9 @@
       <c r="BC48" s="64" t="n">
         <v>47</v>
       </c>
-      <c r="BD48" s="64" t="n"/>
+      <c r="BD48" s="64" t="n">
+        <v>110</v>
+      </c>
       <c r="BE48" s="64" t="n"/>
       <c r="BF48" s="16" t="n">
         <v>15</v>
@@ -16557,9 +16591,11 @@
         <v>15</v>
       </c>
       <c r="BA49" s="16" t="n"/>
-      <c r="BB49" s="64" t="n"/>
+      <c r="BB49" s="64" t="n">
+        <v>70</v>
+      </c>
       <c r="BC49" s="64" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="BD49" s="64" t="n"/>
       <c r="BE49" s="64" t="n"/>
@@ -17138,12 +17174,14 @@
       </c>
       <c r="BA51" s="16" t="n"/>
       <c r="BB51" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BC51" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD51" s="64" t="n"/>
+        <v>130</v>
+      </c>
+      <c r="BD51" s="64" t="n">
+        <v>320</v>
+      </c>
       <c r="BE51" s="64" t="n"/>
       <c r="BF51" s="16" t="n">
         <v>15</v>
@@ -17696,7 +17734,9 @@
       <c r="BC53" s="64" t="n">
         <v>31</v>
       </c>
-      <c r="BD53" s="64" t="n"/>
+      <c r="BD53" s="64" t="n">
+        <v>550</v>
+      </c>
       <c r="BE53" s="64" t="n"/>
       <c r="BF53" s="16" t="n">
         <v>15</v>
@@ -18238,7 +18278,9 @@
       <c r="BC55" s="64" t="n">
         <v>47</v>
       </c>
-      <c r="BD55" s="64" t="n"/>
+      <c r="BD55" s="64" t="n">
+        <v>50</v>
+      </c>
       <c r="BE55" s="64" t="n"/>
       <c r="BF55" s="16" t="inlineStr">
         <is>
@@ -18515,12 +18557,14 @@
         <v>31</v>
       </c>
       <c r="BB56" s="64" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="BC56" s="64" t="n">
-        <v>47</v>
-      </c>
-      <c r="BD56" s="64" t="n"/>
+        <v>80</v>
+      </c>
+      <c r="BD56" s="64" t="n">
+        <v>120</v>
+      </c>
       <c r="BE56" s="64" t="n"/>
       <c r="BF56" s="16" t="n">
         <v>17.5</v>
@@ -18800,7 +18844,9 @@
       <c r="BC57" s="64" t="n">
         <v>78</v>
       </c>
-      <c r="BD57" s="64" t="n"/>
+      <c r="BD57" s="64" t="n">
+        <v>30</v>
+      </c>
       <c r="BE57" s="64" t="n"/>
       <c r="BF57" s="16" t="n">
         <v>18</v>
@@ -19354,12 +19400,14 @@
         <v>31</v>
       </c>
       <c r="BB59" s="64" t="n">
-        <v>31</v>
+        <v>90</v>
       </c>
       <c r="BC59" s="64" t="n">
-        <v>47</v>
-      </c>
-      <c r="BD59" s="64" t="n"/>
+        <v>90</v>
+      </c>
+      <c r="BD59" s="64" t="n">
+        <v>110</v>
+      </c>
       <c r="BE59" s="64" t="n"/>
       <c r="BF59" s="16" t="inlineStr">
         <is>
@@ -19636,12 +19684,14 @@
         <v>31</v>
       </c>
       <c r="BB60" s="64" t="n">
-        <v>31</v>
+        <v>200</v>
       </c>
       <c r="BC60" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD60" s="64" t="n"/>
+        <v>250</v>
+      </c>
+      <c r="BD60" s="64" t="n">
+        <v>330</v>
+      </c>
       <c r="BE60" s="64" t="n"/>
       <c r="BF60" s="16" t="n">
         <v>15</v>
@@ -19913,9 +19963,11 @@
         <v>10</v>
       </c>
       <c r="BA61" s="16" t="n"/>
-      <c r="BB61" s="64" t="n"/>
+      <c r="BB61" s="64" t="n">
+        <v>190</v>
+      </c>
       <c r="BC61" s="64" t="n">
-        <v>31</v>
+        <v>180</v>
       </c>
       <c r="BD61" s="64" t="n"/>
       <c r="BE61" s="64" t="n"/>
@@ -20475,7 +20527,9 @@
         <v>31</v>
       </c>
       <c r="BC63" s="64" t="n"/>
-      <c r="BD63" s="64" t="n"/>
+      <c r="BD63" s="64" t="n">
+        <v>350</v>
+      </c>
       <c r="BE63" s="64" t="n"/>
       <c r="BF63" s="16" t="n">
         <v>12.5</v>
@@ -20755,10 +20809,10 @@
         <v>31</v>
       </c>
       <c r="BB64" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BC64" s="64" t="n">
-        <v>31</v>
+        <v>140</v>
       </c>
       <c r="BD64" s="64" t="n"/>
       <c r="BE64" s="64" t="n"/>
@@ -21040,7 +21094,9 @@
         <v>31</v>
       </c>
       <c r="BC65" s="64" t="n"/>
-      <c r="BD65" s="64" t="n"/>
+      <c r="BD65" s="64" t="n">
+        <v>500</v>
+      </c>
       <c r="BE65" s="64" t="n"/>
       <c r="BF65" s="16" t="inlineStr">
         <is>
@@ -21326,13 +21382,17 @@
         <v>31</v>
       </c>
       <c r="BB66" s="64" t="n">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="BC66" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD66" s="64" t="n"/>
-      <c r="BE66" s="64" t="n"/>
+        <v>110</v>
+      </c>
+      <c r="BD66" s="64" t="n">
+        <v>80</v>
+      </c>
+      <c r="BE66" s="64" t="n">
+        <v>130</v>
+      </c>
       <c r="BF66" s="16" t="n">
         <v>15</v>
       </c>
@@ -21608,12 +21668,14 @@
       </c>
       <c r="BA67" s="16" t="n"/>
       <c r="BB67" s="64" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="BC67" s="64" t="n">
         <v>78</v>
       </c>
-      <c r="BD67" s="64" t="n"/>
+      <c r="BD67" s="64" t="n">
+        <v>140</v>
+      </c>
       <c r="BE67" s="64" t="n"/>
       <c r="BF67" s="16" t="n">
         <v>20</v>
@@ -21897,14 +21959,18 @@
       <c r="BA68" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB68" s="64" t="n"/>
+      <c r="BB68" s="64" t="n">
+        <v>220</v>
+      </c>
       <c r="BC68" s="64" t="n">
-        <v>78</v>
+        <v>210</v>
       </c>
       <c r="BD68" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BE68" s="64" t="n"/>
+        <v>570</v>
+      </c>
+      <c r="BE68" s="64" t="n">
+        <v>730</v>
+      </c>
       <c r="BF68" s="16" t="n">
         <v>15</v>
       </c>
@@ -22190,12 +22256,14 @@
         <v>31</v>
       </c>
       <c r="BB69" s="64" t="n">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="BC69" s="64" t="n">
         <v>31</v>
       </c>
-      <c r="BD69" s="64" t="n"/>
+      <c r="BD69" s="64" t="n">
+        <v>310</v>
+      </c>
       <c r="BE69" s="64" t="n"/>
       <c r="BF69" s="16" t="n">
         <v>15</v>
@@ -22462,14 +22530,14 @@
         <v>31</v>
       </c>
       <c r="BB70" s="64" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="BC70" s="64" t="n">
-        <v>47</v>
+        <v>130</v>
       </c>
       <c r="BD70" s="64" t="n"/>
       <c r="BE70" s="64" t="n">
-        <v>31</v>
+        <v>520</v>
       </c>
       <c r="BF70" s="16" t="n">
         <v>15</v>
@@ -23032,12 +23100,14 @@
         <v>31</v>
       </c>
       <c r="BB72" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BC72" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD72" s="64" t="n"/>
+        <v>140</v>
+      </c>
+      <c r="BD72" s="64" t="n">
+        <v>360</v>
+      </c>
       <c r="BE72" s="64" t="n"/>
       <c r="BF72" s="16" t="inlineStr">
         <is>
@@ -23310,9 +23380,11 @@
       <c r="BA73" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB73" s="64" t="n"/>
+      <c r="BB73" s="64" t="n">
+        <v>170</v>
+      </c>
       <c r="BC73" s="64" t="n">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="BD73" s="64" t="n"/>
       <c r="BE73" s="64" t="n"/>
@@ -23589,12 +23661,16 @@
       <c r="BA74" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB74" s="64" t="n"/>
+      <c r="BB74" s="64" t="n">
+        <v>280</v>
+      </c>
       <c r="BC74" s="64" t="n">
-        <v>31</v>
+        <v>260</v>
       </c>
       <c r="BD74" s="64" t="n"/>
-      <c r="BE74" s="64" t="n"/>
+      <c r="BE74" s="64" t="n">
+        <v>110</v>
+      </c>
       <c r="BF74" s="16" t="n">
         <v>17.5</v>
       </c>
@@ -23868,12 +23944,16 @@
       <c r="BA75" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB75" s="64" t="n"/>
+      <c r="BB75" s="64" t="n">
+        <v>110</v>
+      </c>
       <c r="BC75" s="64" t="n">
-        <v>31</v>
+        <v>100</v>
       </c>
       <c r="BD75" s="64" t="n"/>
-      <c r="BE75" s="64" t="n"/>
+      <c r="BE75" s="64" t="n">
+        <v>340</v>
+      </c>
       <c r="BF75" s="16" t="n">
         <v>15</v>
       </c>
@@ -24125,9 +24205,11 @@
       <c r="BA76" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB76" s="64" t="n"/>
+      <c r="BB76" s="64" t="n">
+        <v>180</v>
+      </c>
       <c r="BC76" s="64" t="n">
-        <v>31</v>
+        <v>160</v>
       </c>
       <c r="BD76" s="64" t="n"/>
       <c r="BE76" s="64" t="n"/>
@@ -24367,12 +24449,14 @@
       <c r="BA77" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB77" s="64" t="n"/>
+      <c r="BB77" s="64" t="n">
+        <v>670</v>
+      </c>
       <c r="BC77" s="64" t="n">
-        <v>31</v>
+        <v>730</v>
       </c>
       <c r="BD77" s="64" t="n">
-        <v>78</v>
+        <v>510</v>
       </c>
       <c r="BE77" s="64" t="n"/>
       <c r="BF77" s="16" t="n">
@@ -24658,11 +24742,13 @@
         <v>78</v>
       </c>
       <c r="BC78" s="64" t="n">
-        <v>109</v>
-      </c>
-      <c r="BD78" s="64" t="n"/>
+        <v>70</v>
+      </c>
+      <c r="BD78" s="64" t="n">
+        <v>290</v>
+      </c>
       <c r="BE78" s="64" t="n">
-        <v>31</v>
+        <v>320</v>
       </c>
       <c r="BF78" s="16" t="n">
         <v>18</v>
@@ -25236,7 +25322,7 @@
       <c r="BB80" s="64" t="n"/>
       <c r="BC80" s="64" t="n"/>
       <c r="BD80" s="64" t="n">
-        <v>47</v>
+        <v>220</v>
       </c>
       <c r="BE80" s="64" t="n"/>
       <c r="BF80" s="16" t="n">
@@ -26074,13 +26160,17 @@
         <v>31</v>
       </c>
       <c r="BB83" s="64" t="n">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="BC83" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD83" s="64" t="n"/>
-      <c r="BE83" s="64" t="n"/>
+        <v>110</v>
+      </c>
+      <c r="BD83" s="64" t="n">
+        <v>80</v>
+      </c>
+      <c r="BE83" s="64" t="n">
+        <v>130</v>
+      </c>
       <c r="BF83" s="16" t="inlineStr">
         <is>
           <t>20-15</t>
@@ -26359,7 +26449,9 @@
         <v>47</v>
       </c>
       <c r="BC84" s="64" t="n"/>
-      <c r="BD84" s="64" t="n"/>
+      <c r="BD84" s="64" t="n">
+        <v>40</v>
+      </c>
       <c r="BE84" s="64" t="n"/>
       <c r="BF84" s="16" t="n">
         <v>15</v>
@@ -26924,7 +27016,7 @@
       <c r="BB86" s="64" t="n"/>
       <c r="BC86" s="64" t="n"/>
       <c r="BD86" s="64" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="BE86" s="64" t="n"/>
       <c r="BF86" s="16" t="n">
@@ -27203,13 +27295,17 @@
         <v>31</v>
       </c>
       <c r="BB87" s="64" t="n">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="BC87" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD87" s="64" t="n"/>
-      <c r="BE87" s="64" t="n"/>
+        <v>110</v>
+      </c>
+      <c r="BD87" s="64" t="n">
+        <v>80</v>
+      </c>
+      <c r="BE87" s="64" t="n">
+        <v>130</v>
+      </c>
       <c r="BF87" s="16" t="inlineStr">
         <is>
           <t>20-15</t>
@@ -27748,13 +27844,15 @@
       <c r="BA89" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB89" s="64" t="n"/>
+      <c r="BB89" s="64" t="n">
+        <v>160</v>
+      </c>
       <c r="BC89" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BD89" s="64" t="n"/>
       <c r="BE89" s="64" t="n">
-        <v>31</v>
+        <v>410</v>
       </c>
       <c r="BF89" s="16" t="n">
         <v>15</v>
@@ -28331,9 +28429,11 @@
       <c r="BA91" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB91" s="64" t="n"/>
+      <c r="BB91" s="64" t="n">
+        <v>170</v>
+      </c>
       <c r="BC91" s="64" t="n">
-        <v>31</v>
+        <v>130</v>
       </c>
       <c r="BD91" s="64" t="n">
         <v>31</v>
@@ -28609,12 +28709,14 @@
       <c r="BA92" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB92" s="64" t="n"/>
+      <c r="BB92" s="64" t="n">
+        <v>10</v>
+      </c>
       <c r="BC92" s="64" t="n">
         <v>47</v>
       </c>
       <c r="BD92" s="64" t="n">
-        <v>31</v>
+        <v>190</v>
       </c>
       <c r="BE92" s="64" t="n">
         <v>31</v>
@@ -28910,7 +29012,9 @@
       <c r="BC93" s="64" t="n">
         <v>78</v>
       </c>
-      <c r="BD93" s="64" t="n"/>
+      <c r="BD93" s="64" t="n">
+        <v>10</v>
+      </c>
       <c r="BE93" s="64" t="n"/>
       <c r="BF93" s="16" t="n">
         <v>20</v>
@@ -29180,12 +29284,14 @@
       <c r="BA94" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB94" s="64" t="n"/>
+      <c r="BB94" s="64" t="n">
+        <v>130</v>
+      </c>
       <c r="BC94" s="64" t="n">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="BD94" s="64" t="n">
-        <v>31</v>
+        <v>310</v>
       </c>
       <c r="BE94" s="64" t="n">
         <v>31</v>
@@ -29463,12 +29569,14 @@
       <c r="BA95" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB95" s="64" t="n"/>
+      <c r="BB95" s="64" t="n">
+        <v>30</v>
+      </c>
       <c r="BC95" s="64" t="n">
         <v>47</v>
       </c>
       <c r="BD95" s="64" t="n">
-        <v>31</v>
+        <v>210</v>
       </c>
       <c r="BE95" s="64" t="n">
         <v>31</v>
@@ -29746,12 +29854,14 @@
       <c r="BA96" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB96" s="64" t="n"/>
+      <c r="BB96" s="64" t="n">
+        <v>120</v>
+      </c>
       <c r="BC96" s="64" t="n">
-        <v>31</v>
+        <v>90</v>
       </c>
       <c r="BD96" s="64" t="n">
-        <v>47</v>
+        <v>200</v>
       </c>
       <c r="BE96" s="64" t="n"/>
       <c r="BF96" s="16" t="n">
@@ -30026,7 +30136,9 @@
       <c r="BC97" s="79" t="n">
         <v>31</v>
       </c>
-      <c r="BD97" s="64" t="n"/>
+      <c r="BD97" s="64" t="n">
+        <v>290</v>
+      </c>
       <c r="BE97" s="79" t="n"/>
       <c r="BF97" s="16" t="n">
         <v>17.5</v>
@@ -30298,9 +30410,11 @@
       <c r="BA98" s="16" t="n"/>
       <c r="BB98" s="64" t="n"/>
       <c r="BC98" s="64" t="n"/>
-      <c r="BD98" s="64" t="n"/>
+      <c r="BD98" s="64" t="n">
+        <v>100</v>
+      </c>
       <c r="BE98" s="64" t="n">
-        <v>156</v>
+        <v>60</v>
       </c>
       <c r="BF98" s="16" t="n">
         <v>17.5</v>
@@ -31126,9 +31240,11 @@
       <c r="BA101" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB101" s="64" t="n"/>
+      <c r="BB101" s="64" t="n">
+        <v>180</v>
+      </c>
       <c r="BC101" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BD101" s="64" t="n"/>
       <c r="BE101" s="64" t="n"/>
@@ -31952,7 +32068,7 @@
         <v>31</v>
       </c>
       <c r="BB104" s="64" t="n">
-        <v>78</v>
+        <v>20</v>
       </c>
       <c r="BC104" s="64" t="n">
         <v>31</v>
@@ -32770,7 +32886,9 @@
       <c r="BC107" s="79" t="n">
         <v>31</v>
       </c>
-      <c r="BD107" s="64" t="n"/>
+      <c r="BD107" s="64" t="n">
+        <v>290</v>
+      </c>
       <c r="BE107" s="79" t="n"/>
       <c r="BF107" s="16" t="n">
         <v>15</v>
@@ -33306,7 +33424,7 @@
         <v>78</v>
       </c>
       <c r="BD109" s="64" t="n">
-        <v>31</v>
+        <v>250</v>
       </c>
       <c r="BE109" s="64" t="n">
         <v>31</v>
@@ -33847,9 +33965,11 @@
       <c r="BA111" s="16" t="n"/>
       <c r="BB111" s="64" t="n"/>
       <c r="BC111" s="64" t="n"/>
-      <c r="BD111" s="64" t="n"/>
+      <c r="BD111" s="64" t="n">
+        <v>100</v>
+      </c>
       <c r="BE111" s="64" t="n">
-        <v>156</v>
+        <v>60</v>
       </c>
       <c r="BF111" s="16" t="n">
         <v>15</v>
@@ -34400,7 +34520,9 @@
       <c r="BC113" s="64" t="n">
         <v>78</v>
       </c>
-      <c r="BD113" s="64" t="n"/>
+      <c r="BD113" s="64" t="n">
+        <v>10</v>
+      </c>
       <c r="BE113" s="64" t="n"/>
       <c r="BF113" s="16" t="inlineStr">
         <is>
@@ -34677,12 +34799,14 @@
         <v>31</v>
       </c>
       <c r="BB114" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BC114" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD114" s="64" t="n"/>
+        <v>140</v>
+      </c>
+      <c r="BD114" s="64" t="n">
+        <v>360</v>
+      </c>
       <c r="BE114" s="64" t="n"/>
       <c r="BF114" s="16" t="n">
         <v>17.5</v>
@@ -34958,12 +35082,14 @@
         <v>31</v>
       </c>
       <c r="BB115" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BC115" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD115" s="64" t="n"/>
+        <v>140</v>
+      </c>
+      <c r="BD115" s="64" t="n">
+        <v>360</v>
+      </c>
       <c r="BE115" s="64" t="n"/>
       <c r="BF115" s="16" t="n">
         <v>17.5</v>
@@ -35239,12 +35365,14 @@
         <v>31</v>
       </c>
       <c r="BB116" s="64" t="n">
-        <v>31</v>
+        <v>170</v>
       </c>
       <c r="BC116" s="64" t="n">
-        <v>31</v>
-      </c>
-      <c r="BD116" s="64" t="n"/>
+        <v>140</v>
+      </c>
+      <c r="BD116" s="64" t="n">
+        <v>360</v>
+      </c>
       <c r="BE116" s="64" t="n"/>
       <c r="BF116" s="16" t="n">
         <v>17.5</v>
@@ -35513,7 +35641,9 @@
       </c>
       <c r="BB117" s="64" t="n"/>
       <c r="BC117" s="64" t="n"/>
-      <c r="BD117" s="64" t="n"/>
+      <c r="BD117" s="64" t="n">
+        <v>750</v>
+      </c>
       <c r="BE117" s="64" t="n">
         <v>47</v>
       </c>
@@ -35790,7 +35920,9 @@
       <c r="BA118" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB118" s="64" t="n"/>
+      <c r="BB118" s="64" t="n">
+        <v>90</v>
+      </c>
       <c r="BC118" s="64" t="n">
         <v>31</v>
       </c>
@@ -36341,13 +36473,15 @@
         <v>31</v>
       </c>
       <c r="BB120" s="79" t="n">
-        <v>47</v>
+        <v>270</v>
       </c>
       <c r="BC120" s="79" t="n">
-        <v>31</v>
+        <v>390</v>
       </c>
       <c r="BD120" s="111" t="n"/>
-      <c r="BE120" s="111" t="n"/>
+      <c r="BE120" s="111" t="n">
+        <v>590</v>
+      </c>
       <c r="BF120" s="77" t="inlineStr">
         <is>
           <t>22-16</t>
@@ -36618,12 +36752,14 @@
       <c r="BA121" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB121" s="79" t="n"/>
+      <c r="BB121" s="79" t="n">
+        <v>310</v>
+      </c>
       <c r="BC121" s="79" t="n">
-        <v>47</v>
+        <v>330</v>
       </c>
       <c r="BD121" s="79" t="n">
-        <v>109</v>
+        <v>230</v>
       </c>
       <c r="BE121" s="79" t="n">
         <v>47</v>
@@ -37164,15 +37300,17 @@
       <c r="BA123" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB123" s="64" t="n"/>
+      <c r="BB123" s="64" t="n">
+        <v>720</v>
+      </c>
       <c r="BC123" s="64" t="n">
-        <v>31</v>
+        <v>760</v>
       </c>
       <c r="BD123" s="64" t="n">
-        <v>109</v>
+        <v>770</v>
       </c>
       <c r="BE123" s="79" t="n">
-        <v>47</v>
+        <v>800</v>
       </c>
       <c r="BF123" s="16" t="inlineStr">
         <is>
@@ -37451,7 +37589,7 @@
       <c r="BB124" s="16" t="n"/>
       <c r="BC124" s="77" t="n"/>
       <c r="BD124" s="112" t="n">
-        <v>47</v>
+        <v>220</v>
       </c>
       <c r="BE124" s="77" t="n"/>
       <c r="BF124" s="16" t="inlineStr">
@@ -37724,14 +37862,18 @@
       <c r="BA125" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB125" s="79" t="n"/>
+      <c r="BB125" s="79" t="n">
+        <v>150</v>
+      </c>
       <c r="BC125" s="79" t="n">
-        <v>31</v>
+        <v>140</v>
       </c>
       <c r="BD125" s="79" t="n">
-        <v>78</v>
-      </c>
-      <c r="BE125" s="79" t="n"/>
+        <v>70</v>
+      </c>
+      <c r="BE125" s="79" t="n">
+        <v>260</v>
+      </c>
       <c r="BF125" s="77" t="n">
         <v>23</v>
       </c>
@@ -38000,7 +38142,9 @@
       <c r="BA126" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB126" s="79" t="n"/>
+      <c r="BB126" s="79" t="n">
+        <v>420</v>
+      </c>
       <c r="BC126" s="79" t="n">
         <v>31</v>
       </c>
@@ -38286,7 +38430,9 @@
       <c r="BA127" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB127" s="64" t="n"/>
+      <c r="BB127" s="64" t="n">
+        <v>420</v>
+      </c>
       <c r="BC127" s="79" t="n">
         <v>31</v>
       </c>
@@ -38563,9 +38709,11 @@
       <c r="BB128" s="77" t="n"/>
       <c r="BC128" s="77" t="n"/>
       <c r="BD128" s="79" t="n">
-        <v>31</v>
-      </c>
-      <c r="BE128" s="79" t="n"/>
+        <v>470</v>
+      </c>
+      <c r="BE128" s="79" t="n">
+        <v>1080</v>
+      </c>
       <c r="BF128" s="77" t="n">
         <v>15</v>
       </c>
@@ -38851,7 +38999,7 @@
       <c r="BB129" s="79" t="n"/>
       <c r="BC129" s="79" t="n"/>
       <c r="BD129" s="79" t="n">
-        <v>156</v>
+        <v>80</v>
       </c>
       <c r="BE129" s="79" t="n">
         <v>47</v>
@@ -39131,10 +39279,10 @@
       <c r="BB130" s="16" t="n"/>
       <c r="BC130" s="77" t="n"/>
       <c r="BD130" s="64" t="n">
-        <v>78</v>
+        <v>400</v>
       </c>
       <c r="BE130" s="79" t="n">
-        <v>31</v>
+        <v>720</v>
       </c>
       <c r="BF130" s="16" t="inlineStr">
         <is>
@@ -39954,11 +40102,15 @@
       <c r="BA133" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB133" s="64" t="n"/>
+      <c r="BB133" s="64" t="n">
+        <v>290</v>
+      </c>
       <c r="BC133" s="79" t="n">
         <v>31</v>
       </c>
-      <c r="BD133" s="64" t="n"/>
+      <c r="BD133" s="64" t="n">
+        <v>340</v>
+      </c>
       <c r="BE133" s="79" t="n">
         <v>47</v>
       </c>
@@ -40801,7 +40953,7 @@
         <v>31</v>
       </c>
       <c r="BD136" s="64" t="n">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="BE136" s="79" t="n">
         <v>109</v>
@@ -41079,10 +41231,10 @@
       <c r="BB137" s="64" t="n"/>
       <c r="BC137" s="64" t="n"/>
       <c r="BD137" s="112" t="n">
-        <v>78</v>
+        <v>430</v>
       </c>
       <c r="BE137" s="111" t="n">
-        <v>31</v>
+        <v>510</v>
       </c>
       <c r="BF137" s="16" t="inlineStr">
         <is>
@@ -41919,10 +42071,10 @@
       <c r="BB140" s="77" t="n"/>
       <c r="BC140" s="79" t="n"/>
       <c r="BD140" s="79" t="n">
-        <v>31</v>
+        <v>450</v>
       </c>
       <c r="BE140" s="79" t="n">
-        <v>31</v>
+        <v>720</v>
       </c>
       <c r="BF140" s="77" t="inlineStr">
         <is>
@@ -42199,10 +42351,10 @@
       <c r="BB141" s="16" t="n"/>
       <c r="BC141" s="77" t="n"/>
       <c r="BD141" s="112" t="n">
-        <v>234</v>
+        <v>420</v>
       </c>
       <c r="BE141" s="111" t="n">
-        <v>47</v>
+        <v>640</v>
       </c>
       <c r="BF141" s="77" t="inlineStr">
         <is>
@@ -43295,16 +43447,16 @@
         <v>31</v>
       </c>
       <c r="BB145" s="79" t="n">
-        <v>78</v>
+        <v>300</v>
       </c>
       <c r="BC145" s="79" t="n">
-        <v>78</v>
+        <v>360</v>
       </c>
       <c r="BD145" s="79" t="n">
-        <v>31</v>
+        <v>270</v>
       </c>
       <c r="BE145" s="79" t="n">
-        <v>31</v>
+        <v>320</v>
       </c>
       <c r="BF145" s="16" t="inlineStr">
         <is>
@@ -43580,7 +43732,9 @@
       <c r="BA146" s="16" t="n"/>
       <c r="BB146" s="16" t="n"/>
       <c r="BC146" s="77" t="n"/>
-      <c r="BD146" s="16" t="n"/>
+      <c r="BD146" s="16" t="n">
+        <v>670</v>
+      </c>
       <c r="BE146" s="79" t="n">
         <v>31</v>
       </c>
@@ -43859,15 +44013,17 @@
       </c>
       <c r="BA147" s="77" t="n"/>
       <c r="BB147" s="64" t="n">
-        <v>234</v>
+        <v>320</v>
       </c>
       <c r="BC147" s="64" t="n">
-        <v>31</v>
+        <v>340</v>
       </c>
       <c r="BD147" s="79" t="n">
-        <v>78</v>
-      </c>
-      <c r="BE147" s="79" t="n"/>
+        <v>300</v>
+      </c>
+      <c r="BE147" s="79" t="n">
+        <v>530</v>
+      </c>
       <c r="BF147" s="16" t="n">
         <v>23</v>
       </c>
@@ -44145,10 +44301,10 @@
       <c r="BB148" s="16" t="n"/>
       <c r="BC148" s="16" t="n"/>
       <c r="BD148" s="79" t="n">
-        <v>31</v>
+        <v>400</v>
       </c>
       <c r="BE148" s="79" t="n">
-        <v>31</v>
+        <v>640</v>
       </c>
       <c r="BF148" s="16" t="inlineStr">
         <is>
@@ -44425,10 +44581,10 @@
       <c r="BB149" s="64" t="n"/>
       <c r="BC149" s="79" t="n"/>
       <c r="BD149" s="64" t="n">
-        <v>234</v>
+        <v>340</v>
       </c>
       <c r="BE149" s="79" t="n">
-        <v>109</v>
+        <v>350</v>
       </c>
       <c r="BF149" s="16" t="inlineStr">
         <is>
@@ -44700,13 +44856,17 @@
       <c r="BA150" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB150" s="79" t="n"/>
+      <c r="BB150" s="79" t="n">
+        <v>110</v>
+      </c>
       <c r="BC150" s="79" t="n">
-        <v>47</v>
-      </c>
-      <c r="BD150" s="79" t="n"/>
+        <v>90</v>
+      </c>
+      <c r="BD150" s="79" t="n">
+        <v>100</v>
+      </c>
       <c r="BE150" s="79" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="BF150" s="77" t="inlineStr">
         <is>
@@ -44979,13 +45139,15 @@
         <v>31</v>
       </c>
       <c r="BB151" s="79" t="n">
-        <v>47</v>
+        <v>270</v>
       </c>
       <c r="BC151" s="79" t="n">
-        <v>31</v>
+        <v>390</v>
       </c>
       <c r="BD151" s="111" t="n"/>
-      <c r="BE151" s="111" t="n"/>
+      <c r="BE151" s="111" t="n">
+        <v>590</v>
+      </c>
       <c r="BF151" s="77" t="inlineStr">
         <is>
           <t>22-16</t>
@@ -45542,7 +45704,9 @@
       <c r="BA153" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB153" s="79" t="n"/>
+      <c r="BB153" s="79" t="n">
+        <v>280</v>
+      </c>
       <c r="BC153" s="79" t="n">
         <v>47</v>
       </c>
@@ -46088,14 +46252,18 @@
       <c r="BA155" s="77" t="n">
         <v>31</v>
       </c>
-      <c r="BB155" s="79" t="n"/>
+      <c r="BB155" s="79" t="n">
+        <v>170</v>
+      </c>
       <c r="BC155" s="79" t="n">
-        <v>47</v>
+        <v>160</v>
       </c>
       <c r="BD155" s="79" t="n">
-        <v>47</v>
-      </c>
-      <c r="BE155" s="79" t="n"/>
+        <v>80</v>
+      </c>
+      <c r="BE155" s="79" t="n">
+        <v>290</v>
+      </c>
       <c r="BF155" s="77" t="n">
         <v>23</v>
       </c>
@@ -46368,15 +46536,17 @@
       <c r="BA156" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="BB156" s="64" t="n"/>
+      <c r="BB156" s="64" t="n">
+        <v>720</v>
+      </c>
       <c r="BC156" s="64" t="n">
-        <v>31</v>
+        <v>760</v>
       </c>
       <c r="BD156" s="64" t="n">
-        <v>78</v>
+        <v>770</v>
       </c>
       <c r="BE156" s="79" t="n">
-        <v>47</v>
+        <v>930</v>
       </c>
       <c r="BF156" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rewrite durability/steerability scoring to use cutlet-derived metrics
Replace proxy-based scoring (cutter counts, average backrake, spacing CV)
with direct cutlet geometry measurements from the cutlet engine:

Durability (7 components): load uniformity (Gini coefficient), working
cutter count, work-per-cutter, blade balance (CV), backup engagement
fraction, backrake, and cutter size.

Steerability (7 components): gauge openness (area fraction), gauge
aggressiveness, cone aggressiveness, blade factor, profile depth,
siderake, and low cutter count.

All components are rank-normalized across the 130-bit population and
weighted to produce 0-9 scores. Updated Bit Applications Tool r2.xlsx
columns AO & AP with new scores.

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Bit Applications Tool r2.xlsx
+++ b/Bit Applications Tool r2.xlsx
@@ -4401,10 +4401,10 @@
         </is>
       </c>
       <c r="AO5" s="47" t="n">
-        <v>5.6</v>
+        <v>3.6</v>
       </c>
       <c r="AP5" s="48" t="n">
-        <v>4.8</v>
+        <v>1.3</v>
       </c>
       <c r="AQ5" s="163" t="n">
         <v>0</v>
@@ -4935,10 +4935,10 @@
         </is>
       </c>
       <c r="AO7" s="74" t="n">
-        <v>5.3</v>
+        <v>4.7</v>
       </c>
       <c r="AP7" s="75" t="n">
-        <v>3</v>
+        <v>4.1</v>
       </c>
       <c r="AQ7" s="168" t="n">
         <v>0.1</v>
@@ -5993,10 +5993,10 @@
         </is>
       </c>
       <c r="AO11" s="47" t="n">
-        <v>3.1</v>
+        <v>5.5</v>
       </c>
       <c r="AP11" s="48" t="n">
-        <v>5.5</v>
+        <v>1.3</v>
       </c>
       <c r="AQ11" s="167" t="n">
         <v>0.02</v>
@@ -6263,10 +6263,10 @@
         </is>
       </c>
       <c r="AO12" s="47" t="n">
-        <v>5.3</v>
+        <v>3.8</v>
       </c>
       <c r="AP12" s="48" t="n">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="AQ12" s="163" t="n">
         <v>0</v>
@@ -6805,10 +6805,10 @@
         </is>
       </c>
       <c r="AO14" s="47" t="n">
-        <v>6.3</v>
+        <v>4.1</v>
       </c>
       <c r="AP14" s="48" t="n">
-        <v>3.8</v>
+        <v>2.7</v>
       </c>
       <c r="AQ14" s="163" t="n">
         <v>0</v>
@@ -8671,10 +8671,10 @@
         </is>
       </c>
       <c r="AO21" s="47" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
       <c r="AP21" s="48" t="n">
-        <v>2.6</v>
+        <v>1.7</v>
       </c>
       <c r="AQ21" s="163" t="n">
         <v>0</v>
@@ -9739,10 +9739,10 @@
         </is>
       </c>
       <c r="AO25" s="47" t="n">
-        <v>2.9</v>
+        <v>6.1</v>
       </c>
       <c r="AP25" s="48" t="n">
-        <v>5.1</v>
+        <v>4.5</v>
       </c>
       <c r="AQ25" s="163" t="n">
         <v>0</v>
@@ -10555,10 +10555,10 @@
         </is>
       </c>
       <c r="AO28" s="47" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="AP28" s="48" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ28" s="163" t="n">
         <v>0</v>
@@ -10837,10 +10837,10 @@
         </is>
       </c>
       <c r="AO29" s="47" t="n">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="AP29" s="48" t="n">
-        <v>3.4</v>
+        <v>4.1</v>
       </c>
       <c r="AQ29" s="163" t="n">
         <v>0</v>
@@ -11117,10 +11117,10 @@
         </is>
       </c>
       <c r="AO30" s="47" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="AP30" s="48" t="n">
-        <v>3.9</v>
+        <v>2.6</v>
       </c>
       <c r="AQ30" s="163" t="n">
         <v>0</v>
@@ -11425,10 +11425,10 @@
         </is>
       </c>
       <c r="AO31" s="46" t="n">
-        <v>5</v>
+        <v>6.3</v>
       </c>
       <c r="AP31" s="48" t="n">
-        <v>3.6</v>
+        <v>1</v>
       </c>
       <c r="AQ31" s="163" t="n">
         <v>0</v>
@@ -11727,10 +11727,10 @@
         </is>
       </c>
       <c r="AO32" s="46" t="n">
-        <v>4.9</v>
+        <v>7.9</v>
       </c>
       <c r="AP32" s="48" t="n">
-        <v>3.9</v>
+        <v>0</v>
       </c>
       <c r="AQ32" s="163" t="n">
         <v>0</v>
@@ -12007,10 +12007,10 @@
         </is>
       </c>
       <c r="AO33" s="47" t="n">
-        <v>7.4</v>
+        <v>8.1</v>
       </c>
       <c r="AP33" s="48" t="n">
-        <v>4</v>
+        <v>1.6</v>
       </c>
       <c r="AQ33" s="163" t="n">
         <v>0</v>
@@ -12289,10 +12289,10 @@
         </is>
       </c>
       <c r="AO34" s="47" t="n">
-        <v>7.2</v>
+        <v>8.1</v>
       </c>
       <c r="AP34" s="48" t="n">
-        <v>4.1</v>
+        <v>1.3</v>
       </c>
       <c r="AQ34" s="163" t="n">
         <v>0</v>
@@ -12571,10 +12571,10 @@
         </is>
       </c>
       <c r="AO35" s="47" t="n">
-        <v>3.3</v>
+        <v>4.6</v>
       </c>
       <c r="AP35" s="48" t="n">
-        <v>2.7</v>
+        <v>5.1</v>
       </c>
       <c r="AQ35" s="163" t="n">
         <v>0</v>
@@ -12857,10 +12857,10 @@
         </is>
       </c>
       <c r="AO36" s="46" t="n">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
       <c r="AP36" s="48" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="AQ36" s="163" t="n">
         <v>0</v>
@@ -13135,10 +13135,10 @@
         </is>
       </c>
       <c r="AO37" s="47" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="AP37" s="48" t="n">
-        <v>4.2</v>
+        <v>2.6</v>
       </c>
       <c r="AQ37" s="163" t="n">
         <v>0</v>
@@ -13437,10 +13437,10 @@
         </is>
       </c>
       <c r="AO38" s="46" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="AP38" s="48" t="n">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="AQ38" s="163" t="n">
         <v>0</v>
@@ -13975,10 +13975,10 @@
         </is>
       </c>
       <c r="AO40" s="47" t="n">
-        <v>7.1</v>
+        <v>5.2</v>
       </c>
       <c r="AP40" s="48" t="n">
-        <v>3.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ40" s="163" t="n">
         <v>0</v>
@@ -14271,10 +14271,10 @@
         </is>
       </c>
       <c r="AO41" s="46" t="n">
-        <v>4.2</v>
+        <v>6.4</v>
       </c>
       <c r="AP41" s="48" t="n">
-        <v>5.9</v>
+        <v>0.6</v>
       </c>
       <c r="AQ41" s="163" t="n">
         <v>0</v>
@@ -14551,10 +14551,10 @@
         </is>
       </c>
       <c r="AO42" s="47" t="n">
-        <v>6.2</v>
+        <v>3.7</v>
       </c>
       <c r="AP42" s="48" t="n">
-        <v>4.5</v>
+        <v>1.4</v>
       </c>
       <c r="AQ42" s="163" t="n">
         <v>0</v>
@@ -14851,10 +14851,10 @@
         </is>
       </c>
       <c r="AO43" s="46" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="AP43" s="48" t="n">
-        <v>3.7</v>
+        <v>4.2</v>
       </c>
       <c r="AQ43" s="163" t="n">
         <v>0</v>
@@ -15133,10 +15133,10 @@
         </is>
       </c>
       <c r="AO44" s="47" t="n">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="AP44" s="48" t="n">
-        <v>1.5</v>
+        <v>3.2</v>
       </c>
       <c r="AQ44" s="163" t="n">
         <v>0</v>
@@ -15411,10 +15411,10 @@
         </is>
       </c>
       <c r="AO45" s="47" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="AP45" s="48" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="AQ45" s="163" t="n">
         <v>0</v>
@@ -15689,10 +15689,10 @@
         </is>
       </c>
       <c r="AO46" s="47" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="AP46" s="48" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="AQ46" s="163" t="n">
         <v>0</v>
@@ -15967,10 +15967,10 @@
         </is>
       </c>
       <c r="AO47" s="47" t="n">
-        <v>7.1</v>
+        <v>5.9</v>
       </c>
       <c r="AP47" s="48" t="n">
-        <v>4.4</v>
+        <v>3.3</v>
       </c>
       <c r="AQ47" s="163" t="n">
         <v>0</v>
@@ -16255,10 +16255,10 @@
         </is>
       </c>
       <c r="AO48" s="47" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="AP48" s="48" t="n">
-        <v>5.3</v>
+        <v>4.1</v>
       </c>
       <c r="AQ48" s="163" t="n">
         <v>0</v>
@@ -16549,10 +16549,10 @@
         </is>
       </c>
       <c r="AO49" s="46" t="n">
-        <v>3.3</v>
+        <v>5</v>
       </c>
       <c r="AP49" s="48" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="AQ49" s="163" t="n">
         <v>0</v>
@@ -16829,10 +16829,10 @@
         </is>
       </c>
       <c r="AO50" s="47" t="n">
-        <v>5.1</v>
+        <v>3.5</v>
       </c>
       <c r="AP50" s="48" t="n">
-        <v>5.4</v>
+        <v>2.3</v>
       </c>
       <c r="AQ50" s="163" t="n">
         <v>0</v>
@@ -17131,10 +17131,10 @@
         </is>
       </c>
       <c r="AO51" s="46" t="n">
-        <v>5.5</v>
+        <v>5.3</v>
       </c>
       <c r="AP51" s="48" t="n">
-        <v>4.6</v>
+        <v>4.1</v>
       </c>
       <c r="AQ51" s="163" t="n">
         <v>0</v>
@@ -17415,10 +17415,10 @@
         </is>
       </c>
       <c r="AO52" s="47" t="n">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
       <c r="AP52" s="48" t="n">
-        <v>4.6</v>
+        <v>2.7</v>
       </c>
       <c r="AQ52" s="163" t="n">
         <v>0</v>
@@ -17686,10 +17686,10 @@
         </is>
       </c>
       <c r="AO53" s="47" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="AP53" s="48" t="n">
-        <v>3.9</v>
+        <v>3.3</v>
       </c>
       <c r="AQ53" s="163" t="n">
         <v>0</v>
@@ -17962,10 +17962,10 @@
         </is>
       </c>
       <c r="AO54" s="47" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="AP54" s="48" t="n">
-        <v>5.4</v>
+        <v>4.8</v>
       </c>
       <c r="AQ54" s="163" t="n">
         <v>0</v>
@@ -18228,10 +18228,10 @@
         </is>
       </c>
       <c r="AO55" s="47" t="n">
-        <v>3.5</v>
+        <v>3.1</v>
       </c>
       <c r="AP55" s="48" t="n">
-        <v>8.800000000000001</v>
+        <v>1.6</v>
       </c>
       <c r="AQ55" s="163" t="n">
         <v>0</v>
@@ -18512,10 +18512,10 @@
         </is>
       </c>
       <c r="AO56" s="47" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="AP56" s="48" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="AQ56" s="163" t="n">
         <v>0</v>
@@ -18794,10 +18794,10 @@
         </is>
       </c>
       <c r="AO57" s="47" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="AP57" s="48" t="n">
-        <v>7.9</v>
+        <v>2.1</v>
       </c>
       <c r="AQ57" s="163" t="n">
         <v>0</v>
@@ -19076,10 +19076,10 @@
         </is>
       </c>
       <c r="AO58" s="47" t="n">
-        <v>4.1</v>
+        <v>5</v>
       </c>
       <c r="AP58" s="48" t="n">
-        <v>4.2</v>
+        <v>1.9</v>
       </c>
       <c r="AQ58" s="163" t="n">
         <v>0</v>
@@ -19355,10 +19355,10 @@
         </is>
       </c>
       <c r="AO59" s="47" t="n">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="AP59" s="48" t="n">
-        <v>3.1</v>
+        <v>1.2</v>
       </c>
       <c r="AQ59" s="163" t="n">
         <v>0</v>
@@ -19639,10 +19639,10 @@
         </is>
       </c>
       <c r="AO60" s="47" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="AP60" s="48" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="AQ60" s="163" t="n">
         <v>0</v>
@@ -19921,10 +19921,10 @@
         </is>
       </c>
       <c r="AO61" s="47" t="n">
-        <v>3.4</v>
+        <v>4.4</v>
       </c>
       <c r="AP61" s="48" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="AQ61" s="163" t="n">
         <v>0</v>
@@ -20203,10 +20203,10 @@
         </is>
       </c>
       <c r="AO62" s="47" t="n">
-        <v>6.2</v>
+        <v>5.5</v>
       </c>
       <c r="AP62" s="48" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="AQ62" s="163" t="n">
         <v>0</v>
@@ -20481,10 +20481,10 @@
         </is>
       </c>
       <c r="AO63" s="47" t="n">
-        <v>2.9</v>
+        <v>5</v>
       </c>
       <c r="AP63" s="48" t="n">
-        <v>6.3</v>
+        <v>4.1</v>
       </c>
       <c r="AQ63" s="163" t="n">
         <v>0</v>
@@ -20764,10 +20764,10 @@
         </is>
       </c>
       <c r="AO64" s="47" t="n">
-        <v>5.6</v>
+        <v>4.1</v>
       </c>
       <c r="AP64" s="48" t="n">
-        <v>4.5</v>
+        <v>2.7</v>
       </c>
       <c r="AQ64" s="163" t="n">
         <v>0</v>
@@ -21044,10 +21044,10 @@
         </is>
       </c>
       <c r="AO65" s="47" t="n">
-        <v>4.3</v>
+        <v>0.6</v>
       </c>
       <c r="AP65" s="48" t="n">
-        <v>6.2</v>
+        <v>2.6</v>
       </c>
       <c r="AQ65" s="163" t="n">
         <v>0.083</v>
@@ -21335,10 +21335,10 @@
         </is>
       </c>
       <c r="AO66" s="47" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="AP66" s="48" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ66" s="163" t="n">
         <v>0</v>
@@ -21625,10 +21625,10 @@
         </is>
       </c>
       <c r="AO67" s="47" t="n">
-        <v>6.4</v>
+        <v>5.8</v>
       </c>
       <c r="AP67" s="48" t="n">
-        <v>2.5</v>
+        <v>1.7</v>
       </c>
       <c r="AQ67" s="163" t="n">
         <v>0</v>
@@ -21913,10 +21913,10 @@
         </is>
       </c>
       <c r="AO68" s="47" t="n">
-        <v>6.3</v>
+        <v>3.9</v>
       </c>
       <c r="AP68" s="48" t="n">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="AQ68" s="163" t="n">
         <v>0</v>
@@ -22211,10 +22211,10 @@
         </is>
       </c>
       <c r="AO69" s="47" t="n">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="AP69" s="48" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="AQ69" s="163" t="n">
         <v>0</v>
@@ -22485,10 +22485,10 @@
         </is>
       </c>
       <c r="AO70" s="47" t="n">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
       <c r="AP70" s="48" t="n">
-        <v>4.7</v>
+        <v>2.4</v>
       </c>
       <c r="AQ70" s="163" t="n">
         <v>0</v>
@@ -22777,10 +22777,10 @@
         </is>
       </c>
       <c r="AO71" s="47" t="n">
-        <v>5.8</v>
+        <v>3.7</v>
       </c>
       <c r="AP71" s="48" t="n">
-        <v>2.6</v>
+        <v>0.6</v>
       </c>
       <c r="AQ71" s="163" t="n">
         <v>0</v>
@@ -23055,10 +23055,10 @@
         </is>
       </c>
       <c r="AO72" s="47" t="n">
-        <v>6.6</v>
+        <v>3.3</v>
       </c>
       <c r="AP72" s="48" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="AQ72" s="163" t="n">
         <v>0</v>
@@ -23336,10 +23336,10 @@
         </is>
       </c>
       <c r="AO73" s="47" t="n">
-        <v>6.3</v>
+        <v>5.4</v>
       </c>
       <c r="AP73" s="48" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="AQ73" s="163" t="n">
         <v>0</v>
@@ -23617,10 +23617,10 @@
         </is>
       </c>
       <c r="AO74" s="47" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="AP74" s="48" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="AQ74" s="163" t="n">
         <v>0</v>
@@ -23900,10 +23900,10 @@
         </is>
       </c>
       <c r="AO75" s="47" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="AP75" s="48" t="n">
-        <v>6.8</v>
+        <v>4.8</v>
       </c>
       <c r="AQ75" s="163" t="n">
         <v>0</v>
@@ -24179,10 +24179,10 @@
         </is>
       </c>
       <c r="AO76" s="47" t="n">
-        <v>4.9</v>
+        <v>3.9</v>
       </c>
       <c r="AP76" s="48" t="n">
-        <v>3.4</v>
+        <v>4.6</v>
       </c>
       <c r="AQ76" s="163" t="n">
         <v>0</v>
@@ -24403,10 +24403,10 @@
         </is>
       </c>
       <c r="AO77" s="47" t="n">
-        <v>7.4</v>
+        <v>5</v>
       </c>
       <c r="AP77" s="48" t="n">
-        <v>5.4</v>
+        <v>4.5</v>
       </c>
       <c r="AQ77" s="163" t="n">
         <v>0</v>
@@ -24694,10 +24694,10 @@
         </is>
       </c>
       <c r="AO78" s="47" t="n">
-        <v>6.4</v>
+        <v>5.5</v>
       </c>
       <c r="AP78" s="48" t="n">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="AQ78" s="163" t="n">
         <v>0</v>
@@ -24987,7 +24987,7 @@
         </is>
       </c>
       <c r="AO79" s="47" t="n">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="AP79" s="48" t="n">
         <v>9</v>
@@ -25275,10 +25275,10 @@
         </is>
       </c>
       <c r="AO80" s="47" t="n">
-        <v>7.1</v>
+        <v>8.9</v>
       </c>
       <c r="AP80" s="48" t="n">
-        <v>4.4</v>
+        <v>0.5</v>
       </c>
       <c r="AQ80" s="163" t="n">
         <v>0</v>
@@ -25545,10 +25545,10 @@
         </is>
       </c>
       <c r="AO81" s="47" t="n">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="AP81" s="48" t="n">
-        <v>5</v>
+        <v>2.7</v>
       </c>
       <c r="AQ81" s="163" t="n">
         <v>0</v>
@@ -25821,10 +25821,10 @@
         </is>
       </c>
       <c r="AO82" s="47" t="n">
-        <v>6.6</v>
+        <v>5.7</v>
       </c>
       <c r="AP82" s="48" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="AQ82" s="163" t="n">
         <v>0</v>
@@ -26113,10 +26113,10 @@
         </is>
       </c>
       <c r="AO83" s="47" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="AP83" s="48" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ83" s="163" t="n">
         <v>0</v>
@@ -26401,10 +26401,10 @@
         </is>
       </c>
       <c r="AO84" s="47" t="n">
-        <v>5.7</v>
+        <v>7.1</v>
       </c>
       <c r="AP84" s="48" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="AQ84" s="163" t="n">
         <v>0</v>
@@ -26687,10 +26687,10 @@
         </is>
       </c>
       <c r="AO85" s="47" t="n">
-        <v>5.3</v>
+        <v>4.7</v>
       </c>
       <c r="AP85" s="48" t="n">
-        <v>3</v>
+        <v>4.1</v>
       </c>
       <c r="AQ85" s="163" t="n">
         <v>0</v>
@@ -26969,10 +26969,10 @@
         </is>
       </c>
       <c r="AO86" s="47" t="n">
-        <v>3.3</v>
+        <v>6.6</v>
       </c>
       <c r="AP86" s="48" t="n">
-        <v>8.4</v>
+        <v>2.2</v>
       </c>
       <c r="AQ86" s="163" t="n">
         <v>0</v>
@@ -27248,10 +27248,10 @@
         </is>
       </c>
       <c r="AO87" s="47" t="n">
-        <v>9</v>
+        <v>7.2</v>
       </c>
       <c r="AP87" s="48" t="n">
-        <v>4.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ87" s="163" t="n">
         <v>0</v>
@@ -27528,10 +27528,10 @@
         </is>
       </c>
       <c r="AO88" s="47" t="n">
-        <v>7.2</v>
+        <v>4.1</v>
       </c>
       <c r="AP88" s="48" t="n">
-        <v>3.3</v>
+        <v>1.7</v>
       </c>
       <c r="AQ88" s="163" t="n">
         <v>0</v>
@@ -27800,10 +27800,10 @@
         </is>
       </c>
       <c r="AO89" s="47" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="AP89" s="48" t="n">
-        <v>4.1</v>
+        <v>2.9</v>
       </c>
       <c r="AQ89" s="163" t="n">
         <v>0</v>
@@ -28093,10 +28093,10 @@
         </is>
       </c>
       <c r="AO90" s="47" t="n">
-        <v>7.4</v>
+        <v>6.8</v>
       </c>
       <c r="AP90" s="48" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="AQ90" s="163" t="n">
         <v>0</v>
@@ -28385,10 +28385,10 @@
         </is>
       </c>
       <c r="AO91" s="45" t="n">
-        <v>7</v>
+        <v>4.9</v>
       </c>
       <c r="AP91" s="48" t="n">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="AQ91" s="163" t="n">
         <v>0</v>
@@ -28665,10 +28665,10 @@
         </is>
       </c>
       <c r="AO92" s="47" t="n">
-        <v>6.3</v>
+        <v>3.5</v>
       </c>
       <c r="AP92" s="48" t="n">
-        <v>4.1</v>
+        <v>2.5</v>
       </c>
       <c r="AQ92" s="163" t="n">
         <v>0</v>
@@ -28962,10 +28962,10 @@
         </is>
       </c>
       <c r="AO93" s="47" t="n">
-        <v>8.800000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="AP93" s="48" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="AQ93" s="163" t="n">
         <v>0</v>
@@ -29240,10 +29240,10 @@
         </is>
       </c>
       <c r="AO94" s="47" t="n">
-        <v>6.6</v>
+        <v>4.7</v>
       </c>
       <c r="AP94" s="48" t="n">
-        <v>4.2</v>
+        <v>2.5</v>
       </c>
       <c r="AQ94" s="163" t="n">
         <v>0</v>
@@ -29525,10 +29525,10 @@
         </is>
       </c>
       <c r="AO95" s="47" t="n">
-        <v>6.3</v>
+        <v>2.9</v>
       </c>
       <c r="AP95" s="48" t="n">
-        <v>4.1</v>
+        <v>2.6</v>
       </c>
       <c r="AQ95" s="163" t="n">
         <v>0</v>
@@ -29810,10 +29810,10 @@
         </is>
       </c>
       <c r="AO96" s="47" t="n">
-        <v>5.9</v>
+        <v>2.3</v>
       </c>
       <c r="AP96" s="48" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="AQ96" s="163" t="n">
         <v>0</v>
@@ -30088,10 +30088,10 @@
         </is>
       </c>
       <c r="AO97" s="47" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="AP97" s="88" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="AQ97" s="165" t="n">
         <v>0</v>
@@ -30366,10 +30366,10 @@
         </is>
       </c>
       <c r="AO98" s="47" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="AP98" s="48" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="AQ98" s="163" t="n">
         <v>0</v>
@@ -30637,10 +30637,10 @@
         </is>
       </c>
       <c r="AO99" s="47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP99" s="48" t="n">
-        <v>4.8</v>
+        <v>2.5</v>
       </c>
       <c r="AQ99" s="163" t="n">
         <v>0.1</v>
@@ -30918,10 +30918,10 @@
         </is>
       </c>
       <c r="AO100" s="47" t="n">
-        <v>4.3</v>
+        <v>5.5</v>
       </c>
       <c r="AP100" s="48" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="AQ100" s="163" t="n">
         <v>0</v>
@@ -31196,10 +31196,10 @@
         </is>
       </c>
       <c r="AO101" s="47" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
       <c r="AP101" s="48" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="AQ101" s="163" t="n">
         <v>0.01</v>
@@ -31473,10 +31473,10 @@
         </is>
       </c>
       <c r="AO102" s="47" t="n">
-        <v>6</v>
+        <v>2.9</v>
       </c>
       <c r="AP102" s="48" t="n">
-        <v>5.4</v>
+        <v>1</v>
       </c>
       <c r="AQ102" s="163" t="n">
         <v>0</v>
@@ -31743,10 +31743,10 @@
         </is>
       </c>
       <c r="AO103" s="47" t="n">
-        <v>7.9</v>
+        <v>8.9</v>
       </c>
       <c r="AP103" s="48" t="n">
-        <v>2.1</v>
+        <v>1.4</v>
       </c>
       <c r="AQ103" s="163" t="n">
         <v>0</v>
@@ -32026,7 +32026,7 @@
         <v>6.6</v>
       </c>
       <c r="AP104" s="48" t="n">
-        <v>1.1</v>
+        <v>0.1</v>
       </c>
       <c r="AQ104" s="163" t="n">
         <v>0</v>
@@ -32300,10 +32300,10 @@
         </is>
       </c>
       <c r="AO105" s="47" t="n">
-        <v>5.8</v>
+        <v>2.1</v>
       </c>
       <c r="AP105" s="48" t="n">
-        <v>5.6</v>
+        <v>1.3</v>
       </c>
       <c r="AQ105" s="163" t="n">
         <v>0</v>
@@ -32572,10 +32572,10 @@
         </is>
       </c>
       <c r="AO106" s="47" t="n">
-        <v>1.3</v>
+        <v>3.6</v>
       </c>
       <c r="AP106" s="48" t="n">
-        <v>6.8</v>
+        <v>2.1</v>
       </c>
       <c r="AQ106" s="163" t="n">
         <v>0</v>
@@ -32838,10 +32838,10 @@
         </is>
       </c>
       <c r="AO107" s="47" t="n">
-        <v>6</v>
+        <v>6.3</v>
       </c>
       <c r="AP107" s="88" t="n">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
       <c r="AQ107" s="165" t="n">
         <v>0</v>
@@ -33107,10 +33107,10 @@
         </is>
       </c>
       <c r="AO108" s="47" t="n">
-        <v>2.8</v>
+        <v>5.4</v>
       </c>
       <c r="AP108" s="48" t="n">
-        <v>6.2</v>
+        <v>3.1</v>
       </c>
       <c r="AQ108" s="163" t="n">
         <v>0</v>
@@ -33375,10 +33375,10 @@
         </is>
       </c>
       <c r="AO109" s="47" t="n">
-        <v>6.1</v>
+        <v>1.7</v>
       </c>
       <c r="AP109" s="48" t="n">
-        <v>5.5</v>
+        <v>2.3</v>
       </c>
       <c r="AQ109" s="163" t="n">
         <v>0</v>
@@ -33645,10 +33645,10 @@
         </is>
       </c>
       <c r="AO110" s="47" t="n">
-        <v>1.6</v>
+        <v>4.1</v>
       </c>
       <c r="AP110" s="48" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
       <c r="AQ110" s="163" t="n">
         <v>0</v>
@@ -33921,10 +33921,10 @@
         </is>
       </c>
       <c r="AO111" s="47" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="AP111" s="48" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="AQ111" s="163" t="n">
         <v>0</v>
@@ -34193,10 +34193,10 @@
         </is>
       </c>
       <c r="AO112" s="47" t="n">
-        <v>3.3</v>
+        <v>1.5</v>
       </c>
       <c r="AP112" s="48" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="AQ112" s="163" t="n">
         <v>0.03</v>
@@ -34470,10 +34470,10 @@
         </is>
       </c>
       <c r="AO113" s="47" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="AP113" s="48" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="AQ113" s="163" t="n">
         <v>0</v>
@@ -34754,10 +34754,10 @@
         </is>
       </c>
       <c r="AO114" s="47" t="n">
-        <v>6.8</v>
+        <v>2.3</v>
       </c>
       <c r="AP114" s="48" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="AQ114" s="163" t="n">
         <v>0.03</v>
@@ -35037,7 +35037,7 @@
         </is>
       </c>
       <c r="AO115" s="47" t="n">
-        <v>6.8</v>
+        <v>1.2</v>
       </c>
       <c r="AP115" s="48" t="n">
         <v>4.5</v>
@@ -35320,10 +35320,10 @@
         </is>
       </c>
       <c r="AO116" s="47" t="n">
-        <v>6.6</v>
+        <v>1.1</v>
       </c>
       <c r="AP116" s="48" t="n">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
       <c r="AQ116" s="163" t="n">
         <v>0.09</v>
@@ -35595,10 +35595,10 @@
         </is>
       </c>
       <c r="AO117" s="47" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
       <c r="AP117" s="48" t="n">
-        <v>5.4</v>
+        <v>3.5</v>
       </c>
       <c r="AQ117" s="163" t="n">
         <v>0</v>
@@ -35876,10 +35876,10 @@
         </is>
       </c>
       <c r="AO118" s="47" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="AP118" s="48" t="n">
-        <v>6.4</v>
+        <v>4.1</v>
       </c>
       <c r="AQ118" s="163" t="n">
         <v>0</v>
@@ -36153,10 +36153,10 @@
         </is>
       </c>
       <c r="AO119" s="74" t="n">
-        <v>4.6</v>
+        <v>3.3</v>
       </c>
       <c r="AP119" s="75" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="AQ119" s="173" t="n">
         <v>0</v>
@@ -36428,10 +36428,10 @@
         </is>
       </c>
       <c r="AO120" s="74" t="n">
-        <v>4.4</v>
+        <v>2.8</v>
       </c>
       <c r="AP120" s="75" t="n">
-        <v>3.9</v>
+        <v>0.5</v>
       </c>
       <c r="AQ120" s="168" t="n">
         <v>0</v>
@@ -36711,7 +36711,7 @@
         <v>6.8</v>
       </c>
       <c r="AP121" s="75" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="AQ121" s="168" t="n">
         <v>0</v>
@@ -36984,10 +36984,10 @@
         </is>
       </c>
       <c r="AO122" s="74" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="AP122" s="75" t="n">
-        <v>4.9</v>
+        <v>1.1</v>
       </c>
       <c r="AQ122" s="168" t="n">
         <v>0</v>
@@ -37256,10 +37256,10 @@
         </is>
       </c>
       <c r="AO123" s="47" t="n">
-        <v>5.9</v>
+        <v>4.1</v>
       </c>
       <c r="AP123" s="88" t="n">
-        <v>5.8</v>
+        <v>4.9</v>
       </c>
       <c r="AQ123" s="164" t="n">
         <v>0.035</v>
@@ -37542,10 +37542,10 @@
         </is>
       </c>
       <c r="AO124" s="47" t="n">
-        <v>7.1</v>
+        <v>8.9</v>
       </c>
       <c r="AP124" s="88" t="n">
-        <v>4.4</v>
+        <v>0.5</v>
       </c>
       <c r="AQ124" s="164" t="n">
         <v>0</v>
@@ -37818,10 +37818,10 @@
         </is>
       </c>
       <c r="AO125" s="74" t="n">
-        <v>7.3</v>
+        <v>6.7</v>
       </c>
       <c r="AP125" s="75" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ125" s="168" t="n">
         <v>0</v>
@@ -38098,10 +38098,10 @@
         </is>
       </c>
       <c r="AO126" s="74" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="AP126" s="75" t="n">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
       <c r="AQ126" s="168" t="n">
         <v>0</v>
@@ -38386,10 +38386,10 @@
         </is>
       </c>
       <c r="AO127" s="74" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="AP127" s="48" t="n">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
       <c r="AQ127" s="167" t="n">
         <v>0</v>
@@ -38660,10 +38660,10 @@
         </is>
       </c>
       <c r="AO128" s="74" t="n">
-        <v>5.4</v>
+        <v>1.6</v>
       </c>
       <c r="AP128" s="75" t="n">
-        <v>5.7</v>
+        <v>3.2</v>
       </c>
       <c r="AQ128" s="168" t="n">
         <v>0.083</v>
@@ -38950,10 +38950,10 @@
         </is>
       </c>
       <c r="AO129" s="74" t="n">
-        <v>5.9</v>
+        <v>4.2</v>
       </c>
       <c r="AP129" s="75" t="n">
-        <v>7.1</v>
+        <v>2.6</v>
       </c>
       <c r="AQ129" s="167" t="n">
         <v>0</v>
@@ -39230,10 +39230,10 @@
         </is>
       </c>
       <c r="AO130" s="47" t="n">
-        <v>7.4</v>
+        <v>4.8</v>
       </c>
       <c r="AP130" s="88" t="n">
-        <v>7.2</v>
+        <v>2.6</v>
       </c>
       <c r="AQ130" s="164" t="n">
         <v>0</v>
@@ -39510,10 +39510,10 @@
         </is>
       </c>
       <c r="AO131" s="47" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="AP131" s="88" t="n">
-        <v>4.9</v>
+        <v>2.2</v>
       </c>
       <c r="AQ131" s="164" t="n">
         <v>0</v>
@@ -39782,10 +39782,10 @@
         </is>
       </c>
       <c r="AO132" s="47" t="n">
-        <v>3.1</v>
+        <v>5.5</v>
       </c>
       <c r="AP132" s="88" t="n">
-        <v>5.5</v>
+        <v>1.3</v>
       </c>
       <c r="AQ132" s="164" t="n">
         <v>0</v>
@@ -40058,10 +40058,10 @@
         </is>
       </c>
       <c r="AO133" s="47" t="n">
-        <v>4.9</v>
+        <v>5.4</v>
       </c>
       <c r="AP133" s="88" t="n">
-        <v>4.7</v>
+        <v>1.2</v>
       </c>
       <c r="AQ133" s="164" t="n">
         <v>0</v>
@@ -40614,10 +40614,10 @@
         </is>
       </c>
       <c r="AO135" s="47" t="n">
-        <v>1.6</v>
+        <v>3.6</v>
       </c>
       <c r="AP135" s="88" t="n">
-        <v>4.6</v>
+        <v>2.3</v>
       </c>
       <c r="AQ135" s="164" t="n">
         <v>0</v>
@@ -40904,10 +40904,10 @@
         </is>
       </c>
       <c r="AO136" s="47" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="AP136" s="88" t="n">
-        <v>6.3</v>
+        <v>1</v>
       </c>
       <c r="AQ136" s="164" t="n">
         <v>0</v>
@@ -41182,10 +41182,10 @@
         </is>
       </c>
       <c r="AO137" s="45" t="n">
-        <v>6.9</v>
+        <v>3.8</v>
       </c>
       <c r="AP137" s="48" t="n">
-        <v>6.7</v>
+        <v>3.2</v>
       </c>
       <c r="AQ137" s="167" t="n">
         <v>0</v>
@@ -41747,7 +41747,7 @@
         <v>4.4</v>
       </c>
       <c r="AP139" s="48" t="n">
-        <v>4.5</v>
+        <v>2.3</v>
       </c>
       <c r="AQ139" s="167" t="n">
         <v>0</v>
@@ -42022,10 +42022,10 @@
         </is>
       </c>
       <c r="AO140" s="88" t="n">
-        <v>6.9</v>
+        <v>2.8</v>
       </c>
       <c r="AP140" s="118" t="n">
-        <v>6.7</v>
+        <v>3.4</v>
       </c>
       <c r="AQ140" s="172" t="n">
         <v>0.038</v>
@@ -42302,10 +42302,10 @@
         </is>
       </c>
       <c r="AO141" s="74" t="n">
-        <v>7.1</v>
+        <v>3.2</v>
       </c>
       <c r="AP141" s="88" t="n">
-        <v>6.4</v>
+        <v>2.5</v>
       </c>
       <c r="AQ141" s="167" t="n">
         <v>0</v>
@@ -42578,10 +42578,10 @@
         </is>
       </c>
       <c r="AO142" s="47" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="AP142" s="118" t="n">
-        <v>5.4</v>
+        <v>2.2</v>
       </c>
       <c r="AQ142" s="167" t="n">
         <v>0.01</v>
@@ -42848,10 +42848,10 @@
         </is>
       </c>
       <c r="AO143" s="47" t="n">
-        <v>5.2</v>
+        <v>6.7</v>
       </c>
       <c r="AP143" s="118" t="n">
-        <v>2.6</v>
+        <v>0.3</v>
       </c>
       <c r="AQ143" s="172" t="n">
         <v>0</v>
@@ -43402,10 +43402,10 @@
         </is>
       </c>
       <c r="AO145" s="74" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="AP145" s="118" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="AQ145" s="172" t="n">
         <v>0</v>
@@ -43688,10 +43688,10 @@
         </is>
       </c>
       <c r="AO146" s="47" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="AP146" s="88" t="n">
-        <v>7.7</v>
+        <v>3.2</v>
       </c>
       <c r="AQ146" s="164" t="n">
         <v>0</v>
@@ -43970,10 +43970,10 @@
         </is>
       </c>
       <c r="AO147" s="74" t="n">
-        <v>4.9</v>
+        <v>5.2</v>
       </c>
       <c r="AP147" s="48" t="n">
-        <v>4.6</v>
+        <v>2.9</v>
       </c>
       <c r="AQ147" s="167" t="n">
         <v>0</v>
@@ -44252,10 +44252,10 @@
         </is>
       </c>
       <c r="AO148" s="74" t="n">
-        <v>6.9</v>
+        <v>4</v>
       </c>
       <c r="AP148" s="48" t="n">
-        <v>6.7</v>
+        <v>3.3</v>
       </c>
       <c r="AQ148" s="167" t="n">
         <v>0</v>
@@ -44532,10 +44532,10 @@
         </is>
       </c>
       <c r="AO149" s="47" t="n">
-        <v>7.1</v>
+        <v>5.5</v>
       </c>
       <c r="AP149" s="118" t="n">
-        <v>6.9</v>
+        <v>3</v>
       </c>
       <c r="AQ149" s="164" t="n">
         <v>0</v>
@@ -44812,10 +44812,10 @@
         </is>
       </c>
       <c r="AO150" s="47" t="n">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="AP150" s="118" t="n">
-        <v>5.4</v>
+        <v>3.5</v>
       </c>
       <c r="AQ150" s="172" t="n">
         <v>0</v>
@@ -45094,10 +45094,10 @@
         </is>
       </c>
       <c r="AO151" s="74" t="n">
-        <v>5.3</v>
+        <v>3.2</v>
       </c>
       <c r="AP151" s="118" t="n">
-        <v>3.3</v>
+        <v>0.8</v>
       </c>
       <c r="AQ151" s="172" t="n">
         <v>0</v>
@@ -45660,10 +45660,10 @@
         </is>
       </c>
       <c r="AO153" s="74" t="n">
-        <v>4.7</v>
+        <v>6.8</v>
       </c>
       <c r="AP153" s="118" t="n">
-        <v>3.9</v>
+        <v>2.9</v>
       </c>
       <c r="AQ153" s="174" t="n">
         <v>0</v>
@@ -46208,10 +46208,10 @@
         </is>
       </c>
       <c r="AO155" s="74" t="n">
-        <v>7.2</v>
+        <v>9</v>
       </c>
       <c r="AP155" s="118" t="n">
-        <v>2.5</v>
+        <v>0.6</v>
       </c>
       <c r="AQ155" s="172" t="n">
         <v>0</v>
@@ -46492,10 +46492,10 @@
         </is>
       </c>
       <c r="AO156" s="47" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="AP156" s="88" t="n">
-        <v>5.7</v>
+        <v>4.5</v>
       </c>
       <c r="AQ156" s="164" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Rework scoring: per-size-bucket with chamfer fraction and force distribution shape
- Add chamfer fraction metric: 0.020" x 45° chamfer on all PDCs means smaller
  cutlets have proportionally more chamfer area → less efficient but more durable
- Score each bit size bucket independently 0-9, then best-fit rescale across
  buckets using size-independent reference metrics as anchors
- Replace absolute metrics (cutter count, work per cutter) with distribution
  shape metrics: force uniformity (entropy), force spread, load balance (Gini)
- Add perimeter output to cutlet_engine for chamfer fraction computation
- Remove Rev 3 from cutlet engine (Rev 3 never masks Rev 2, ~55% speedup)
- Update CUTLET_ANALYSIS_NOTES.md with chamfer physics and per-size methodology

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Bit Applications Tool r2.xlsx
+++ b/Bit Applications Tool r2.xlsx
@@ -4401,10 +4401,10 @@
         </is>
       </c>
       <c r="AO5" s="47" t="n">
-        <v>3.6</v>
+        <v>0.9</v>
       </c>
       <c r="AP5" s="48" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="AQ5" s="163" t="n">
         <v>0</v>
@@ -4935,10 +4935,10 @@
         </is>
       </c>
       <c r="AO7" s="74" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="AP7" s="75" t="n">
-        <v>4.1</v>
+        <v>3.7</v>
       </c>
       <c r="AQ7" s="168" t="n">
         <v>0.1</v>
@@ -5993,10 +5993,10 @@
         </is>
       </c>
       <c r="AO11" s="47" t="n">
-        <v>5.5</v>
+        <v>4.8</v>
       </c>
       <c r="AP11" s="48" t="n">
-        <v>1.3</v>
+        <v>4.8</v>
       </c>
       <c r="AQ11" s="167" t="n">
         <v>0.02</v>
@@ -6263,10 +6263,10 @@
         </is>
       </c>
       <c r="AO12" s="47" t="n">
-        <v>3.8</v>
+        <v>4.9</v>
       </c>
       <c r="AP12" s="48" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="AQ12" s="163" t="n">
         <v>0</v>
@@ -6805,10 +6805,10 @@
         </is>
       </c>
       <c r="AO14" s="47" t="n">
-        <v>4.1</v>
+        <v>5.4</v>
       </c>
       <c r="AP14" s="48" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="AQ14" s="163" t="n">
         <v>0</v>
@@ -8671,10 +8671,10 @@
         </is>
       </c>
       <c r="AO21" s="47" t="n">
-        <v>5.8</v>
+        <v>6.6</v>
       </c>
       <c r="AP21" s="48" t="n">
-        <v>1.7</v>
+        <v>5.4</v>
       </c>
       <c r="AQ21" s="163" t="n">
         <v>0</v>
@@ -9739,10 +9739,10 @@
         </is>
       </c>
       <c r="AO25" s="47" t="n">
-        <v>6.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AP25" s="48" t="n">
-        <v>4.5</v>
+        <v>1.9</v>
       </c>
       <c r="AQ25" s="163" t="n">
         <v>0</v>
@@ -10555,10 +10555,10 @@
         </is>
       </c>
       <c r="AO28" s="47" t="n">
-        <v>7.2</v>
+        <v>3.3</v>
       </c>
       <c r="AP28" s="48" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="AQ28" s="163" t="n">
         <v>0</v>
@@ -10840,7 +10840,7 @@
         <v>5.5</v>
       </c>
       <c r="AP29" s="48" t="n">
-        <v>4.1</v>
+        <v>7.5</v>
       </c>
       <c r="AQ29" s="163" t="n">
         <v>0</v>
@@ -11117,10 +11117,10 @@
         </is>
       </c>
       <c r="AO30" s="47" t="n">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="AP30" s="48" t="n">
-        <v>2.6</v>
+        <v>4.9</v>
       </c>
       <c r="AQ30" s="163" t="n">
         <v>0</v>
@@ -11425,10 +11425,10 @@
         </is>
       </c>
       <c r="AO31" s="46" t="n">
-        <v>6.3</v>
+        <v>7.2</v>
       </c>
       <c r="AP31" s="48" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AQ31" s="163" t="n">
         <v>0</v>
@@ -11727,10 +11727,10 @@
         </is>
       </c>
       <c r="AO32" s="46" t="n">
-        <v>7.9</v>
+        <v>7.8</v>
       </c>
       <c r="AP32" s="48" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="AQ32" s="163" t="n">
         <v>0</v>
@@ -12007,10 +12007,10 @@
         </is>
       </c>
       <c r="AO33" s="47" t="n">
-        <v>8.1</v>
+        <v>7.3</v>
       </c>
       <c r="AP33" s="48" t="n">
-        <v>1.6</v>
+        <v>6.1</v>
       </c>
       <c r="AQ33" s="163" t="n">
         <v>0</v>
@@ -12289,10 +12289,10 @@
         </is>
       </c>
       <c r="AO34" s="47" t="n">
-        <v>8.1</v>
+        <v>6.5</v>
       </c>
       <c r="AP34" s="48" t="n">
-        <v>1.3</v>
+        <v>3.3</v>
       </c>
       <c r="AQ34" s="163" t="n">
         <v>0</v>
@@ -12571,10 +12571,10 @@
         </is>
       </c>
       <c r="AO35" s="47" t="n">
-        <v>4.6</v>
+        <v>7.9</v>
       </c>
       <c r="AP35" s="48" t="n">
-        <v>5.1</v>
+        <v>1.2</v>
       </c>
       <c r="AQ35" s="163" t="n">
         <v>0</v>
@@ -12857,10 +12857,10 @@
         </is>
       </c>
       <c r="AO36" s="46" t="n">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="AP36" s="48" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="AQ36" s="163" t="n">
         <v>0</v>
@@ -13135,10 +13135,10 @@
         </is>
       </c>
       <c r="AO37" s="47" t="n">
-        <v>6.1</v>
+        <v>4.4</v>
       </c>
       <c r="AP37" s="48" t="n">
-        <v>2.6</v>
+        <v>5.7</v>
       </c>
       <c r="AQ37" s="163" t="n">
         <v>0</v>
@@ -13437,10 +13437,10 @@
         </is>
       </c>
       <c r="AO38" s="46" t="n">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="AP38" s="48" t="n">
-        <v>4.5</v>
+        <v>7.4</v>
       </c>
       <c r="AQ38" s="163" t="n">
         <v>0</v>
@@ -13975,10 +13975,10 @@
         </is>
       </c>
       <c r="AO40" s="47" t="n">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
       <c r="AP40" s="48" t="n">
-        <v>2.5</v>
+        <v>5.6</v>
       </c>
       <c r="AQ40" s="163" t="n">
         <v>0</v>
@@ -14271,10 +14271,10 @@
         </is>
       </c>
       <c r="AO41" s="46" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="AP41" s="48" t="n">
-        <v>0.6</v>
+        <v>3.1</v>
       </c>
       <c r="AQ41" s="163" t="n">
         <v>0</v>
@@ -14551,10 +14551,10 @@
         </is>
       </c>
       <c r="AO42" s="47" t="n">
-        <v>3.7</v>
+        <v>2.8</v>
       </c>
       <c r="AP42" s="48" t="n">
-        <v>1.4</v>
+        <v>4.9</v>
       </c>
       <c r="AQ42" s="163" t="n">
         <v>0</v>
@@ -14851,10 +14851,10 @@
         </is>
       </c>
       <c r="AO43" s="46" t="n">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
       <c r="AP43" s="48" t="n">
-        <v>4.2</v>
+        <v>5.9</v>
       </c>
       <c r="AQ43" s="163" t="n">
         <v>0</v>
@@ -15133,10 +15133,10 @@
         </is>
       </c>
       <c r="AO44" s="47" t="n">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
       <c r="AP44" s="48" t="n">
-        <v>3.2</v>
+        <v>5.4</v>
       </c>
       <c r="AQ44" s="163" t="n">
         <v>0</v>
@@ -15411,10 +15411,10 @@
         </is>
       </c>
       <c r="AO45" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP45" s="48" t="n">
-        <v>4.3</v>
+        <v>7.6</v>
       </c>
       <c r="AQ45" s="163" t="n">
         <v>0</v>
@@ -15689,10 +15689,10 @@
         </is>
       </c>
       <c r="AO46" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP46" s="48" t="n">
-        <v>4.3</v>
+        <v>7.6</v>
       </c>
       <c r="AQ46" s="163" t="n">
         <v>0</v>
@@ -15967,10 +15967,10 @@
         </is>
       </c>
       <c r="AO47" s="47" t="n">
-        <v>5.9</v>
+        <v>4.6</v>
       </c>
       <c r="AP47" s="48" t="n">
-        <v>3.3</v>
+        <v>6.6</v>
       </c>
       <c r="AQ47" s="163" t="n">
         <v>0</v>
@@ -16255,10 +16255,10 @@
         </is>
       </c>
       <c r="AO48" s="47" t="n">
-        <v>4.5</v>
+        <v>5.7</v>
       </c>
       <c r="AP48" s="48" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="AQ48" s="163" t="n">
         <v>0</v>
@@ -16549,10 +16549,10 @@
         </is>
       </c>
       <c r="AO49" s="46" t="n">
-        <v>5</v>
+        <v>4.3</v>
       </c>
       <c r="AP49" s="48" t="n">
-        <v>2.8</v>
+        <v>5.1</v>
       </c>
       <c r="AQ49" s="163" t="n">
         <v>0</v>
@@ -16829,10 +16829,10 @@
         </is>
       </c>
       <c r="AO50" s="47" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="AP50" s="48" t="n">
-        <v>2.3</v>
+        <v>5.9</v>
       </c>
       <c r="AQ50" s="163" t="n">
         <v>0</v>
@@ -17131,10 +17131,10 @@
         </is>
       </c>
       <c r="AO51" s="46" t="n">
-        <v>5.3</v>
+        <v>3.8</v>
       </c>
       <c r="AP51" s="48" t="n">
-        <v>4.1</v>
+        <v>6.2</v>
       </c>
       <c r="AQ51" s="163" t="n">
         <v>0</v>
@@ -17415,10 +17415,10 @@
         </is>
       </c>
       <c r="AO52" s="47" t="n">
-        <v>4.3</v>
+        <v>5.1</v>
       </c>
       <c r="AP52" s="48" t="n">
-        <v>2.7</v>
+        <v>6.8</v>
       </c>
       <c r="AQ52" s="163" t="n">
         <v>0</v>
@@ -17686,10 +17686,10 @@
         </is>
       </c>
       <c r="AO53" s="47" t="n">
-        <v>4.1</v>
+        <v>3.8</v>
       </c>
       <c r="AP53" s="48" t="n">
-        <v>3.3</v>
+        <v>5.8</v>
       </c>
       <c r="AQ53" s="163" t="n">
         <v>0</v>
@@ -17962,10 +17962,10 @@
         </is>
       </c>
       <c r="AO54" s="47" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="AP54" s="48" t="n">
-        <v>4.8</v>
+        <v>6.5</v>
       </c>
       <c r="AQ54" s="163" t="n">
         <v>0</v>
@@ -18228,10 +18228,10 @@
         </is>
       </c>
       <c r="AO55" s="47" t="n">
-        <v>3.1</v>
+        <v>3.6</v>
       </c>
       <c r="AP55" s="48" t="n">
-        <v>1.6</v>
+        <v>4.5</v>
       </c>
       <c r="AQ55" s="163" t="n">
         <v>0</v>
@@ -18512,10 +18512,10 @@
         </is>
       </c>
       <c r="AO56" s="47" t="n">
-        <v>6.2</v>
+        <v>4.8</v>
       </c>
       <c r="AP56" s="48" t="n">
-        <v>4.1</v>
+        <v>7.4</v>
       </c>
       <c r="AQ56" s="163" t="n">
         <v>0</v>
@@ -18794,10 +18794,10 @@
         </is>
       </c>
       <c r="AO57" s="47" t="n">
-        <v>3.9</v>
+        <v>5.5</v>
       </c>
       <c r="AP57" s="48" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="AQ57" s="163" t="n">
         <v>0</v>
@@ -19076,10 +19076,10 @@
         </is>
       </c>
       <c r="AO58" s="47" t="n">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="AP58" s="48" t="n">
-        <v>1.9</v>
+        <v>4.6</v>
       </c>
       <c r="AQ58" s="163" t="n">
         <v>0</v>
@@ -19355,10 +19355,10 @@
         </is>
       </c>
       <c r="AO59" s="47" t="n">
-        <v>4.3</v>
+        <v>4.9</v>
       </c>
       <c r="AP59" s="48" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="AQ59" s="163" t="n">
         <v>0</v>
@@ -19639,10 +19639,10 @@
         </is>
       </c>
       <c r="AO60" s="47" t="n">
-        <v>5.4</v>
+        <v>4.6</v>
       </c>
       <c r="AP60" s="48" t="n">
-        <v>3.8</v>
+        <v>6.9</v>
       </c>
       <c r="AQ60" s="163" t="n">
         <v>0</v>
@@ -19921,10 +19921,10 @@
         </is>
       </c>
       <c r="AO61" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP61" s="48" t="n">
-        <v>4.3</v>
+        <v>7.6</v>
       </c>
       <c r="AQ61" s="163" t="n">
         <v>0</v>
@@ -20203,10 +20203,10 @@
         </is>
       </c>
       <c r="AO62" s="47" t="n">
-        <v>5.5</v>
+        <v>4.7</v>
       </c>
       <c r="AP62" s="48" t="n">
-        <v>1.9</v>
+        <v>5.7</v>
       </c>
       <c r="AQ62" s="163" t="n">
         <v>0</v>
@@ -20481,10 +20481,10 @@
         </is>
       </c>
       <c r="AO63" s="47" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="AP63" s="48" t="n">
-        <v>4.1</v>
+        <v>6.3</v>
       </c>
       <c r="AQ63" s="163" t="n">
         <v>0</v>
@@ -20764,10 +20764,10 @@
         </is>
       </c>
       <c r="AO64" s="47" t="n">
-        <v>4.1</v>
+        <v>4.5</v>
       </c>
       <c r="AP64" s="48" t="n">
-        <v>2.7</v>
+        <v>5.8</v>
       </c>
       <c r="AQ64" s="163" t="n">
         <v>0</v>
@@ -21044,10 +21044,10 @@
         </is>
       </c>
       <c r="AO65" s="47" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="AP65" s="48" t="n">
-        <v>2.6</v>
+        <v>5</v>
       </c>
       <c r="AQ65" s="163" t="n">
         <v>0.083</v>
@@ -21335,10 +21335,10 @@
         </is>
       </c>
       <c r="AO66" s="47" t="n">
-        <v>7.2</v>
+        <v>3.3</v>
       </c>
       <c r="AP66" s="48" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="AQ66" s="163" t="n">
         <v>0</v>
@@ -21625,10 +21625,10 @@
         </is>
       </c>
       <c r="AO67" s="47" t="n">
-        <v>5.8</v>
+        <v>6.7</v>
       </c>
       <c r="AP67" s="48" t="n">
-        <v>1.7</v>
+        <v>5.4</v>
       </c>
       <c r="AQ67" s="163" t="n">
         <v>0</v>
@@ -21913,10 +21913,10 @@
         </is>
       </c>
       <c r="AO68" s="47" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="AP68" s="48" t="n">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
       <c r="AQ68" s="163" t="n">
         <v>0</v>
@@ -22211,10 +22211,10 @@
         </is>
       </c>
       <c r="AO69" s="47" t="n">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="AP69" s="48" t="n">
-        <v>2.5</v>
+        <v>5.6</v>
       </c>
       <c r="AQ69" s="163" t="n">
         <v>0</v>
@@ -22485,10 +22485,10 @@
         </is>
       </c>
       <c r="AO70" s="47" t="n">
-        <v>2.9</v>
+        <v>3.4</v>
       </c>
       <c r="AP70" s="48" t="n">
-        <v>2.4</v>
+        <v>4.7</v>
       </c>
       <c r="AQ70" s="163" t="n">
         <v>0</v>
@@ -22777,10 +22777,10 @@
         </is>
       </c>
       <c r="AO71" s="47" t="n">
-        <v>3.7</v>
+        <v>5</v>
       </c>
       <c r="AP71" s="48" t="n">
-        <v>0.6</v>
+        <v>3.1</v>
       </c>
       <c r="AQ71" s="163" t="n">
         <v>0</v>
@@ -23055,10 +23055,10 @@
         </is>
       </c>
       <c r="AO72" s="47" t="n">
-        <v>3.3</v>
+        <v>4.2</v>
       </c>
       <c r="AP72" s="48" t="n">
-        <v>4.3</v>
+        <v>7.2</v>
       </c>
       <c r="AQ72" s="163" t="n">
         <v>0</v>
@@ -23336,10 +23336,10 @@
         </is>
       </c>
       <c r="AO73" s="47" t="n">
-        <v>5.4</v>
+        <v>4.6</v>
       </c>
       <c r="AP73" s="48" t="n">
-        <v>3.4</v>
+        <v>6.8</v>
       </c>
       <c r="AQ73" s="163" t="n">
         <v>0</v>
@@ -23617,10 +23617,10 @@
         </is>
       </c>
       <c r="AO74" s="47" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="AP74" s="48" t="n">
-        <v>3.6</v>
+        <v>8</v>
       </c>
       <c r="AQ74" s="163" t="n">
         <v>0</v>
@@ -23900,10 +23900,10 @@
         </is>
       </c>
       <c r="AO75" s="47" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="AP75" s="48" t="n">
-        <v>4.8</v>
+        <v>6.5</v>
       </c>
       <c r="AQ75" s="163" t="n">
         <v>0</v>
@@ -24179,10 +24179,10 @@
         </is>
       </c>
       <c r="AO76" s="47" t="n">
-        <v>3.9</v>
+        <v>5.6</v>
       </c>
       <c r="AP76" s="48" t="n">
-        <v>4.6</v>
+        <v>6.7</v>
       </c>
       <c r="AQ76" s="163" t="n">
         <v>0</v>
@@ -24403,10 +24403,10 @@
         </is>
       </c>
       <c r="AO77" s="47" t="n">
-        <v>5</v>
+        <v>4.4</v>
       </c>
       <c r="AP77" s="48" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="AQ77" s="163" t="n">
         <v>0</v>
@@ -24694,10 +24694,10 @@
         </is>
       </c>
       <c r="AO78" s="47" t="n">
-        <v>5.5</v>
+        <v>6.2</v>
       </c>
       <c r="AP78" s="48" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="AQ78" s="163" t="n">
         <v>0</v>
@@ -24987,10 +24987,10 @@
         </is>
       </c>
       <c r="AO79" s="47" t="n">
-        <v>3.7</v>
+        <v>1.4</v>
       </c>
       <c r="AP79" s="48" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="AQ79" s="163" t="n">
         <v>0</v>
@@ -25275,10 +25275,10 @@
         </is>
       </c>
       <c r="AO80" s="47" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
       <c r="AP80" s="48" t="n">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="AQ80" s="163" t="n">
         <v>0</v>
@@ -25545,10 +25545,10 @@
         </is>
       </c>
       <c r="AO81" s="47" t="n">
-        <v>3.5</v>
+        <v>5.3</v>
       </c>
       <c r="AP81" s="48" t="n">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
       <c r="AQ81" s="163" t="n">
         <v>0</v>
@@ -25821,10 +25821,10 @@
         </is>
       </c>
       <c r="AO82" s="47" t="n">
-        <v>5.7</v>
+        <v>4</v>
       </c>
       <c r="AP82" s="48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ82" s="163" t="n">
         <v>0</v>
@@ -26113,10 +26113,10 @@
         </is>
       </c>
       <c r="AO83" s="47" t="n">
-        <v>7.2</v>
+        <v>3.3</v>
       </c>
       <c r="AP83" s="48" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="AQ83" s="163" t="n">
         <v>0</v>
@@ -26401,10 +26401,10 @@
         </is>
       </c>
       <c r="AO84" s="47" t="n">
-        <v>7.1</v>
+        <v>6.1</v>
       </c>
       <c r="AP84" s="48" t="n">
-        <v>2.3</v>
+        <v>3.9</v>
       </c>
       <c r="AQ84" s="163" t="n">
         <v>0</v>
@@ -26687,10 +26687,10 @@
         </is>
       </c>
       <c r="AO85" s="47" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="AP85" s="48" t="n">
-        <v>4.1</v>
+        <v>3.7</v>
       </c>
       <c r="AQ85" s="163" t="n">
         <v>0</v>
@@ -26969,10 +26969,10 @@
         </is>
       </c>
       <c r="AO86" s="47" t="n">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="AP86" s="48" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="AQ86" s="163" t="n">
         <v>0</v>
@@ -27248,10 +27248,10 @@
         </is>
       </c>
       <c r="AO87" s="47" t="n">
-        <v>7.2</v>
+        <v>3.3</v>
       </c>
       <c r="AP87" s="48" t="n">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="AQ87" s="163" t="n">
         <v>0</v>
@@ -27528,10 +27528,10 @@
         </is>
       </c>
       <c r="AO88" s="47" t="n">
-        <v>4.1</v>
+        <v>3.5</v>
       </c>
       <c r="AP88" s="48" t="n">
-        <v>1.7</v>
+        <v>3.7</v>
       </c>
       <c r="AQ88" s="163" t="n">
         <v>0</v>
@@ -27800,10 +27800,10 @@
         </is>
       </c>
       <c r="AO89" s="47" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
       <c r="AP89" s="48" t="n">
-        <v>2.9</v>
+        <v>5.5</v>
       </c>
       <c r="AQ89" s="163" t="n">
         <v>0</v>
@@ -28093,10 +28093,10 @@
         </is>
       </c>
       <c r="AO90" s="47" t="n">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="AP90" s="48" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="AQ90" s="163" t="n">
         <v>0</v>
@@ -28385,10 +28385,10 @@
         </is>
       </c>
       <c r="AO91" s="45" t="n">
-        <v>4.9</v>
+        <v>4.7</v>
       </c>
       <c r="AP91" s="48" t="n">
-        <v>3.1</v>
+        <v>6.3</v>
       </c>
       <c r="AQ91" s="163" t="n">
         <v>0</v>
@@ -28665,10 +28665,10 @@
         </is>
       </c>
       <c r="AO92" s="47" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="AP92" s="48" t="n">
-        <v>2.5</v>
+        <v>6.1</v>
       </c>
       <c r="AQ92" s="163" t="n">
         <v>0</v>
@@ -28962,10 +28962,10 @@
         </is>
       </c>
       <c r="AO93" s="47" t="n">
-        <v>8.4</v>
+        <v>9</v>
       </c>
       <c r="AP93" s="48" t="n">
-        <v>3.2</v>
+        <v>1.8</v>
       </c>
       <c r="AQ93" s="163" t="n">
         <v>0</v>
@@ -29240,10 +29240,10 @@
         </is>
       </c>
       <c r="AO94" s="47" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="AP94" s="48" t="n">
-        <v>2.5</v>
+        <v>5.7</v>
       </c>
       <c r="AQ94" s="163" t="n">
         <v>0</v>
@@ -29525,10 +29525,10 @@
         </is>
       </c>
       <c r="AO95" s="47" t="n">
-        <v>2.9</v>
+        <v>4.1</v>
       </c>
       <c r="AP95" s="48" t="n">
-        <v>2.6</v>
+        <v>6</v>
       </c>
       <c r="AQ95" s="163" t="n">
         <v>0</v>
@@ -29810,10 +29810,10 @@
         </is>
       </c>
       <c r="AO96" s="47" t="n">
-        <v>2.3</v>
+        <v>4.7</v>
       </c>
       <c r="AP96" s="48" t="n">
-        <v>4.7</v>
+        <v>3.8</v>
       </c>
       <c r="AQ96" s="163" t="n">
         <v>0</v>
@@ -30088,10 +30088,10 @@
         </is>
       </c>
       <c r="AO97" s="47" t="n">
-        <v>6.3</v>
+        <v>7.4</v>
       </c>
       <c r="AP97" s="88" t="n">
-        <v>3.9</v>
+        <v>2</v>
       </c>
       <c r="AQ97" s="165" t="n">
         <v>0</v>
@@ -30366,10 +30366,10 @@
         </is>
       </c>
       <c r="AO98" s="47" t="n">
-        <v>3.2</v>
+        <v>6.7</v>
       </c>
       <c r="AP98" s="48" t="n">
-        <v>6.5</v>
+        <v>2.6</v>
       </c>
       <c r="AQ98" s="163" t="n">
         <v>0</v>
@@ -30637,10 +30637,10 @@
         </is>
       </c>
       <c r="AO99" s="47" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="AP99" s="48" t="n">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="AQ99" s="163" t="n">
         <v>0.1</v>
@@ -30918,10 +30918,10 @@
         </is>
       </c>
       <c r="AO100" s="47" t="n">
-        <v>5.5</v>
+        <v>5</v>
       </c>
       <c r="AP100" s="48" t="n">
-        <v>4.2</v>
+        <v>7</v>
       </c>
       <c r="AQ100" s="163" t="n">
         <v>0</v>
@@ -31196,10 +31196,10 @@
         </is>
       </c>
       <c r="AO101" s="47" t="n">
-        <v>2.3</v>
+        <v>4.8</v>
       </c>
       <c r="AP101" s="48" t="n">
-        <v>4.5</v>
+        <v>6.4</v>
       </c>
       <c r="AQ101" s="163" t="n">
         <v>0.01</v>
@@ -31473,10 +31473,10 @@
         </is>
       </c>
       <c r="AO102" s="47" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="AP102" s="48" t="n">
-        <v>1</v>
+        <v>3.1</v>
       </c>
       <c r="AQ102" s="163" t="n">
         <v>0</v>
@@ -31743,10 +31743,10 @@
         </is>
       </c>
       <c r="AO103" s="47" t="n">
-        <v>8.9</v>
+        <v>7.3</v>
       </c>
       <c r="AP103" s="48" t="n">
-        <v>1.4</v>
+        <v>6</v>
       </c>
       <c r="AQ103" s="163" t="n">
         <v>0</v>
@@ -32023,10 +32023,10 @@
         </is>
       </c>
       <c r="AO104" s="47" t="n">
-        <v>6.6</v>
+        <v>4.8</v>
       </c>
       <c r="AP104" s="48" t="n">
-        <v>0.1</v>
+        <v>4.7</v>
       </c>
       <c r="AQ104" s="163" t="n">
         <v>0</v>
@@ -32300,10 +32300,10 @@
         </is>
       </c>
       <c r="AO105" s="47" t="n">
-        <v>2.1</v>
+        <v>0.2</v>
       </c>
       <c r="AP105" s="48" t="n">
-        <v>1.3</v>
+        <v>4.6</v>
       </c>
       <c r="AQ105" s="163" t="n">
         <v>0</v>
@@ -32572,10 +32572,10 @@
         </is>
       </c>
       <c r="AO106" s="47" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="AP106" s="48" t="n">
-        <v>2.1</v>
+        <v>5.2</v>
       </c>
       <c r="AQ106" s="163" t="n">
         <v>0</v>
@@ -32838,10 +32838,10 @@
         </is>
       </c>
       <c r="AO107" s="47" t="n">
-        <v>6.3</v>
+        <v>7.4</v>
       </c>
       <c r="AP107" s="88" t="n">
-        <v>3.9</v>
+        <v>2</v>
       </c>
       <c r="AQ107" s="165" t="n">
         <v>0</v>
@@ -33107,10 +33107,10 @@
         </is>
       </c>
       <c r="AO108" s="47" t="n">
-        <v>5.4</v>
+        <v>4.3</v>
       </c>
       <c r="AP108" s="48" t="n">
-        <v>3.1</v>
+        <v>1.5</v>
       </c>
       <c r="AQ108" s="163" t="n">
         <v>0</v>
@@ -33375,10 +33375,10 @@
         </is>
       </c>
       <c r="AO109" s="47" t="n">
-        <v>1.7</v>
+        <v>3.9</v>
       </c>
       <c r="AP109" s="48" t="n">
-        <v>2.3</v>
+        <v>6.2</v>
       </c>
       <c r="AQ109" s="163" t="n">
         <v>0</v>
@@ -33645,10 +33645,10 @@
         </is>
       </c>
       <c r="AO110" s="47" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="AP110" s="48" t="n">
         <v>4.1</v>
-      </c>
-      <c r="AP110" s="48" t="n">
-        <v>2.6</v>
       </c>
       <c r="AQ110" s="163" t="n">
         <v>0</v>
@@ -33921,10 +33921,10 @@
         </is>
       </c>
       <c r="AO111" s="47" t="n">
-        <v>3.2</v>
+        <v>6.7</v>
       </c>
       <c r="AP111" s="48" t="n">
-        <v>6.5</v>
+        <v>2.6</v>
       </c>
       <c r="AQ111" s="163" t="n">
         <v>0</v>
@@ -34193,10 +34193,10 @@
         </is>
       </c>
       <c r="AO112" s="47" t="n">
-        <v>1.5</v>
+        <v>4.4</v>
       </c>
       <c r="AP112" s="48" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="AQ112" s="163" t="n">
         <v>0.03</v>
@@ -34470,10 +34470,10 @@
         </is>
       </c>
       <c r="AO113" s="47" t="n">
-        <v>8.4</v>
+        <v>4.7</v>
       </c>
       <c r="AP113" s="48" t="n">
-        <v>2.9</v>
+        <v>2.2</v>
       </c>
       <c r="AQ113" s="163" t="n">
         <v>0</v>
@@ -34754,10 +34754,10 @@
         </is>
       </c>
       <c r="AO114" s="47" t="n">
-        <v>2.3</v>
+        <v>4.1</v>
       </c>
       <c r="AP114" s="48" t="n">
-        <v>4.4</v>
+        <v>7.3</v>
       </c>
       <c r="AQ114" s="163" t="n">
         <v>0.03</v>
@@ -35037,10 +35037,10 @@
         </is>
       </c>
       <c r="AO115" s="47" t="n">
-        <v>1.2</v>
+        <v>3.8</v>
       </c>
       <c r="AP115" s="48" t="n">
-        <v>4.5</v>
+        <v>7.4</v>
       </c>
       <c r="AQ115" s="163" t="n">
         <v>0.06</v>
@@ -35320,10 +35320,10 @@
         </is>
       </c>
       <c r="AO116" s="47" t="n">
-        <v>1.1</v>
+        <v>3.6</v>
       </c>
       <c r="AP116" s="48" t="n">
-        <v>5.1</v>
+        <v>7.5</v>
       </c>
       <c r="AQ116" s="163" t="n">
         <v>0.09</v>
@@ -35595,10 +35595,10 @@
         </is>
       </c>
       <c r="AO117" s="47" t="n">
-        <v>1.9</v>
+        <v>3.3</v>
       </c>
       <c r="AP117" s="48" t="n">
-        <v>3.5</v>
+        <v>5.9</v>
       </c>
       <c r="AQ117" s="163" t="n">
         <v>0</v>
@@ -35876,10 +35876,10 @@
         </is>
       </c>
       <c r="AO118" s="47" t="n">
-        <v>3.9</v>
+        <v>6.1</v>
       </c>
       <c r="AP118" s="48" t="n">
-        <v>4.1</v>
+        <v>6.2</v>
       </c>
       <c r="AQ118" s="163" t="n">
         <v>0</v>
@@ -36153,10 +36153,10 @@
         </is>
       </c>
       <c r="AO119" s="74" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="AP119" s="75" t="n">
-        <v>2.8</v>
+        <v>5.6</v>
       </c>
       <c r="AQ119" s="173" t="n">
         <v>0</v>
@@ -36428,10 +36428,10 @@
         </is>
       </c>
       <c r="AO120" s="74" t="n">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="AP120" s="75" t="n">
-        <v>0.5</v>
+        <v>7.2</v>
       </c>
       <c r="AQ120" s="168" t="n">
         <v>0</v>
@@ -36708,10 +36708,10 @@
         </is>
       </c>
       <c r="AO121" s="74" t="n">
-        <v>6.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AP121" s="75" t="n">
-        <v>4.5</v>
+        <v>2.2</v>
       </c>
       <c r="AQ121" s="168" t="n">
         <v>0</v>
@@ -36984,10 +36984,10 @@
         </is>
       </c>
       <c r="AO122" s="74" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="AP122" s="75" t="n">
-        <v>1.1</v>
+        <v>3.8</v>
       </c>
       <c r="AQ122" s="168" t="n">
         <v>0</v>
@@ -37256,10 +37256,10 @@
         </is>
       </c>
       <c r="AO123" s="47" t="n">
-        <v>4.1</v>
+        <v>5.6</v>
       </c>
       <c r="AP123" s="88" t="n">
-        <v>4.9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AQ123" s="164" t="n">
         <v>0.035</v>
@@ -37542,10 +37542,10 @@
         </is>
       </c>
       <c r="AO124" s="47" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
       <c r="AP124" s="88" t="n">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="AQ124" s="164" t="n">
         <v>0</v>
@@ -37818,10 +37818,10 @@
         </is>
       </c>
       <c r="AO125" s="74" t="n">
+        <v>7</v>
+      </c>
+      <c r="AP125" s="75" t="n">
         <v>6.7</v>
-      </c>
-      <c r="AP125" s="75" t="n">
-        <v>2.5</v>
       </c>
       <c r="AQ125" s="168" t="n">
         <v>0</v>
@@ -38098,10 +38098,10 @@
         </is>
       </c>
       <c r="AO126" s="74" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="AP126" s="75" t="n">
-        <v>4.1</v>
+        <v>6</v>
       </c>
       <c r="AQ126" s="168" t="n">
         <v>0</v>
@@ -38386,10 +38386,10 @@
         </is>
       </c>
       <c r="AO127" s="74" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="AP127" s="48" t="n">
-        <v>4.1</v>
+        <v>6</v>
       </c>
       <c r="AQ127" s="167" t="n">
         <v>0</v>
@@ -38660,10 +38660,10 @@
         </is>
       </c>
       <c r="AO128" s="74" t="n">
-        <v>1.6</v>
+        <v>2.5</v>
       </c>
       <c r="AP128" s="75" t="n">
-        <v>3.2</v>
+        <v>5.9</v>
       </c>
       <c r="AQ128" s="168" t="n">
         <v>0.083</v>
@@ -38950,7 +38950,7 @@
         </is>
       </c>
       <c r="AO129" s="74" t="n">
-        <v>4.2</v>
+        <v>3.7</v>
       </c>
       <c r="AP129" s="75" t="n">
         <v>2.6</v>
@@ -39230,10 +39230,10 @@
         </is>
       </c>
       <c r="AO130" s="47" t="n">
-        <v>4.8</v>
+        <v>1.4</v>
       </c>
       <c r="AP130" s="88" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="AQ130" s="164" t="n">
         <v>0</v>
@@ -39510,10 +39510,10 @@
         </is>
       </c>
       <c r="AO131" s="47" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="AP131" s="88" t="n">
-        <v>2.2</v>
+        <v>6.3</v>
       </c>
       <c r="AQ131" s="164" t="n">
         <v>0</v>
@@ -39782,10 +39782,10 @@
         </is>
       </c>
       <c r="AO132" s="47" t="n">
-        <v>5.5</v>
+        <v>4.8</v>
       </c>
       <c r="AP132" s="88" t="n">
-        <v>1.3</v>
+        <v>4.8</v>
       </c>
       <c r="AQ132" s="164" t="n">
         <v>0</v>
@@ -40061,7 +40061,7 @@
         <v>5.4</v>
       </c>
       <c r="AP133" s="88" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
       <c r="AQ133" s="164" t="n">
         <v>0</v>
@@ -40614,10 +40614,10 @@
         </is>
       </c>
       <c r="AO135" s="47" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="AP135" s="88" t="n">
-        <v>2.3</v>
+        <v>4.5</v>
       </c>
       <c r="AQ135" s="164" t="n">
         <v>0</v>
@@ -40904,10 +40904,10 @@
         </is>
       </c>
       <c r="AO136" s="47" t="n">
-        <v>5.7</v>
+        <v>6.4</v>
       </c>
       <c r="AP136" s="88" t="n">
-        <v>1</v>
+        <v>4.2</v>
       </c>
       <c r="AQ136" s="164" t="n">
         <v>0</v>
@@ -41182,7 +41182,7 @@
         </is>
       </c>
       <c r="AO137" s="45" t="n">
-        <v>3.8</v>
+        <v>1.6</v>
       </c>
       <c r="AP137" s="48" t="n">
         <v>3.2</v>
@@ -41744,10 +41744,10 @@
         </is>
       </c>
       <c r="AO139" s="47" t="n">
-        <v>4.4</v>
+        <v>6.4</v>
       </c>
       <c r="AP139" s="48" t="n">
-        <v>2.3</v>
+        <v>5.9</v>
       </c>
       <c r="AQ139" s="167" t="n">
         <v>0</v>
@@ -42022,10 +42022,10 @@
         </is>
       </c>
       <c r="AO140" s="88" t="n">
-        <v>2.8</v>
+        <v>0.9</v>
       </c>
       <c r="AP140" s="118" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="AQ140" s="172" t="n">
         <v>0.038</v>
@@ -42302,10 +42302,10 @@
         </is>
       </c>
       <c r="AO141" s="74" t="n">
-        <v>3.2</v>
+        <v>2.1</v>
       </c>
       <c r="AP141" s="88" t="n">
-        <v>2.5</v>
+        <v>1.9</v>
       </c>
       <c r="AQ141" s="167" t="n">
         <v>0</v>
@@ -42578,10 +42578,10 @@
         </is>
       </c>
       <c r="AO142" s="47" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="AP142" s="118" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="AQ142" s="167" t="n">
         <v>0.01</v>
@@ -42848,10 +42848,10 @@
         </is>
       </c>
       <c r="AO143" s="47" t="n">
-        <v>6.7</v>
+        <v>8.1</v>
       </c>
       <c r="AP143" s="118" t="n">
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="AQ143" s="172" t="n">
         <v>0</v>
@@ -43402,10 +43402,10 @@
         </is>
       </c>
       <c r="AO145" s="74" t="n">
-        <v>6.4</v>
+        <v>4.3</v>
       </c>
       <c r="AP145" s="118" t="n">
-        <v>2.7</v>
+        <v>5</v>
       </c>
       <c r="AQ145" s="172" t="n">
         <v>0</v>
@@ -43688,10 +43688,10 @@
         </is>
       </c>
       <c r="AO146" s="47" t="n">
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
       <c r="AP146" s="88" t="n">
-        <v>3.2</v>
+        <v>5.2</v>
       </c>
       <c r="AQ146" s="164" t="n">
         <v>0</v>
@@ -43970,10 +43970,10 @@
         </is>
       </c>
       <c r="AO147" s="74" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="AP147" s="48" t="n">
         <v>5.2</v>
-      </c>
-      <c r="AP147" s="48" t="n">
-        <v>2.9</v>
       </c>
       <c r="AQ147" s="167" t="n">
         <v>0</v>
@@ -44252,10 +44252,10 @@
         </is>
       </c>
       <c r="AO148" s="74" t="n">
-        <v>4</v>
+        <v>1.8</v>
       </c>
       <c r="AP148" s="48" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="AQ148" s="167" t="n">
         <v>0</v>
@@ -44532,10 +44532,10 @@
         </is>
       </c>
       <c r="AO149" s="47" t="n">
-        <v>5.5</v>
+        <v>2.9</v>
       </c>
       <c r="AP149" s="118" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
       <c r="AQ149" s="164" t="n">
         <v>0</v>
@@ -44812,10 +44812,10 @@
         </is>
       </c>
       <c r="AO150" s="47" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="AP150" s="118" t="n">
-        <v>3.5</v>
+        <v>5.7</v>
       </c>
       <c r="AQ150" s="172" t="n">
         <v>0</v>
@@ -45094,10 +45094,10 @@
         </is>
       </c>
       <c r="AO151" s="74" t="n">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="AP151" s="118" t="n">
-        <v>0.8</v>
+        <v>5.5</v>
       </c>
       <c r="AQ151" s="172" t="n">
         <v>0</v>
@@ -45660,10 +45660,10 @@
         </is>
       </c>
       <c r="AO153" s="74" t="n">
-        <v>6.8</v>
+        <v>4</v>
       </c>
       <c r="AP153" s="118" t="n">
-        <v>2.9</v>
+        <v>6.5</v>
       </c>
       <c r="AQ153" s="174" t="n">
         <v>0</v>
@@ -46208,10 +46208,10 @@
         </is>
       </c>
       <c r="AO155" s="74" t="n">
-        <v>9</v>
+        <v>4.5</v>
       </c>
       <c r="AP155" s="118" t="n">
-        <v>0.6</v>
+        <v>5.1</v>
       </c>
       <c r="AQ155" s="172" t="n">
         <v>0</v>
@@ -46492,10 +46492,10 @@
         </is>
       </c>
       <c r="AO156" s="47" t="n">
-        <v>5.8</v>
+        <v>4.1</v>
       </c>
       <c r="AP156" s="88" t="n">
-        <v>4.5</v>
+        <v>9</v>
       </c>
       <c r="AQ156" s="164" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Improve Layout Durability scoring with multi-IPR layout balance analysis
Key changes:
- Add _compute_pri_sec_ratio() helper for standalone ratio computation
- Compute cutlets at IPR=0.100 for every bit to capture worst-case
  primary/secondary blade imbalance (the "low IPR stress test")
- Replace old pri_sec_balance (6% weight, single IPR) with:
  - low_ipr_layout_balance (20%): 1/log2(ratio+1) at IPR=0.100
  - layout_stability (8%): ratio consistency across IPR values
- Rebalance all durability component weights based on multi-IPR study
- Add AI_LEARNED_NOTES.md documenting key findings from F-type vs 6-3
  comparative analysis across three IPR values

Study bits before/after: 8896 (F-type good shift) 1.5->4.5,
2746 (F-type small shift) 3.5->2.5, 2226 (6-3) 0.4->0.7

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Bit Applications Tool r2.xlsx
+++ b/Bit Applications Tool r2.xlsx
@@ -4401,7 +4401,7 @@
         </is>
       </c>
       <c r="AO5" s="47" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="AP5" s="48" t="n">
         <v>1.4</v>
@@ -4935,7 +4935,7 @@
         </is>
       </c>
       <c r="AO7" s="74" t="n">
-        <v>5</v>
+        <v>6.6</v>
       </c>
       <c r="AP7" s="75" t="n">
         <v>3.1</v>
@@ -5993,7 +5993,7 @@
         </is>
       </c>
       <c r="AO11" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP11" s="48" t="n">
         <v>2.4</v>
@@ -6263,7 +6263,7 @@
         </is>
       </c>
       <c r="AO12" s="47" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="AP12" s="48" t="n">
         <v>3</v>
@@ -6805,7 +6805,7 @@
         </is>
       </c>
       <c r="AO14" s="47" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="AP14" s="48" t="n">
         <v>2.2</v>
@@ -8671,7 +8671,7 @@
         </is>
       </c>
       <c r="AO21" s="47" t="n">
-        <v>5.3</v>
+        <v>6.8</v>
       </c>
       <c r="AP21" s="48" t="n">
         <v>2.8</v>
@@ -9739,7 +9739,7 @@
         </is>
       </c>
       <c r="AO25" s="47" t="n">
-        <v>6.4</v>
+        <v>7.1</v>
       </c>
       <c r="AP25" s="48" t="n">
         <v>4.2</v>
@@ -10555,7 +10555,7 @@
         </is>
       </c>
       <c r="AO28" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP28" s="48" t="n">
         <v>3.4</v>
@@ -10837,7 +10837,7 @@
         </is>
       </c>
       <c r="AO29" s="47" t="n">
-        <v>6.2</v>
+        <v>7.3</v>
       </c>
       <c r="AP29" s="48" t="n">
         <v>4.9</v>
@@ -11117,7 +11117,7 @@
         </is>
       </c>
       <c r="AO30" s="47" t="n">
-        <v>5.5</v>
+        <v>6.3</v>
       </c>
       <c r="AP30" s="48" t="n">
         <v>2.8</v>
@@ -11425,7 +11425,7 @@
         </is>
       </c>
       <c r="AO31" s="46" t="n">
-        <v>6</v>
+        <v>7.1</v>
       </c>
       <c r="AP31" s="48" t="n">
         <v>1.8</v>
@@ -11727,7 +11727,7 @@
         </is>
       </c>
       <c r="AO32" s="46" t="n">
-        <v>6.8</v>
+        <v>7.4</v>
       </c>
       <c r="AP32" s="48" t="n">
         <v>0.1</v>
@@ -12007,7 +12007,7 @@
         </is>
       </c>
       <c r="AO33" s="47" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="AP33" s="48" t="n">
         <v>2.4</v>
@@ -12289,7 +12289,7 @@
         </is>
       </c>
       <c r="AO34" s="47" t="n">
-        <v>7</v>
+        <v>7.6</v>
       </c>
       <c r="AP34" s="48" t="n">
         <v>2.4</v>
@@ -12571,7 +12571,7 @@
         </is>
       </c>
       <c r="AO35" s="47" t="n">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
       <c r="AP35" s="48" t="n">
         <v>3.7</v>
@@ -12857,7 +12857,7 @@
         </is>
       </c>
       <c r="AO36" s="46" t="n">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="AP36" s="48" t="n">
         <v>3.4</v>
@@ -13135,7 +13135,7 @@
         </is>
       </c>
       <c r="AO37" s="47" t="n">
-        <v>5.6</v>
+        <v>6.7</v>
       </c>
       <c r="AP37" s="48" t="n">
         <v>3.5</v>
@@ -13437,7 +13437,7 @@
         </is>
       </c>
       <c r="AO38" s="46" t="n">
-        <v>6.8</v>
+        <v>6.2</v>
       </c>
       <c r="AP38" s="48" t="n">
         <v>6.1</v>
@@ -13975,7 +13975,7 @@
         </is>
       </c>
       <c r="AO40" s="47" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AP40" s="48" t="n">
         <v>3.4</v>
@@ -14271,7 +14271,7 @@
         </is>
       </c>
       <c r="AO41" s="46" t="n">
-        <v>6.5</v>
+        <v>6.9</v>
       </c>
       <c r="AP41" s="48" t="n">
         <v>0.1</v>
@@ -14551,7 +14551,7 @@
         </is>
       </c>
       <c r="AO42" s="47" t="n">
-        <v>4.1</v>
+        <v>3.2</v>
       </c>
       <c r="AP42" s="48" t="n">
         <v>1</v>
@@ -14851,7 +14851,7 @@
         </is>
       </c>
       <c r="AO43" s="46" t="n">
-        <v>5.9</v>
+        <v>6.8</v>
       </c>
       <c r="AP43" s="48" t="n">
         <v>3.2</v>
@@ -15133,7 +15133,7 @@
         </is>
       </c>
       <c r="AO44" s="47" t="n">
-        <v>3.8</v>
+        <v>5.4</v>
       </c>
       <c r="AP44" s="48" t="n">
         <v>2.2</v>
@@ -15411,7 +15411,7 @@
         </is>
       </c>
       <c r="AO45" s="47" t="n">
-        <v>5.4</v>
+        <v>6.4</v>
       </c>
       <c r="AP45" s="48" t="n">
         <v>4.3</v>
@@ -15689,7 +15689,7 @@
         </is>
       </c>
       <c r="AO46" s="47" t="n">
-        <v>5.4</v>
+        <v>6.4</v>
       </c>
       <c r="AP46" s="48" t="n">
         <v>4.3</v>
@@ -15967,7 +15967,7 @@
         </is>
       </c>
       <c r="AO47" s="47" t="n">
-        <v>4.9</v>
+        <v>6.1</v>
       </c>
       <c r="AP47" s="48" t="n">
         <v>3.6</v>
@@ -16255,7 +16255,7 @@
         </is>
       </c>
       <c r="AO48" s="47" t="n">
-        <v>4.4</v>
+        <v>5.8</v>
       </c>
       <c r="AP48" s="48" t="n">
         <v>3.6</v>
@@ -16549,7 +16549,7 @@
         </is>
       </c>
       <c r="AO49" s="46" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP49" s="48" t="n">
         <v>1.7</v>
@@ -16829,7 +16829,7 @@
         </is>
       </c>
       <c r="AO50" s="47" t="n">
-        <v>3</v>
+        <v>5.1</v>
       </c>
       <c r="AP50" s="48" t="n">
         <v>2.9</v>
@@ -17131,7 +17131,7 @@
         </is>
       </c>
       <c r="AO51" s="46" t="n">
-        <v>4.2</v>
+        <v>5.8</v>
       </c>
       <c r="AP51" s="48" t="n">
         <v>6</v>
@@ -17415,7 +17415,7 @@
         </is>
       </c>
       <c r="AO52" s="47" t="n">
-        <v>4.1</v>
+        <v>5.6</v>
       </c>
       <c r="AP52" s="48" t="n">
         <v>4.8</v>
@@ -17686,7 +17686,7 @@
         </is>
       </c>
       <c r="AO53" s="47" t="n">
-        <v>5.3</v>
+        <v>6.1</v>
       </c>
       <c r="AP53" s="48" t="n">
         <v>2.9</v>
@@ -17962,7 +17962,7 @@
         </is>
       </c>
       <c r="AO54" s="47" t="n">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="AP54" s="48" t="n">
         <v>3.1</v>
@@ -18228,7 +18228,7 @@
         </is>
       </c>
       <c r="AO55" s="47" t="n">
-        <v>3.7</v>
+        <v>4.5</v>
       </c>
       <c r="AP55" s="48" t="n">
         <v>1.6</v>
@@ -18512,7 +18512,7 @@
         </is>
       </c>
       <c r="AO56" s="47" t="n">
-        <v>6.1</v>
+        <v>6.9</v>
       </c>
       <c r="AP56" s="48" t="n">
         <v>4.5</v>
@@ -18794,7 +18794,7 @@
         </is>
       </c>
       <c r="AO57" s="47" t="n">
-        <v>4.1</v>
+        <v>5.8</v>
       </c>
       <c r="AP57" s="48" t="n">
         <v>1.7</v>
@@ -19076,7 +19076,7 @@
         </is>
       </c>
       <c r="AO58" s="47" t="n">
-        <v>4.9</v>
+        <v>5.8</v>
       </c>
       <c r="AP58" s="48" t="n">
         <v>2.5</v>
@@ -19355,7 +19355,7 @@
         </is>
       </c>
       <c r="AO59" s="47" t="n">
-        <v>4.9</v>
+        <v>6</v>
       </c>
       <c r="AP59" s="48" t="n">
         <v>1.9</v>
@@ -19639,7 +19639,7 @@
         </is>
       </c>
       <c r="AO60" s="47" t="n">
-        <v>5.3</v>
+        <v>6.3</v>
       </c>
       <c r="AP60" s="48" t="n">
         <v>4.2</v>
@@ -19921,7 +19921,7 @@
         </is>
       </c>
       <c r="AO61" s="47" t="n">
-        <v>5.4</v>
+        <v>6.4</v>
       </c>
       <c r="AP61" s="48" t="n">
         <v>4.3</v>
@@ -20203,7 +20203,7 @@
         </is>
       </c>
       <c r="AO62" s="47" t="n">
-        <v>3.9</v>
+        <v>5.7</v>
       </c>
       <c r="AP62" s="48" t="n">
         <v>2.5</v>
@@ -20481,7 +20481,7 @@
         </is>
       </c>
       <c r="AO63" s="47" t="n">
-        <v>5.9</v>
+        <v>6.4</v>
       </c>
       <c r="AP63" s="48" t="n">
         <v>3.3</v>
@@ -20764,7 +20764,7 @@
         </is>
       </c>
       <c r="AO64" s="47" t="n">
-        <v>3.4</v>
+        <v>5.2</v>
       </c>
       <c r="AP64" s="48" t="n">
         <v>2.9</v>
@@ -21044,7 +21044,7 @@
         </is>
       </c>
       <c r="AO65" s="47" t="n">
-        <v>0.6</v>
+        <v>1.8</v>
       </c>
       <c r="AP65" s="48" t="n">
         <v>1.5</v>
@@ -21335,7 +21335,7 @@
         </is>
       </c>
       <c r="AO66" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP66" s="48" t="n">
         <v>3.4</v>
@@ -21625,7 +21625,7 @@
         </is>
       </c>
       <c r="AO67" s="47" t="n">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="AP67" s="48" t="n">
         <v>1.4</v>
@@ -21913,7 +21913,7 @@
         </is>
       </c>
       <c r="AO68" s="47" t="n">
-        <v>2.6</v>
+        <v>4.6</v>
       </c>
       <c r="AP68" s="48" t="n">
         <v>2.4</v>
@@ -22211,7 +22211,7 @@
         </is>
       </c>
       <c r="AO69" s="47" t="n">
-        <v>3.6</v>
+        <v>5.4</v>
       </c>
       <c r="AP69" s="48" t="n">
         <v>5.5</v>
@@ -22485,7 +22485,7 @@
         </is>
       </c>
       <c r="AO70" s="47" t="n">
-        <v>3.6</v>
+        <v>5.2</v>
       </c>
       <c r="AP70" s="48" t="n">
         <v>2</v>
@@ -22777,7 +22777,7 @@
         </is>
       </c>
       <c r="AO71" s="47" t="n">
-        <v>5.3</v>
+        <v>6.8</v>
       </c>
       <c r="AP71" s="48" t="n">
         <v>0.2</v>
@@ -23055,7 +23055,7 @@
         </is>
       </c>
       <c r="AO72" s="47" t="n">
-        <v>2.2</v>
+        <v>5</v>
       </c>
       <c r="AP72" s="48" t="n">
         <v>4.4</v>
@@ -23336,7 +23336,7 @@
         </is>
       </c>
       <c r="AO73" s="47" t="n">
-        <v>5.2</v>
+        <v>6.4</v>
       </c>
       <c r="AP73" s="48" t="n">
         <v>4.4</v>
@@ -23617,7 +23617,7 @@
         </is>
       </c>
       <c r="AO74" s="47" t="n">
-        <v>6</v>
+        <v>6.7</v>
       </c>
       <c r="AP74" s="48" t="n">
         <v>4.6</v>
@@ -23900,7 +23900,7 @@
         </is>
       </c>
       <c r="AO75" s="47" t="n">
-        <v>5.3</v>
+        <v>6.4</v>
       </c>
       <c r="AP75" s="48" t="n">
         <v>4.6</v>
@@ -24179,7 +24179,7 @@
         </is>
       </c>
       <c r="AO76" s="47" t="n">
-        <v>4.3</v>
+        <v>5.5</v>
       </c>
       <c r="AP76" s="48" t="n">
         <v>4.5</v>
@@ -24403,7 +24403,7 @@
         </is>
       </c>
       <c r="AO77" s="47" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="AP77" s="48" t="n">
         <v>4.7</v>
@@ -24694,7 +24694,7 @@
         </is>
       </c>
       <c r="AO78" s="47" t="n">
-        <v>5.6</v>
+        <v>6.6</v>
       </c>
       <c r="AP78" s="48" t="n">
         <v>2.7</v>
@@ -24987,7 +24987,7 @@
         </is>
       </c>
       <c r="AO79" s="47" t="n">
-        <v>3.9</v>
+        <v>5.6</v>
       </c>
       <c r="AP79" s="48" t="n">
         <v>9</v>
@@ -25275,7 +25275,7 @@
         </is>
       </c>
       <c r="AO80" s="47" t="n">
-        <v>8.1</v>
+        <v>7.7</v>
       </c>
       <c r="AP80" s="48" t="n">
         <v>5</v>
@@ -25545,7 +25545,7 @@
         </is>
       </c>
       <c r="AO81" s="47" t="n">
-        <v>4.1</v>
+        <v>5.5</v>
       </c>
       <c r="AP81" s="48" t="n">
         <v>2.1</v>
@@ -25821,7 +25821,7 @@
         </is>
       </c>
       <c r="AO82" s="47" t="n">
-        <v>5.9</v>
+        <v>6.8</v>
       </c>
       <c r="AP82" s="48" t="n">
         <v>0</v>
@@ -26113,7 +26113,7 @@
         </is>
       </c>
       <c r="AO83" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP83" s="48" t="n">
         <v>3.4</v>
@@ -26401,7 +26401,7 @@
         </is>
       </c>
       <c r="AO84" s="47" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="AP84" s="48" t="n">
         <v>5.1</v>
@@ -26687,7 +26687,7 @@
         </is>
       </c>
       <c r="AO85" s="47" t="n">
-        <v>5</v>
+        <v>6.6</v>
       </c>
       <c r="AP85" s="48" t="n">
         <v>3.1</v>
@@ -26969,7 +26969,7 @@
         </is>
       </c>
       <c r="AO86" s="47" t="n">
-        <v>5.8</v>
+        <v>6.5</v>
       </c>
       <c r="AP86" s="48" t="n">
         <v>3.6</v>
@@ -27248,7 +27248,7 @@
         </is>
       </c>
       <c r="AO87" s="47" t="n">
-        <v>4.4</v>
+        <v>6.1</v>
       </c>
       <c r="AP87" s="48" t="n">
         <v>3.4</v>
@@ -27528,7 +27528,7 @@
         </is>
       </c>
       <c r="AO88" s="47" t="n">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
       <c r="AP88" s="48" t="n">
         <v>1.7</v>
@@ -27800,7 +27800,7 @@
         </is>
       </c>
       <c r="AO89" s="47" t="n">
-        <v>5</v>
+        <v>6.2</v>
       </c>
       <c r="AP89" s="48" t="n">
         <v>3.2</v>
@@ -28093,7 +28093,7 @@
         </is>
       </c>
       <c r="AO90" s="47" t="n">
-        <v>5.5</v>
+        <v>7.1</v>
       </c>
       <c r="AP90" s="48" t="n">
         <v>3.4</v>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="AO91" s="45" t="n">
-        <v>4.4</v>
+        <v>5.9</v>
       </c>
       <c r="AP91" s="48" t="n">
         <v>3.7</v>
@@ -28665,7 +28665,7 @@
         </is>
       </c>
       <c r="AO92" s="47" t="n">
-        <v>2.3</v>
+        <v>5.1</v>
       </c>
       <c r="AP92" s="48" t="n">
         <v>3.6</v>
@@ -28962,7 +28962,7 @@
         </is>
       </c>
       <c r="AO93" s="47" t="n">
-        <v>5.8</v>
+        <v>7.4</v>
       </c>
       <c r="AP93" s="48" t="n">
         <v>4.4</v>
@@ -29240,7 +29240,7 @@
         </is>
       </c>
       <c r="AO94" s="47" t="n">
-        <v>4</v>
+        <v>5.6</v>
       </c>
       <c r="AP94" s="48" t="n">
         <v>3.3</v>
@@ -29525,7 +29525,7 @@
         </is>
       </c>
       <c r="AO95" s="47" t="n">
-        <v>2.1</v>
+        <v>4.9</v>
       </c>
       <c r="AP95" s="48" t="n">
         <v>3.6</v>
@@ -29810,7 +29810,7 @@
         </is>
       </c>
       <c r="AO96" s="47" t="n">
-        <v>2.7</v>
+        <v>5.4</v>
       </c>
       <c r="AP96" s="48" t="n">
         <v>5.7</v>
@@ -30088,7 +30088,7 @@
         </is>
       </c>
       <c r="AO97" s="47" t="n">
-        <v>4.9</v>
+        <v>6.3</v>
       </c>
       <c r="AP97" s="88" t="n">
         <v>4.3</v>
@@ -30366,7 +30366,7 @@
         </is>
       </c>
       <c r="AO98" s="47" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
       <c r="AP98" s="48" t="n">
         <v>5.5</v>
@@ -30637,7 +30637,7 @@
         </is>
       </c>
       <c r="AO99" s="47" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="AP99" s="48" t="n">
         <v>2.1</v>
@@ -30918,7 +30918,7 @@
         </is>
       </c>
       <c r="AO100" s="47" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AP100" s="48" t="n">
         <v>4.2</v>
@@ -31196,7 +31196,7 @@
         </is>
       </c>
       <c r="AO101" s="47" t="n">
-        <v>3.3</v>
+        <v>5.1</v>
       </c>
       <c r="AP101" s="48" t="n">
         <v>4.6</v>
@@ -31473,7 +31473,7 @@
         </is>
       </c>
       <c r="AO102" s="47" t="n">
-        <v>2</v>
+        <v>4.6</v>
       </c>
       <c r="AP102" s="48" t="n">
         <v>1.3</v>
@@ -31743,7 +31743,7 @@
         </is>
       </c>
       <c r="AO103" s="47" t="n">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AP103" s="48" t="n">
         <v>3.8</v>
@@ -32023,7 +32023,7 @@
         </is>
       </c>
       <c r="AO104" s="47" t="n">
-        <v>5</v>
+        <v>6.7</v>
       </c>
       <c r="AP104" s="48" t="n">
         <v>1.8</v>
@@ -32300,7 +32300,7 @@
         </is>
       </c>
       <c r="AO105" s="47" t="n">
-        <v>2.5</v>
+        <v>4.9</v>
       </c>
       <c r="AP105" s="48" t="n">
         <v>1.2</v>
@@ -32572,7 +32572,7 @@
         </is>
       </c>
       <c r="AO106" s="47" t="n">
-        <v>3.9</v>
+        <v>5.6</v>
       </c>
       <c r="AP106" s="48" t="n">
         <v>2.6</v>
@@ -32838,7 +32838,7 @@
         </is>
       </c>
       <c r="AO107" s="47" t="n">
-        <v>4.9</v>
+        <v>6.3</v>
       </c>
       <c r="AP107" s="88" t="n">
         <v>4.3</v>
@@ -33107,7 +33107,7 @@
         </is>
       </c>
       <c r="AO108" s="47" t="n">
-        <v>8.1</v>
+        <v>7.5</v>
       </c>
       <c r="AP108" s="48" t="n">
         <v>5.6</v>
@@ -33375,7 +33375,7 @@
         </is>
       </c>
       <c r="AO109" s="47" t="n">
-        <v>0.8</v>
+        <v>4</v>
       </c>
       <c r="AP109" s="48" t="n">
         <v>3.5</v>
@@ -33645,7 +33645,7 @@
         </is>
       </c>
       <c r="AO110" s="47" t="n">
-        <v>4.2</v>
+        <v>5.6</v>
       </c>
       <c r="AP110" s="48" t="n">
         <v>0.9</v>
@@ -33921,7 +33921,7 @@
         </is>
       </c>
       <c r="AO111" s="47" t="n">
-        <v>4.8</v>
+        <v>6.1</v>
       </c>
       <c r="AP111" s="48" t="n">
         <v>5.5</v>
@@ -34193,7 +34193,7 @@
         </is>
       </c>
       <c r="AO112" s="47" t="n">
-        <v>1.1</v>
+        <v>4</v>
       </c>
       <c r="AP112" s="48" t="n">
         <v>2.9</v>
@@ -34470,7 +34470,7 @@
         </is>
       </c>
       <c r="AO113" s="47" t="n">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="AP113" s="48" t="n">
         <v>4.6</v>
@@ -34754,7 +34754,7 @@
         </is>
       </c>
       <c r="AO114" s="47" t="n">
-        <v>1.3</v>
+        <v>3.4</v>
       </c>
       <c r="AP114" s="48" t="n">
         <v>4.4</v>
@@ -35037,7 +35037,7 @@
         </is>
       </c>
       <c r="AO115" s="47" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="AP115" s="48" t="n">
         <v>4.3</v>
@@ -35595,7 +35595,7 @@
         </is>
       </c>
       <c r="AO117" s="47" t="n">
-        <v>1.9</v>
+        <v>4.6</v>
       </c>
       <c r="AP117" s="48" t="n">
         <v>3.7</v>
@@ -35876,7 +35876,7 @@
         </is>
       </c>
       <c r="AO118" s="47" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AP118" s="48" t="n">
         <v>4.9</v>
@@ -36153,7 +36153,7 @@
         </is>
       </c>
       <c r="AO119" s="74" t="n">
-        <v>3.3</v>
+        <v>5.8</v>
       </c>
       <c r="AP119" s="75" t="n">
         <v>3.4</v>
@@ -36428,7 +36428,7 @@
         </is>
       </c>
       <c r="AO120" s="74" t="n">
-        <v>2.4</v>
+        <v>5.1</v>
       </c>
       <c r="AP120" s="75" t="n">
         <v>0.8</v>
@@ -36708,7 +36708,7 @@
         </is>
       </c>
       <c r="AO121" s="74" t="n">
-        <v>5.1</v>
+        <v>6.3</v>
       </c>
       <c r="AP121" s="75" t="n">
         <v>4.9</v>
@@ -36984,7 +36984,7 @@
         </is>
       </c>
       <c r="AO122" s="74" t="n">
-        <v>4.3</v>
+        <v>5.4</v>
       </c>
       <c r="AP122" s="75" t="n">
         <v>0.8</v>
@@ -37256,7 +37256,7 @@
         </is>
       </c>
       <c r="AO123" s="47" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="AP123" s="88" t="n">
         <v>5.8</v>
@@ -37542,7 +37542,7 @@
         </is>
       </c>
       <c r="AO124" s="47" t="n">
-        <v>8.1</v>
+        <v>7.7</v>
       </c>
       <c r="AP124" s="88" t="n">
         <v>5</v>
@@ -37818,7 +37818,7 @@
         </is>
       </c>
       <c r="AO125" s="74" t="n">
-        <v>6.3</v>
+        <v>7.2</v>
       </c>
       <c r="AP125" s="75" t="n">
         <v>3.2</v>
@@ -38098,7 +38098,7 @@
         </is>
       </c>
       <c r="AO126" s="74" t="n">
-        <v>3.1</v>
+        <v>5.4</v>
       </c>
       <c r="AP126" s="75" t="n">
         <v>4.2</v>
@@ -38386,7 +38386,7 @@
         </is>
       </c>
       <c r="AO127" s="74" t="n">
-        <v>3.1</v>
+        <v>5.4</v>
       </c>
       <c r="AP127" s="48" t="n">
         <v>4.2</v>
@@ -38660,7 +38660,7 @@
         </is>
       </c>
       <c r="AO128" s="74" t="n">
-        <v>1.1</v>
+        <v>2.4</v>
       </c>
       <c r="AP128" s="75" t="n">
         <v>2.4</v>
@@ -38950,7 +38950,7 @@
         </is>
       </c>
       <c r="AO129" s="74" t="n">
-        <v>3.3</v>
+        <v>4.9</v>
       </c>
       <c r="AP129" s="75" t="n">
         <v>2.1</v>
@@ -39230,7 +39230,7 @@
         </is>
       </c>
       <c r="AO130" s="47" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AP130" s="88" t="n">
         <v>2.9</v>
@@ -39510,7 +39510,7 @@
         </is>
       </c>
       <c r="AO131" s="47" t="n">
-        <v>2.9</v>
+        <v>4.3</v>
       </c>
       <c r="AP131" s="88" t="n">
         <v>3.2</v>
@@ -39782,7 +39782,7 @@
         </is>
       </c>
       <c r="AO132" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP132" s="88" t="n">
         <v>2.4</v>
@@ -40058,7 +40058,7 @@
         </is>
       </c>
       <c r="AO133" s="47" t="n">
-        <v>6.2</v>
+        <v>7.3</v>
       </c>
       <c r="AP133" s="88" t="n">
         <v>5.6</v>
@@ -40614,7 +40614,7 @@
         </is>
       </c>
       <c r="AO135" s="47" t="n">
-        <v>3.6</v>
+        <v>5.5</v>
       </c>
       <c r="AP135" s="88" t="n">
         <v>1.8</v>
@@ -40904,7 +40904,7 @@
         </is>
       </c>
       <c r="AO136" s="47" t="n">
-        <v>5.4</v>
+        <v>6.3</v>
       </c>
       <c r="AP136" s="88" t="n">
         <v>1.9</v>
@@ -41182,7 +41182,7 @@
         </is>
       </c>
       <c r="AO137" s="45" t="n">
-        <v>2.7</v>
+        <v>4.8</v>
       </c>
       <c r="AP137" s="48" t="n">
         <v>3.3</v>
@@ -41744,7 +41744,7 @@
         </is>
       </c>
       <c r="AO139" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP139" s="48" t="n">
         <v>3.2</v>
@@ -42022,7 +42022,7 @@
         </is>
       </c>
       <c r="AO140" s="88" t="n">
-        <v>1.4</v>
+        <v>4.4</v>
       </c>
       <c r="AP140" s="118" t="n">
         <v>3.5</v>
@@ -42302,7 +42302,7 @@
         </is>
       </c>
       <c r="AO141" s="74" t="n">
-        <v>1.7</v>
+        <v>4</v>
       </c>
       <c r="AP141" s="88" t="n">
         <v>0.7</v>
@@ -42578,7 +42578,7 @@
         </is>
       </c>
       <c r="AO142" s="47" t="n">
-        <v>4.8</v>
+        <v>6.3</v>
       </c>
       <c r="AP142" s="118" t="n">
         <v>1.5</v>
@@ -42848,7 +42848,7 @@
         </is>
       </c>
       <c r="AO143" s="47" t="n">
-        <v>4.9</v>
+        <v>6.2</v>
       </c>
       <c r="AP143" s="118" t="n">
         <v>1.5</v>
@@ -43402,7 +43402,7 @@
         </is>
       </c>
       <c r="AO145" s="74" t="n">
-        <v>5.5</v>
+        <v>6.6</v>
       </c>
       <c r="AP145" s="118" t="n">
         <v>4.8</v>
@@ -43688,7 +43688,7 @@
         </is>
       </c>
       <c r="AO146" s="47" t="n">
-        <v>5.2</v>
+        <v>6.2</v>
       </c>
       <c r="AP146" s="88" t="n">
         <v>2.9</v>
@@ -43970,7 +43970,7 @@
         </is>
       </c>
       <c r="AO147" s="74" t="n">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="AP147" s="48" t="n">
         <v>3</v>
@@ -44252,7 +44252,7 @@
         </is>
       </c>
       <c r="AO148" s="74" t="n">
-        <v>2.9</v>
+        <v>4.9</v>
       </c>
       <c r="AP148" s="48" t="n">
         <v>3.4</v>
@@ -44532,7 +44532,7 @@
         </is>
       </c>
       <c r="AO149" s="47" t="n">
-        <v>3.1</v>
+        <v>5</v>
       </c>
       <c r="AP149" s="118" t="n">
         <v>3.3</v>
@@ -44812,7 +44812,7 @@
         </is>
       </c>
       <c r="AO150" s="47" t="n">
-        <v>4.7</v>
+        <v>5.9</v>
       </c>
       <c r="AP150" s="118" t="n">
         <v>3.4</v>
@@ -45094,10 +45094,10 @@
         </is>
       </c>
       <c r="AO151" s="74" t="n">
-        <v>2.7</v>
+        <v>4.5</v>
       </c>
       <c r="AP151" s="118" t="n">
-        <v>2.1</v>
+        <v>0.8</v>
       </c>
       <c r="AQ151" s="172" t="n">
         <v>0</v>
@@ -45660,7 +45660,7 @@
         </is>
       </c>
       <c r="AO153" s="74" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="AP153" s="118" t="n">
         <v>6.9</v>
@@ -46492,7 +46492,7 @@
         </is>
       </c>
       <c r="AO156" s="47" t="n">
-        <v>5.6</v>
+        <v>6.6</v>
       </c>
       <c r="AP156" s="88" t="n">
         <v>6.5</v>

</xml_diff>